<commit_message>
DBJ: regenerate Excel with 6W data (W1-W6) and updated labels
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dbj/DBJ_US_Feb-Mar_2026.xlsx
+++ b/dbj/DBJ_US_Feb-Mar_2026.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📊 5W Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📊 6W Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📋 Weekly Raw Data" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="🔍 Child ASIN Detail" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="📈 WoW Change" sheetId="4" state="visible" r:id="rId4"/>
@@ -379,7 +379,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="265">
+  <cellXfs count="269">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -908,6 +908,18 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="3" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
@@ -1615,7 +1627,7 @@
       </c>
       <c r="AA3" s="9" t="inlineStr">
         <is>
-          <t>5W TOTAL</t>
+          <t>6W TOTAL</t>
         </is>
       </c>
     </row>
@@ -8847,12 +8859,12 @@
       </c>
       <c r="L3" s="46" t="inlineStr">
         <is>
-          <t>5W Sales</t>
+          <t>6W Sales</t>
         </is>
       </c>
       <c r="M3" s="46" t="inlineStr">
         <is>
-          <t>5W Units</t>
+          <t>6W Units</t>
         </is>
       </c>
     </row>
@@ -18923,7 +18935,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -18972,6 +18984,11 @@
           <t>W5: $0 (0 ord)</t>
         </is>
       </c>
+      <c r="K2" s="177" t="inlineStr">
+        <is>
+          <t>W6: $613 (6 ord)</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="4" customHeight="1"/>
     <row r="4" ht="20" customHeight="1">
@@ -19031,36 +19048,327 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="42" t="inlineStr">
-        <is>
-          <t>5W GRAND TOTAL  (6 rows)</t>
-        </is>
-      </c>
-      <c r="G5" s="177" t="n">
+    <row r="5" ht="16" customHeight="1">
+      <c r="A5" s="178" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  W6 — Mar 8–9  |  6 筆  |  Sales $613  Orders 6  NTB $613</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="15" customHeight="1">
+      <c r="A6" s="83" t="inlineStr">
+        <is>
+          <t>W6</t>
+        </is>
+      </c>
+      <c r="B6" s="179" t="inlineStr">
+        <is>
+          <t>03/08</t>
+        </is>
+      </c>
+      <c r="C6" s="180" t="inlineStr">
+        <is>
+          <t>Dryer Rack</t>
+        </is>
+      </c>
+      <c r="D6" s="83" t="inlineStr">
+        <is>
+          <t>B097V3JSWH</t>
+        </is>
+      </c>
+      <c r="E6" s="83" t="inlineStr">
+        <is>
+          <t>B097V3JSWH</t>
+        </is>
+      </c>
+      <c r="F6" s="82" t="inlineStr">
+        <is>
+          <t>SB_extendable garment rack_$0.79_01020920</t>
+        </is>
+      </c>
+      <c r="G6" s="85" t="n">
+        <v>57.6</v>
+      </c>
+      <c r="H6" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" s="85" t="n">
+        <v>57.6</v>
+      </c>
+      <c r="K6" s="129" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" ht="15" customHeight="1">
+      <c r="A7" s="83" t="inlineStr">
+        <is>
+          <t>W6</t>
+        </is>
+      </c>
+      <c r="B7" s="179" t="inlineStr">
+        <is>
+          <t>03/08</t>
+        </is>
+      </c>
+      <c r="C7" s="180" t="inlineStr">
+        <is>
+          <t>Storage Cart 10D</t>
+        </is>
+      </c>
+      <c r="D7" s="83" t="inlineStr">
+        <is>
+          <t>B0FVFCYKGB</t>
+        </is>
+      </c>
+      <c r="E7" s="83" t="inlineStr">
+        <is>
+          <t>B0FVF9GS2S</t>
+        </is>
+      </c>
+      <c r="F7" s="82" t="inlineStr">
+        <is>
+          <t>DBJ Drawer Cart_clear plastic drawer cart_$0.77_01021180</t>
+        </is>
+      </c>
+      <c r="G7" s="85" t="n">
+        <v>69.98999999999999</v>
+      </c>
+      <c r="H7" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" s="85" t="n">
+        <v>69.98999999999999</v>
+      </c>
+      <c r="K7" s="129" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1">
+      <c r="A8" s="83" t="inlineStr">
+        <is>
+          <t>W6</t>
+        </is>
+      </c>
+      <c r="B8" s="179" t="inlineStr">
+        <is>
+          <t>03/09</t>
+        </is>
+      </c>
+      <c r="C8" s="180" t="inlineStr">
+        <is>
+          <t>Dryer Rack</t>
+        </is>
+      </c>
+      <c r="D8" s="83" t="inlineStr">
+        <is>
+          <t>B097V3JSWH</t>
+        </is>
+      </c>
+      <c r="E8" s="83" t="inlineStr">
+        <is>
+          <t>B097V3JSWH</t>
+        </is>
+      </c>
+      <c r="F8" s="82" t="inlineStr">
+        <is>
+          <t>SB_industrial clothing rack_$0.79_01020920</t>
+        </is>
+      </c>
+      <c r="G8" s="85" t="n">
+        <v>65</v>
+      </c>
+      <c r="H8" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" s="85" t="n">
+        <v>65</v>
+      </c>
+      <c r="K8" s="129" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1">
+      <c r="A9" s="83" t="inlineStr">
+        <is>
+          <t>W6</t>
+        </is>
+      </c>
+      <c r="B9" s="179" t="inlineStr">
+        <is>
+          <t>03/09</t>
+        </is>
+      </c>
+      <c r="C9" s="180" t="inlineStr">
+        <is>
+          <t>Storage Cart 10D</t>
+        </is>
+      </c>
+      <c r="D9" s="83" t="inlineStr">
+        <is>
+          <t>B0FVFCYKGB</t>
+        </is>
+      </c>
+      <c r="E9" s="83" t="inlineStr">
+        <is>
+          <t>B0FVFBZKSQ</t>
+        </is>
+      </c>
+      <c r="F9" s="82" t="inlineStr">
+        <is>
+          <t>DBJ Drawer Cart_wheeled plastic drawers_$0.77_01021180</t>
+        </is>
+      </c>
+      <c r="G9" s="85" t="n">
+        <v>209.97</v>
+      </c>
+      <c r="H9" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" s="23" t="n">
+        <v>3</v>
+      </c>
+      <c r="J9" s="85" t="n">
+        <v>209.97</v>
+      </c>
+      <c r="K9" s="129" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" ht="15" customHeight="1">
+      <c r="A10" s="83" t="inlineStr">
+        <is>
+          <t>W6</t>
+        </is>
+      </c>
+      <c r="B10" s="179" t="inlineStr">
+        <is>
+          <t>03/09</t>
+        </is>
+      </c>
+      <c r="C10" s="180" t="inlineStr">
+        <is>
+          <t>Storage Cart 10D</t>
+        </is>
+      </c>
+      <c r="D10" s="83" t="inlineStr">
+        <is>
+          <t>B0FVFCYKGB</t>
+        </is>
+      </c>
+      <c r="E10" s="83" t="inlineStr">
+        <is>
+          <t>B0FVF9GS2S</t>
+        </is>
+      </c>
+      <c r="F10" s="82" t="inlineStr">
+        <is>
+          <t>DBJ Drawer Cart_utility drawer cart_$0.77_01021180</t>
+        </is>
+      </c>
+      <c r="G10" s="85" t="n">
+        <v>139.98</v>
+      </c>
+      <c r="H10" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="J10" s="85" t="n">
+        <v>139.98</v>
+      </c>
+      <c r="K10" s="129" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" ht="15" customHeight="1">
+      <c r="A11" s="83" t="inlineStr">
+        <is>
+          <t>W6</t>
+        </is>
+      </c>
+      <c r="B11" s="179" t="inlineStr">
+        <is>
+          <t>03/09</t>
+        </is>
+      </c>
+      <c r="C11" s="180" t="inlineStr">
+        <is>
+          <t>Storage Cart 10D</t>
+        </is>
+      </c>
+      <c r="D11" s="83" t="inlineStr">
+        <is>
+          <t>B0FVFCYKGB</t>
+        </is>
+      </c>
+      <c r="E11" s="83" t="inlineStr">
+        <is>
+          <t>B0FVFGJT63</t>
+        </is>
+      </c>
+      <c r="F11" s="82" t="inlineStr">
+        <is>
+          <t>DBJ Drawer Cart_15 drawer craft cart_$0.77_01021180</t>
+        </is>
+      </c>
+      <c r="G11" s="85" t="n">
+        <v>69.98999999999999</v>
+      </c>
+      <c r="H11" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="I11" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="J11" s="85" t="n">
+        <v>69.98999999999999</v>
+      </c>
+      <c r="K11" s="129" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="42" t="inlineStr">
+        <is>
+          <t>6W GRAND TOTAL  (6 rows)</t>
+        </is>
+      </c>
+      <c r="G12" s="181" t="n">
         <v>612.53</v>
       </c>
-      <c r="H5" s="43" t="n">
+      <c r="H12" s="43" t="n">
         <v>6</v>
       </c>
-      <c r="I5" s="43" t="n">
+      <c r="I12" s="43" t="n">
         <v>9</v>
       </c>
-      <c r="J5" s="177" t="n">
+      <c r="J12" s="181" t="n">
         <v>612.53</v>
       </c>
-      <c r="K5" s="44" t="n">
+      <c r="K12" s="44" t="n">
         <v>1</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="9">
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="G2:H2"/>
     <mergeCell ref="E2:F2"/>
+    <mergeCell ref="K2:L2"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A5:K5"/>
     <mergeCell ref="A1:K1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -19099,22 +19407,22 @@
     </row>
     <row r="2" ht="6" customHeight="1"/>
     <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="178" t="inlineStr">
+      <c r="A3" s="182" t="inlineStr">
         <is>
           <t>⭐ Star  (1 個產品)</t>
         </is>
       </c>
-      <c r="C3" s="179" t="inlineStr">
+      <c r="C3" s="183" t="inlineStr">
         <is>
           <t>⚠️ Question  (6 個產品)</t>
         </is>
       </c>
-      <c r="E3" s="180" t="inlineStr">
+      <c r="E3" s="184" t="inlineStr">
         <is>
           <t>🔴 Cut  (6 個產品)</t>
         </is>
       </c>
-      <c r="G3" s="181" t="inlineStr">
+      <c r="G3" s="185" t="inlineStr">
         <is>
           <t>💤 Potential  (1 個產品)</t>
         </is>
@@ -19139,17 +19447,17 @@
       </c>
       <c r="D5" s="46" t="inlineStr">
         <is>
-          <t>5W Sales ($)</t>
+          <t>6W Sales ($)</t>
         </is>
       </c>
       <c r="E5" s="46" t="inlineStr">
         <is>
-          <t>5W Spend ($)</t>
+          <t>6W Spend ($)</t>
         </is>
       </c>
       <c r="F5" s="46" t="inlineStr">
         <is>
-          <t>5W TACOS</t>
+          <t>6W TACOS</t>
         </is>
       </c>
       <c r="G5" s="46" t="inlineStr">
@@ -19179,644 +19487,644 @@
       </c>
     </row>
     <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="182" t="inlineStr">
+      <c r="A6" s="186" t="inlineStr">
         <is>
           <t xml:space="preserve">  ⭐ Star  ·  高銷售 · 低 TACOS  (1 個產品)</t>
         </is>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="183" t="inlineStr">
+      <c r="A7" s="187" t="inlineStr">
         <is>
           <t>⭐ Star</t>
         </is>
       </c>
-      <c r="B7" s="184" t="inlineStr">
+      <c r="B7" s="188" t="inlineStr">
         <is>
           <t>Sweater Hangers</t>
         </is>
       </c>
-      <c r="C7" s="185" t="inlineStr">
+      <c r="C7" s="189" t="inlineStr">
         <is>
           <t>B0CTK9VRFR</t>
         </is>
       </c>
-      <c r="D7" s="186" t="n">
+      <c r="D7" s="190" t="n">
         <v>1093.87</v>
       </c>
-      <c r="E7" s="186" t="n">
+      <c r="E7" s="190" t="n">
         <v>119.62</v>
       </c>
-      <c r="F7" s="187" t="n">
+      <c r="F7" s="191" t="n">
         <v>0.07200000000000001</v>
       </c>
-      <c r="G7" s="188" t="n">
+      <c r="G7" s="192" t="n">
         <v>1</v>
       </c>
-      <c r="H7" s="189" t="n">
+      <c r="H7" s="193" t="n">
         <v>0.2230210196779963</v>
       </c>
-      <c r="I7" s="190" t="n">
+      <c r="I7" s="194" t="n">
         <v>159.88</v>
       </c>
-      <c r="J7" s="191" t="inlineStr">
+      <c r="J7" s="195" t="inlineStr">
         <is>
           <t>擴大預算 · 複製 SP · 加 SB</t>
         </is>
       </c>
-      <c r="K7" s="192" t="inlineStr">
+      <c r="K7" s="196" t="inlineStr">
         <is>
           <t>本週執行</t>
         </is>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1">
-      <c r="A8" s="193" t="inlineStr">
+      <c r="A8" s="197" t="inlineStr">
         <is>
           <t xml:space="preserve">  ⚠️ Question  ·  高銷售 · 高 TACOS  (6 個產品)</t>
         </is>
       </c>
     </row>
     <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="194" t="inlineStr">
+      <c r="A9" s="198" t="inlineStr">
         <is>
           <t>⚠️ Question</t>
         </is>
       </c>
-      <c r="B9" s="195" t="inlineStr">
+      <c r="B9" s="199" t="inlineStr">
         <is>
           <t>Wire Shelving</t>
         </is>
       </c>
-      <c r="C9" s="196" t="inlineStr">
+      <c r="C9" s="200" t="inlineStr">
         <is>
           <t>B09XGY3FQ1</t>
         </is>
       </c>
-      <c r="D9" s="197" t="n">
+      <c r="D9" s="201" t="n">
         <v>9567.030000000001</v>
       </c>
-      <c r="E9" s="197" t="n">
+      <c r="E9" s="201" t="n">
         <v>2342.14</v>
       </c>
-      <c r="F9" s="198" t="n">
+      <c r="F9" s="202" t="n">
         <v>0.178</v>
       </c>
-      <c r="G9" s="199" t="n">
+      <c r="G9" s="203" t="n">
         <v>1</v>
       </c>
-      <c r="H9" s="200" t="n">
+      <c r="H9" s="204" t="n">
         <v>9.696589892665475</v>
       </c>
-      <c r="I9" s="201" t="n">
+      <c r="I9" s="205" t="n">
         <v>3607.68</v>
       </c>
-      <c r="J9" s="202" t="inlineStr">
+      <c r="J9" s="206" t="inlineStr">
         <is>
           <t>降 CPC · 暫停高 ACOS KW</t>
         </is>
       </c>
-      <c r="K9" s="203" t="inlineStr">
+      <c r="K9" s="207" t="inlineStr">
         <is>
           <t>本週執行</t>
         </is>
       </c>
     </row>
     <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="194" t="inlineStr">
+      <c r="A10" s="198" t="inlineStr">
         <is>
           <t>⚠️ Question</t>
         </is>
       </c>
-      <c r="B10" s="195" t="inlineStr">
+      <c r="B10" s="199" t="inlineStr">
         <is>
           <t>Storage Cart 10D</t>
         </is>
       </c>
-      <c r="C10" s="196" t="inlineStr">
+      <c r="C10" s="200" t="inlineStr">
         <is>
           <t>B0FVFCYKGB</t>
         </is>
       </c>
-      <c r="D10" s="197" t="n">
+      <c r="D10" s="201" t="n">
         <v>7164.24</v>
       </c>
-      <c r="E10" s="197" t="n">
+      <c r="E10" s="201" t="n">
         <v>2772.11</v>
       </c>
-      <c r="F10" s="204" t="n">
+      <c r="F10" s="208" t="n">
         <v>0.347</v>
       </c>
-      <c r="G10" s="199" t="n">
+      <c r="G10" s="203" t="n">
         <v>2</v>
       </c>
-      <c r="H10" s="200" t="n">
+      <c r="H10" s="204" t="n">
         <v>7.01010733452594</v>
       </c>
-      <c r="I10" s="201" t="n">
+      <c r="I10" s="205" t="n">
         <v>4771.31</v>
       </c>
-      <c r="J10" s="202" t="inlineStr">
+      <c r="J10" s="206" t="inlineStr">
         <is>
           <t>降 CPC · 暫停高 ACOS KW</t>
         </is>
       </c>
-      <c r="K10" s="203" t="inlineStr">
+      <c r="K10" s="207" t="inlineStr">
         <is>
           <t>本週執行</t>
         </is>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
-      <c r="A11" s="194" t="inlineStr">
+      <c r="A11" s="198" t="inlineStr">
         <is>
           <t>⚠️ Question</t>
         </is>
       </c>
-      <c r="B11" s="195" t="inlineStr">
+      <c r="B11" s="199" t="inlineStr">
         <is>
           <t>Laptop Stand A</t>
         </is>
       </c>
-      <c r="C11" s="196" t="inlineStr">
+      <c r="C11" s="200" t="inlineStr">
         <is>
           <t>B0FVD69MYD</t>
         </is>
       </c>
-      <c r="D11" s="197" t="n">
+      <c r="D11" s="201" t="n">
         <v>1451.02</v>
       </c>
-      <c r="E11" s="197" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" s="205" t="n"/>
-      <c r="G11" s="199" t="n">
+      <c r="E11" s="201" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="209" t="n"/>
+      <c r="G11" s="203" t="n">
         <v>3</v>
       </c>
-      <c r="H11" s="200" t="n">
+      <c r="H11" s="204" t="n">
         <v>0.6223389982110913</v>
       </c>
-      <c r="I11" s="201" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" s="202" t="inlineStr">
+      <c r="I11" s="205" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="206" t="inlineStr">
         <is>
           <t>降 CPC · 暫停高 ACOS KW</t>
         </is>
       </c>
-      <c r="K11" s="203" t="inlineStr">
+      <c r="K11" s="207" t="inlineStr">
         <is>
           <t>本週執行</t>
         </is>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="194" t="inlineStr">
+      <c r="A12" s="198" t="inlineStr">
         <is>
           <t>⚠️ Question</t>
         </is>
       </c>
-      <c r="B12" s="195" t="inlineStr">
+      <c r="B12" s="199" t="inlineStr">
         <is>
           <t>Dryer Rack</t>
         </is>
       </c>
-      <c r="C12" s="196" t="inlineStr">
+      <c r="C12" s="200" t="inlineStr">
         <is>
           <t>B097V3JSWH</t>
         </is>
       </c>
-      <c r="D12" s="197" t="n">
+      <c r="D12" s="201" t="n">
         <v>1329.7</v>
       </c>
-      <c r="E12" s="197" t="n">
+      <c r="E12" s="201" t="n">
         <v>337.9</v>
       </c>
-      <c r="F12" s="204" t="n">
+      <c r="F12" s="208" t="n">
         <v>0.294</v>
       </c>
-      <c r="G12" s="199" t="n">
+      <c r="G12" s="203" t="n">
         <v>4</v>
       </c>
-      <c r="H12" s="200" t="n">
+      <c r="H12" s="204" t="n">
         <v>0.4866949910554563</v>
       </c>
-      <c r="I12" s="201" t="n">
+      <c r="I12" s="205" t="n">
         <v>130.99</v>
       </c>
-      <c r="J12" s="202" t="inlineStr">
+      <c r="J12" s="206" t="inlineStr">
         <is>
           <t>降 CPC · 暫停高 ACOS KW</t>
         </is>
       </c>
-      <c r="K12" s="203" t="inlineStr">
+      <c r="K12" s="207" t="inlineStr">
         <is>
           <t>本週執行</t>
         </is>
       </c>
     </row>
     <row r="13" ht="16" customHeight="1">
-      <c r="A13" s="194" t="inlineStr">
+      <c r="A13" s="198" t="inlineStr">
         <is>
           <t>⚠️ Question</t>
         </is>
       </c>
-      <c r="B13" s="195" t="inlineStr">
+      <c r="B13" s="199" t="inlineStr">
         <is>
           <t>Laptop Stand B</t>
         </is>
       </c>
-      <c r="C13" s="196" t="inlineStr">
+      <c r="C13" s="200" t="inlineStr">
         <is>
           <t>B0FVD1Z92C</t>
         </is>
       </c>
-      <c r="D13" s="197" t="n">
+      <c r="D13" s="201" t="n">
         <v>1232.16</v>
       </c>
-      <c r="E13" s="197" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" s="205" t="n"/>
-      <c r="G13" s="199" t="n">
+      <c r="E13" s="201" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="209" t="n"/>
+      <c r="G13" s="203" t="n">
         <v>5</v>
       </c>
-      <c r="H13" s="200" t="n">
+      <c r="H13" s="204" t="n">
         <v>0.3776386404293383</v>
       </c>
-      <c r="I13" s="201" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" s="202" t="inlineStr">
+      <c r="I13" s="205" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="206" t="inlineStr">
         <is>
           <t>降 CPC · 暫停高 ACOS KW</t>
         </is>
       </c>
-      <c r="K13" s="203" t="inlineStr">
+      <c r="K13" s="207" t="inlineStr">
         <is>
           <t>本週執行</t>
         </is>
       </c>
     </row>
     <row r="14" ht="16" customHeight="1">
-      <c r="A14" s="194" t="inlineStr">
+      <c r="A14" s="198" t="inlineStr">
         <is>
           <t>⚠️ Question</t>
         </is>
       </c>
-      <c r="B14" s="195" t="inlineStr">
+      <c r="B14" s="199" t="inlineStr">
         <is>
           <t>Bathroom Storage</t>
         </is>
       </c>
-      <c r="C14" s="196" t="inlineStr">
+      <c r="C14" s="200" t="inlineStr">
         <is>
           <t>B0FVFCJXWB</t>
         </is>
       </c>
-      <c r="D14" s="197" t="n">
+      <c r="D14" s="201" t="n">
         <v>901.4299999999999</v>
       </c>
-      <c r="E14" s="197" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" s="205" t="n"/>
-      <c r="G14" s="199" t="n">
+      <c r="E14" s="201" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="209" t="n"/>
+      <c r="G14" s="203" t="n">
         <v>6</v>
       </c>
-      <c r="H14" s="200" t="n">
+      <c r="H14" s="204" t="n">
         <v>0.007860017889087627</v>
       </c>
-      <c r="I14" s="201" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" s="202" t="inlineStr">
+      <c r="I14" s="205" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="206" t="inlineStr">
         <is>
           <t>降 CPC · 暫停高 ACOS KW</t>
         </is>
       </c>
-      <c r="K14" s="203" t="inlineStr">
+      <c r="K14" s="207" t="inlineStr">
         <is>
           <t>本週執行</t>
         </is>
       </c>
     </row>
     <row r="15" ht="16" customHeight="1">
-      <c r="A15" s="206" t="inlineStr">
+      <c r="A15" s="210" t="inlineStr">
         <is>
           <t xml:space="preserve">  🔴 Cut  ·  低銷售 · 高 TACOS  (6 個產品)</t>
         </is>
       </c>
     </row>
     <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="207" t="inlineStr">
+      <c r="A16" s="211" t="inlineStr">
         <is>
           <t>🔴 Cut</t>
         </is>
       </c>
-      <c r="B16" s="208" t="inlineStr">
+      <c r="B16" s="212" t="inlineStr">
         <is>
           <t>Double Rail Rack</t>
         </is>
       </c>
-      <c r="C16" s="209" t="inlineStr">
+      <c r="C16" s="213" t="inlineStr">
         <is>
           <t>B0FV8XGQV4</t>
         </is>
       </c>
-      <c r="D16" s="210" t="n">
+      <c r="D16" s="214" t="n">
         <v>887.37</v>
       </c>
-      <c r="E16" s="210" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" s="211" t="n"/>
-      <c r="G16" s="212" t="n">
+      <c r="E16" s="214" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="215" t="n"/>
+      <c r="G16" s="216" t="n">
         <v>1</v>
       </c>
-      <c r="H16" s="213" t="n">
+      <c r="H16" s="217" t="n">
         <v>-0.007860017889087627</v>
       </c>
-      <c r="I16" s="214" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" s="215" t="inlineStr">
+      <c r="I16" s="218" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="219" t="inlineStr">
         <is>
           <t>降價 · Coupon · 降 Bid</t>
         </is>
       </c>
-      <c r="K16" s="216" t="inlineStr">
+      <c r="K16" s="220" t="inlineStr">
         <is>
           <t>本週執行</t>
         </is>
       </c>
     </row>
     <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="207" t="inlineStr">
+      <c r="A17" s="211" t="inlineStr">
         <is>
           <t>🔴 Cut</t>
         </is>
       </c>
-      <c r="B17" s="208" t="inlineStr">
+      <c r="B17" s="212" t="inlineStr">
         <is>
           <t>3-Tier Cart</t>
         </is>
       </c>
-      <c r="C17" s="209" t="inlineStr">
+      <c r="C17" s="213" t="inlineStr">
         <is>
           <t>B0FV8YD8DP</t>
         </is>
       </c>
-      <c r="D17" s="210" t="n">
+      <c r="D17" s="214" t="n">
         <v>804.89</v>
       </c>
-      <c r="E17" s="210" t="n">
+      <c r="E17" s="214" t="n">
         <v>40.76</v>
       </c>
-      <c r="F17" s="217" t="n">
+      <c r="F17" s="221" t="n">
         <v>0.3</v>
       </c>
-      <c r="G17" s="212" t="n">
+      <c r="G17" s="216" t="n">
         <v>2</v>
       </c>
-      <c r="H17" s="213" t="n">
+      <c r="H17" s="217" t="n">
         <v>-0.1000782647584973</v>
       </c>
-      <c r="I17" s="214" t="n">
+      <c r="I17" s="218" t="n">
         <v>33.99</v>
       </c>
-      <c r="J17" s="215" t="inlineStr">
+      <c r="J17" s="219" t="inlineStr">
         <is>
           <t>降價 · Coupon · 降 Bid</t>
         </is>
       </c>
-      <c r="K17" s="216" t="inlineStr">
+      <c r="K17" s="220" t="inlineStr">
         <is>
           <t>本週執行</t>
         </is>
       </c>
     </row>
     <row r="18" ht="16" customHeight="1">
-      <c r="A18" s="207" t="inlineStr">
+      <c r="A18" s="211" t="inlineStr">
         <is>
           <t>🔴 Cut</t>
         </is>
       </c>
-      <c r="B18" s="208" t="inlineStr">
+      <c r="B18" s="212" t="inlineStr">
         <is>
           <t>Laptop Stand C</t>
         </is>
       </c>
-      <c r="C18" s="209" t="inlineStr">
+      <c r="C18" s="213" t="inlineStr">
         <is>
           <t>B0FVF8DRZQ</t>
         </is>
       </c>
-      <c r="D18" s="210" t="n">
+      <c r="D18" s="214" t="n">
         <v>670.66</v>
       </c>
-      <c r="E18" s="210" t="n">
-        <v>0</v>
-      </c>
-      <c r="F18" s="211" t="n"/>
-      <c r="G18" s="212" t="n">
+      <c r="E18" s="214" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="215" t="n"/>
+      <c r="G18" s="216" t="n">
         <v>3</v>
       </c>
-      <c r="H18" s="213" t="n">
+      <c r="H18" s="217" t="n">
         <v>-0.2501565295169946</v>
       </c>
-      <c r="I18" s="214" t="n">
-        <v>0</v>
-      </c>
-      <c r="J18" s="215" t="inlineStr">
+      <c r="I18" s="218" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" s="219" t="inlineStr">
         <is>
           <t>降價 · Coupon · 降 Bid</t>
         </is>
       </c>
-      <c r="K18" s="216" t="inlineStr">
+      <c r="K18" s="220" t="inlineStr">
         <is>
           <t>本週執行</t>
         </is>
       </c>
     </row>
     <row r="19" ht="16" customHeight="1">
-      <c r="A19" s="207" t="inlineStr">
+      <c r="A19" s="211" t="inlineStr">
         <is>
           <t>🔴 Cut</t>
         </is>
       </c>
-      <c r="B19" s="208" t="inlineStr">
+      <c r="B19" s="212" t="inlineStr">
         <is>
           <t>Shoe Rack</t>
         </is>
       </c>
-      <c r="C19" s="209" t="inlineStr">
+      <c r="C19" s="213" t="inlineStr">
         <is>
           <t>B0FVFG8W4X</t>
         </is>
       </c>
-      <c r="D19" s="210" t="n">
+      <c r="D19" s="214" t="n">
         <v>616.51</v>
       </c>
-      <c r="E19" s="210" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" s="211" t="n"/>
-      <c r="G19" s="212" t="n">
+      <c r="E19" s="214" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="215" t="n"/>
+      <c r="G19" s="216" t="n">
         <v>4</v>
       </c>
-      <c r="H19" s="213" t="n">
+      <c r="H19" s="217" t="n">
         <v>-0.3106999105545617</v>
       </c>
-      <c r="I19" s="214" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" s="215" t="inlineStr">
+      <c r="I19" s="218" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" s="219" t="inlineStr">
         <is>
           <t>降價 · Coupon · 降 Bid</t>
         </is>
       </c>
-      <c r="K19" s="216" t="inlineStr">
+      <c r="K19" s="220" t="inlineStr">
         <is>
           <t>本週執行</t>
         </is>
       </c>
     </row>
     <row r="20" ht="16" customHeight="1">
-      <c r="A20" s="207" t="inlineStr">
+      <c r="A20" s="211" t="inlineStr">
         <is>
           <t>🔴 Cut</t>
         </is>
       </c>
-      <c r="B20" s="208" t="inlineStr">
+      <c r="B20" s="212" t="inlineStr">
         <is>
           <t>Broom Holder</t>
         </is>
       </c>
-      <c r="C20" s="209" t="inlineStr">
+      <c r="C20" s="213" t="inlineStr">
         <is>
           <t>B09JBVTY9T</t>
         </is>
       </c>
-      <c r="D20" s="210" t="n">
+      <c r="D20" s="214" t="n">
         <v>276.37</v>
       </c>
-      <c r="E20" s="210" t="n">
+      <c r="E20" s="214" t="n">
         <v>82.79000000000001</v>
       </c>
-      <c r="F20" s="217" t="n">
+      <c r="F20" s="221" t="n">
         <v>0.185</v>
       </c>
-      <c r="G20" s="212" t="n">
+      <c r="G20" s="216" t="n">
         <v>5</v>
       </c>
-      <c r="H20" s="213" t="n">
+      <c r="H20" s="217" t="n">
         <v>-0.6909995527728086</v>
       </c>
-      <c r="I20" s="214" t="n">
+      <c r="I20" s="218" t="n">
         <v>14.46</v>
       </c>
-      <c r="J20" s="215" t="inlineStr">
+      <c r="J20" s="219" t="inlineStr">
         <is>
           <t>降價 · Coupon · 降 Bid</t>
         </is>
       </c>
-      <c r="K20" s="216" t="inlineStr">
+      <c r="K20" s="220" t="inlineStr">
         <is>
           <t>本週執行</t>
         </is>
       </c>
     </row>
     <row r="21" ht="16" customHeight="1">
-      <c r="A21" s="207" t="inlineStr">
+      <c r="A21" s="211" t="inlineStr">
         <is>
           <t>🔴 Cut</t>
         </is>
       </c>
-      <c r="B21" s="208" t="inlineStr">
+      <c r="B21" s="212" t="inlineStr">
         <is>
           <t>Shower Caddy</t>
         </is>
       </c>
-      <c r="C21" s="209" t="inlineStr">
+      <c r="C21" s="213" t="inlineStr">
         <is>
           <t>B09MRGLH3L</t>
         </is>
       </c>
-      <c r="D21" s="210" t="n">
+      <c r="D21" s="214" t="n">
         <v>38.72</v>
       </c>
-      <c r="E21" s="210" t="n">
-        <v>0</v>
-      </c>
-      <c r="F21" s="211" t="n"/>
-      <c r="G21" s="212" t="n">
+      <c r="E21" s="214" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="215" t="n"/>
+      <c r="G21" s="216" t="n">
         <v>6</v>
       </c>
-      <c r="H21" s="213" t="n">
+      <c r="H21" s="217" t="n">
         <v>-0.9567084078711985</v>
       </c>
-      <c r="I21" s="214" t="n">
-        <v>0</v>
-      </c>
-      <c r="J21" s="215" t="inlineStr">
+      <c r="I21" s="218" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" s="219" t="inlineStr">
         <is>
           <t>降價 · Coupon · 降 Bid</t>
         </is>
       </c>
-      <c r="K21" s="216" t="inlineStr">
+      <c r="K21" s="220" t="inlineStr">
         <is>
           <t>本週執行</t>
         </is>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
-      <c r="A22" s="218" t="inlineStr">
+      <c r="A22" s="222" t="inlineStr">
         <is>
           <t xml:space="preserve">  💤 Potential  ·  低銷售 · 低 TACOS  (1 個產品)</t>
         </is>
       </c>
     </row>
     <row r="23" ht="16" customHeight="1">
-      <c r="A23" s="219" t="inlineStr">
+      <c r="A23" s="223" t="inlineStr">
         <is>
           <t>💤 Potential</t>
         </is>
       </c>
-      <c r="B23" s="220" t="inlineStr">
+      <c r="B23" s="224" t="inlineStr">
         <is>
           <t>Padded Hangers</t>
         </is>
       </c>
-      <c r="C23" s="221" t="inlineStr">
+      <c r="C23" s="225" t="inlineStr">
         <is>
           <t>B09R3BLFDT</t>
         </is>
       </c>
-      <c r="D23" s="222" t="n">
+      <c r="D23" s="226" t="n">
         <v>734.41</v>
       </c>
-      <c r="E23" s="222" t="n">
+      <c r="E23" s="226" t="n">
         <v>58.23</v>
       </c>
-      <c r="F23" s="223" t="n">
+      <c r="F23" s="227" t="n">
         <v>0.09300000000000001</v>
       </c>
-      <c r="G23" s="224" t="n">
+      <c r="G23" s="228" t="n">
         <v>1</v>
       </c>
-      <c r="H23" s="225" t="n">
+      <c r="H23" s="229" t="n">
         <v>-0.1788796958855099</v>
       </c>
-      <c r="I23" s="226" t="n">
-        <v>0</v>
-      </c>
-      <c r="J23" s="227" t="inlineStr">
+      <c r="I23" s="230" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" s="231" t="inlineStr">
         <is>
           <t>新建 SP/SB/SD · AMC Lookalike</t>
         </is>
       </c>
-      <c r="K23" s="228" t="inlineStr">
+      <c r="K23" s="232" t="inlineStr">
         <is>
           <t>下週執行</t>
         </is>
@@ -19899,7 +20207,7 @@
       </c>
       <c r="G3" s="46" t="inlineStr">
         <is>
-          <t>5W Sales</t>
+          <t>6W Sales</t>
         </is>
       </c>
       <c r="H3" s="46" t="inlineStr">
@@ -19909,1408 +20217,1408 @@
       </c>
     </row>
     <row r="4" ht="15" customHeight="1">
-      <c r="A4" s="182" t="inlineStr">
+      <c r="A4" s="186" t="inlineStr">
         <is>
           <t xml:space="preserve">  ⭐ Star  —  高銷售 · 低 TACOS</t>
         </is>
       </c>
     </row>
     <row r="5" ht="28" customHeight="1">
-      <c r="A5" s="229" t="inlineStr"/>
-      <c r="B5" s="184" t="inlineStr">
+      <c r="A5" s="233" t="inlineStr"/>
+      <c r="B5" s="188" t="inlineStr">
         <is>
           <t>Sweater Hangers</t>
         </is>
       </c>
-      <c r="C5" s="183" t="inlineStr">
+      <c r="C5" s="187" t="inlineStr">
         <is>
           <t>⭐ Star</t>
         </is>
       </c>
-      <c r="D5" s="192" t="inlineStr">
+      <c r="D5" s="196" t="inlineStr">
         <is>
           <t>本週執行</t>
         </is>
       </c>
-      <c r="E5" s="185" t="inlineStr">
+      <c r="E5" s="189" t="inlineStr">
         <is>
           <t>SP Bulk</t>
         </is>
       </c>
-      <c r="F5" s="230" t="inlineStr">
+      <c r="F5" s="234" t="inlineStr">
         <is>
           <t>下載現有 SP 活動 Bulk File → 複製所有 Enabled campaigns → 新命名加 _COPY 後綴</t>
         </is>
       </c>
-      <c r="G5" s="186" t="n">
+      <c r="G5" s="190" t="n">
         <v>1093.87</v>
       </c>
-      <c r="H5" s="187" t="n">
+      <c r="H5" s="191" t="n">
         <v>0.07200000000000001</v>
       </c>
     </row>
     <row r="6" ht="28" customHeight="1">
-      <c r="A6" s="229" t="inlineStr"/>
-      <c r="B6" s="231" t="n"/>
-      <c r="C6" s="231" t="n"/>
-      <c r="D6" s="231" t="n"/>
-      <c r="E6" s="185" t="inlineStr">
+      <c r="A6" s="233" t="inlineStr"/>
+      <c r="B6" s="235" t="n"/>
+      <c r="C6" s="235" t="n"/>
+      <c r="D6" s="235" t="n"/>
+      <c r="E6" s="189" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
       </c>
-      <c r="F6" s="230" t="inlineStr">
+      <c r="F6" s="234" t="inlineStr">
         <is>
           <t>全部 SP 活動預算 × 1.3（+30%）→ 上傳 Bulk File → 確認無錯誤</t>
         </is>
       </c>
-      <c r="G6" s="231" t="n"/>
-      <c r="H6" s="231" t="n"/>
+      <c r="G6" s="235" t="n"/>
+      <c r="H6" s="235" t="n"/>
     </row>
     <row r="7" ht="28" customHeight="1">
-      <c r="A7" s="229" t="inlineStr"/>
-      <c r="B7" s="231" t="n"/>
-      <c r="C7" s="231" t="n"/>
-      <c r="D7" s="231" t="n"/>
-      <c r="E7" s="185" t="inlineStr">
+      <c r="A7" s="233" t="inlineStr"/>
+      <c r="B7" s="235" t="n"/>
+      <c r="C7" s="235" t="n"/>
+      <c r="D7" s="235" t="n"/>
+      <c r="E7" s="189" t="inlineStr">
         <is>
           <t>SB</t>
         </is>
       </c>
-      <c r="F7" s="230" t="inlineStr">
+      <c r="F7" s="234" t="inlineStr">
         <is>
           <t>確認是否有 SB Banner 廣告，若無則新建 SB Campaign 指向此產品</t>
         </is>
       </c>
-      <c r="G7" s="231" t="n"/>
-      <c r="H7" s="231" t="n"/>
+      <c r="G7" s="235" t="n"/>
+      <c r="H7" s="235" t="n"/>
     </row>
     <row r="8" ht="28" customHeight="1">
-      <c r="A8" s="229" t="inlineStr"/>
-      <c r="B8" s="231" t="n"/>
-      <c r="C8" s="231" t="n"/>
-      <c r="D8" s="231" t="n"/>
-      <c r="E8" s="185" t="inlineStr">
+      <c r="A8" s="233" t="inlineStr"/>
+      <c r="B8" s="235" t="n"/>
+      <c r="C8" s="235" t="n"/>
+      <c r="D8" s="235" t="n"/>
+      <c r="E8" s="189" t="inlineStr">
         <is>
           <t>SD</t>
         </is>
       </c>
-      <c r="F8" s="230" t="inlineStr">
+      <c r="F8" s="234" t="inlineStr">
         <is>
           <t>建立 SD Retargeting 活動 targeting 已瀏覽 ASIN 的受眾</t>
         </is>
       </c>
-      <c r="G8" s="231" t="n"/>
-      <c r="H8" s="231" t="n"/>
+      <c r="G8" s="235" t="n"/>
+      <c r="H8" s="235" t="n"/>
     </row>
     <row r="9" ht="4" customHeight="1">
-      <c r="A9" s="232" t="n"/>
-      <c r="B9" s="232" t="n"/>
-      <c r="C9" s="232" t="n"/>
-      <c r="D9" s="232" t="n"/>
-      <c r="E9" s="232" t="n"/>
-      <c r="F9" s="232" t="n"/>
-      <c r="G9" s="232" t="n"/>
-      <c r="H9" s="232" t="n"/>
+      <c r="A9" s="236" t="n"/>
+      <c r="B9" s="236" t="n"/>
+      <c r="C9" s="236" t="n"/>
+      <c r="D9" s="236" t="n"/>
+      <c r="E9" s="236" t="n"/>
+      <c r="F9" s="236" t="n"/>
+      <c r="G9" s="236" t="n"/>
+      <c r="H9" s="236" t="n"/>
     </row>
     <row r="10" ht="15" customHeight="1">
-      <c r="A10" s="193" t="inlineStr">
+      <c r="A10" s="197" t="inlineStr">
         <is>
           <t xml:space="preserve">  ⚠️ Question  —  高銷售 · 高 TACOS</t>
         </is>
       </c>
     </row>
     <row r="11" ht="28" customHeight="1">
-      <c r="A11" s="233" t="inlineStr"/>
-      <c r="B11" s="195" t="inlineStr">
+      <c r="A11" s="237" t="inlineStr"/>
+      <c r="B11" s="199" t="inlineStr">
         <is>
           <t>Wire Shelving</t>
         </is>
       </c>
-      <c r="C11" s="194" t="inlineStr">
+      <c r="C11" s="198" t="inlineStr">
         <is>
           <t>⚠️ Question</t>
         </is>
       </c>
-      <c r="D11" s="203" t="inlineStr">
+      <c r="D11" s="207" t="inlineStr">
         <is>
           <t>本週執行</t>
         </is>
       </c>
-      <c r="E11" s="196" t="inlineStr">
+      <c r="E11" s="200" t="inlineStr">
         <is>
           <t>CPC</t>
         </is>
       </c>
-      <c r="F11" s="234" t="inlineStr">
+      <c r="F11" s="238" t="inlineStr">
         <is>
           <t>下載 SP Bulk File → 找出 ACOS ≥85% 的關鍵字 → Bid × 0.8（降 20%）</t>
         </is>
       </c>
-      <c r="G11" s="197" t="n">
+      <c r="G11" s="201" t="n">
         <v>9567.030000000001</v>
       </c>
-      <c r="H11" s="198" t="n">
+      <c r="H11" s="202" t="n">
         <v>0.178</v>
       </c>
     </row>
     <row r="12" ht="28" customHeight="1">
-      <c r="A12" s="233" t="inlineStr"/>
-      <c r="B12" s="235" t="n"/>
-      <c r="C12" s="235" t="n"/>
-      <c r="D12" s="235" t="n"/>
-      <c r="E12" s="196" t="inlineStr">
+      <c r="A12" s="237" t="inlineStr"/>
+      <c r="B12" s="239" t="n"/>
+      <c r="C12" s="239" t="n"/>
+      <c r="D12" s="239" t="n"/>
+      <c r="E12" s="200" t="inlineStr">
         <is>
           <t>Pause KW</t>
         </is>
       </c>
-      <c r="F12" s="234" t="inlineStr">
+      <c r="F12" s="238" t="inlineStr">
         <is>
           <t>TACOS ≥85% 且過去 14 天無轉換的關鍵字 → 狀態改為 Paused</t>
         </is>
       </c>
-      <c r="G12" s="235" t="n"/>
-      <c r="H12" s="235" t="n"/>
+      <c r="G12" s="239" t="n"/>
+      <c r="H12" s="239" t="n"/>
     </row>
     <row r="13" ht="28" customHeight="1">
-      <c r="A13" s="233" t="inlineStr"/>
-      <c r="B13" s="235" t="n"/>
-      <c r="C13" s="235" t="n"/>
-      <c r="D13" s="235" t="n"/>
-      <c r="E13" s="196" t="inlineStr">
+      <c r="A13" s="237" t="inlineStr"/>
+      <c r="B13" s="239" t="n"/>
+      <c r="C13" s="239" t="n"/>
+      <c r="D13" s="239" t="n"/>
+      <c r="E13" s="200" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
       </c>
-      <c r="F13" s="234" t="inlineStr">
+      <c r="F13" s="238" t="inlineStr">
         <is>
           <t>SP 活動預算維持不變，待 TACOS 下降再考慮增加</t>
         </is>
       </c>
-      <c r="G13" s="235" t="n"/>
-      <c r="H13" s="235" t="n"/>
+      <c r="G13" s="239" t="n"/>
+      <c r="H13" s="239" t="n"/>
     </row>
     <row r="14" ht="28" customHeight="1">
-      <c r="A14" s="233" t="inlineStr"/>
-      <c r="B14" s="235" t="n"/>
-      <c r="C14" s="235" t="n"/>
-      <c r="D14" s="235" t="n"/>
-      <c r="E14" s="196" t="inlineStr">
+      <c r="A14" s="237" t="inlineStr"/>
+      <c r="B14" s="239" t="n"/>
+      <c r="C14" s="239" t="n"/>
+      <c r="D14" s="239" t="n"/>
+      <c r="E14" s="200" t="inlineStr">
         <is>
           <t>Review</t>
         </is>
       </c>
-      <c r="F14" s="234" t="inlineStr">
+      <c r="F14" s="238" t="inlineStr">
         <is>
           <t>檢查競品 listing 定價，評估是否需要調整售價提高轉換率</t>
         </is>
       </c>
-      <c r="G14" s="235" t="n"/>
-      <c r="H14" s="235" t="n"/>
+      <c r="G14" s="239" t="n"/>
+      <c r="H14" s="239" t="n"/>
     </row>
     <row r="15" ht="4" customHeight="1">
-      <c r="A15" s="232" t="n"/>
-      <c r="B15" s="232" t="n"/>
-      <c r="C15" s="232" t="n"/>
-      <c r="D15" s="232" t="n"/>
-      <c r="E15" s="232" t="n"/>
-      <c r="F15" s="232" t="n"/>
-      <c r="G15" s="232" t="n"/>
-      <c r="H15" s="232" t="n"/>
+      <c r="A15" s="236" t="n"/>
+      <c r="B15" s="236" t="n"/>
+      <c r="C15" s="236" t="n"/>
+      <c r="D15" s="236" t="n"/>
+      <c r="E15" s="236" t="n"/>
+      <c r="F15" s="236" t="n"/>
+      <c r="G15" s="236" t="n"/>
+      <c r="H15" s="236" t="n"/>
     </row>
     <row r="16" ht="28" customHeight="1">
-      <c r="A16" s="233" t="inlineStr"/>
-      <c r="B16" s="195" t="inlineStr">
+      <c r="A16" s="237" t="inlineStr"/>
+      <c r="B16" s="199" t="inlineStr">
         <is>
           <t>Storage Cart 10D</t>
         </is>
       </c>
-      <c r="C16" s="194" t="inlineStr">
+      <c r="C16" s="198" t="inlineStr">
         <is>
           <t>⚠️ Question</t>
         </is>
       </c>
-      <c r="D16" s="203" t="inlineStr">
+      <c r="D16" s="207" t="inlineStr">
         <is>
           <t>本週執行</t>
         </is>
       </c>
-      <c r="E16" s="196" t="inlineStr">
+      <c r="E16" s="200" t="inlineStr">
         <is>
           <t>CPC</t>
         </is>
       </c>
-      <c r="F16" s="234" t="inlineStr">
+      <c r="F16" s="238" t="inlineStr">
         <is>
           <t>下載 SP Bulk File → 找出 ACOS ≥85% 的關鍵字 → Bid × 0.8（降 20%）</t>
         </is>
       </c>
-      <c r="G16" s="197" t="n">
+      <c r="G16" s="201" t="n">
         <v>7164.24</v>
       </c>
-      <c r="H16" s="204" t="n">
+      <c r="H16" s="208" t="n">
         <v>0.347</v>
       </c>
     </row>
     <row r="17" ht="28" customHeight="1">
-      <c r="A17" s="233" t="inlineStr"/>
-      <c r="B17" s="235" t="n"/>
-      <c r="C17" s="235" t="n"/>
-      <c r="D17" s="235" t="n"/>
-      <c r="E17" s="196" t="inlineStr">
+      <c r="A17" s="237" t="inlineStr"/>
+      <c r="B17" s="239" t="n"/>
+      <c r="C17" s="239" t="n"/>
+      <c r="D17" s="239" t="n"/>
+      <c r="E17" s="200" t="inlineStr">
         <is>
           <t>Pause KW</t>
         </is>
       </c>
-      <c r="F17" s="234" t="inlineStr">
+      <c r="F17" s="238" t="inlineStr">
         <is>
           <t>TACOS ≥85% 且過去 14 天無轉換的關鍵字 → 狀態改為 Paused</t>
         </is>
       </c>
-      <c r="G17" s="235" t="n"/>
-      <c r="H17" s="235" t="n"/>
+      <c r="G17" s="239" t="n"/>
+      <c r="H17" s="239" t="n"/>
     </row>
     <row r="18" ht="28" customHeight="1">
-      <c r="A18" s="233" t="inlineStr"/>
-      <c r="B18" s="235" t="n"/>
-      <c r="C18" s="235" t="n"/>
-      <c r="D18" s="235" t="n"/>
-      <c r="E18" s="196" t="inlineStr">
+      <c r="A18" s="237" t="inlineStr"/>
+      <c r="B18" s="239" t="n"/>
+      <c r="C18" s="239" t="n"/>
+      <c r="D18" s="239" t="n"/>
+      <c r="E18" s="200" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
       </c>
-      <c r="F18" s="234" t="inlineStr">
+      <c r="F18" s="238" t="inlineStr">
         <is>
           <t>SP 活動預算維持不變，待 TACOS 下降再考慮增加</t>
         </is>
       </c>
-      <c r="G18" s="235" t="n"/>
-      <c r="H18" s="235" t="n"/>
+      <c r="G18" s="239" t="n"/>
+      <c r="H18" s="239" t="n"/>
     </row>
     <row r="19" ht="28" customHeight="1">
-      <c r="A19" s="233" t="inlineStr"/>
-      <c r="B19" s="235" t="n"/>
-      <c r="C19" s="235" t="n"/>
-      <c r="D19" s="235" t="n"/>
-      <c r="E19" s="196" t="inlineStr">
+      <c r="A19" s="237" t="inlineStr"/>
+      <c r="B19" s="239" t="n"/>
+      <c r="C19" s="239" t="n"/>
+      <c r="D19" s="239" t="n"/>
+      <c r="E19" s="200" t="inlineStr">
         <is>
           <t>Review</t>
         </is>
       </c>
-      <c r="F19" s="234" t="inlineStr">
+      <c r="F19" s="238" t="inlineStr">
         <is>
           <t>檢查競品 listing 定價，評估是否需要調整售價提高轉換率</t>
         </is>
       </c>
-      <c r="G19" s="235" t="n"/>
-      <c r="H19" s="235" t="n"/>
+      <c r="G19" s="239" t="n"/>
+      <c r="H19" s="239" t="n"/>
     </row>
     <row r="20" ht="4" customHeight="1">
-      <c r="A20" s="232" t="n"/>
-      <c r="B20" s="232" t="n"/>
-      <c r="C20" s="232" t="n"/>
-      <c r="D20" s="232" t="n"/>
-      <c r="E20" s="232" t="n"/>
-      <c r="F20" s="232" t="n"/>
-      <c r="G20" s="232" t="n"/>
-      <c r="H20" s="232" t="n"/>
+      <c r="A20" s="236" t="n"/>
+      <c r="B20" s="236" t="n"/>
+      <c r="C20" s="236" t="n"/>
+      <c r="D20" s="236" t="n"/>
+      <c r="E20" s="236" t="n"/>
+      <c r="F20" s="236" t="n"/>
+      <c r="G20" s="236" t="n"/>
+      <c r="H20" s="236" t="n"/>
     </row>
     <row r="21" ht="28" customHeight="1">
-      <c r="A21" s="233" t="inlineStr"/>
-      <c r="B21" s="195" t="inlineStr">
+      <c r="A21" s="237" t="inlineStr"/>
+      <c r="B21" s="199" t="inlineStr">
         <is>
           <t>Laptop Stand A</t>
         </is>
       </c>
-      <c r="C21" s="194" t="inlineStr">
+      <c r="C21" s="198" t="inlineStr">
         <is>
           <t>⚠️ Question</t>
         </is>
       </c>
-      <c r="D21" s="203" t="inlineStr">
+      <c r="D21" s="207" t="inlineStr">
         <is>
           <t>本週執行</t>
         </is>
       </c>
-      <c r="E21" s="196" t="inlineStr">
+      <c r="E21" s="200" t="inlineStr">
         <is>
           <t>CPC</t>
         </is>
       </c>
-      <c r="F21" s="234" t="inlineStr">
+      <c r="F21" s="238" t="inlineStr">
         <is>
           <t>下載 SP Bulk File → 找出 ACOS ≥85% 的關鍵字 → Bid × 0.8（降 20%）</t>
         </is>
       </c>
-      <c r="G21" s="197" t="n">
+      <c r="G21" s="201" t="n">
         <v>1451.02</v>
       </c>
-      <c r="H21" s="205" t="n"/>
+      <c r="H21" s="209" t="n"/>
     </row>
     <row r="22" ht="28" customHeight="1">
-      <c r="A22" s="233" t="inlineStr"/>
-      <c r="B22" s="235" t="n"/>
-      <c r="C22" s="235" t="n"/>
-      <c r="D22" s="235" t="n"/>
-      <c r="E22" s="196" t="inlineStr">
+      <c r="A22" s="237" t="inlineStr"/>
+      <c r="B22" s="239" t="n"/>
+      <c r="C22" s="239" t="n"/>
+      <c r="D22" s="239" t="n"/>
+      <c r="E22" s="200" t="inlineStr">
         <is>
           <t>Pause KW</t>
         </is>
       </c>
-      <c r="F22" s="234" t="inlineStr">
+      <c r="F22" s="238" t="inlineStr">
         <is>
           <t>TACOS ≥85% 且過去 14 天無轉換的關鍵字 → 狀態改為 Paused</t>
         </is>
       </c>
-      <c r="G22" s="235" t="n"/>
-      <c r="H22" s="235" t="n"/>
+      <c r="G22" s="239" t="n"/>
+      <c r="H22" s="239" t="n"/>
     </row>
     <row r="23" ht="28" customHeight="1">
-      <c r="A23" s="233" t="inlineStr"/>
-      <c r="B23" s="235" t="n"/>
-      <c r="C23" s="235" t="n"/>
-      <c r="D23" s="235" t="n"/>
-      <c r="E23" s="196" t="inlineStr">
+      <c r="A23" s="237" t="inlineStr"/>
+      <c r="B23" s="239" t="n"/>
+      <c r="C23" s="239" t="n"/>
+      <c r="D23" s="239" t="n"/>
+      <c r="E23" s="200" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
       </c>
-      <c r="F23" s="234" t="inlineStr">
+      <c r="F23" s="238" t="inlineStr">
         <is>
           <t>SP 活動預算維持不變，待 TACOS 下降再考慮增加</t>
         </is>
       </c>
-      <c r="G23" s="235" t="n"/>
-      <c r="H23" s="235" t="n"/>
+      <c r="G23" s="239" t="n"/>
+      <c r="H23" s="239" t="n"/>
     </row>
     <row r="24" ht="28" customHeight="1">
-      <c r="A24" s="233" t="inlineStr"/>
-      <c r="B24" s="235" t="n"/>
-      <c r="C24" s="235" t="n"/>
-      <c r="D24" s="235" t="n"/>
-      <c r="E24" s="196" t="inlineStr">
+      <c r="A24" s="237" t="inlineStr"/>
+      <c r="B24" s="239" t="n"/>
+      <c r="C24" s="239" t="n"/>
+      <c r="D24" s="239" t="n"/>
+      <c r="E24" s="200" t="inlineStr">
         <is>
           <t>Review</t>
         </is>
       </c>
-      <c r="F24" s="234" t="inlineStr">
+      <c r="F24" s="238" t="inlineStr">
         <is>
           <t>檢查競品 listing 定價，評估是否需要調整售價提高轉換率</t>
         </is>
       </c>
-      <c r="G24" s="235" t="n"/>
-      <c r="H24" s="235" t="n"/>
+      <c r="G24" s="239" t="n"/>
+      <c r="H24" s="239" t="n"/>
     </row>
     <row r="25" ht="4" customHeight="1">
-      <c r="A25" s="232" t="n"/>
-      <c r="B25" s="232" t="n"/>
-      <c r="C25" s="232" t="n"/>
-      <c r="D25" s="232" t="n"/>
-      <c r="E25" s="232" t="n"/>
-      <c r="F25" s="232" t="n"/>
-      <c r="G25" s="232" t="n"/>
-      <c r="H25" s="232" t="n"/>
+      <c r="A25" s="236" t="n"/>
+      <c r="B25" s="236" t="n"/>
+      <c r="C25" s="236" t="n"/>
+      <c r="D25" s="236" t="n"/>
+      <c r="E25" s="236" t="n"/>
+      <c r="F25" s="236" t="n"/>
+      <c r="G25" s="236" t="n"/>
+      <c r="H25" s="236" t="n"/>
     </row>
     <row r="26" ht="28" customHeight="1">
-      <c r="A26" s="233" t="inlineStr"/>
-      <c r="B26" s="195" t="inlineStr">
+      <c r="A26" s="237" t="inlineStr"/>
+      <c r="B26" s="199" t="inlineStr">
         <is>
           <t>Dryer Rack</t>
         </is>
       </c>
-      <c r="C26" s="194" t="inlineStr">
+      <c r="C26" s="198" t="inlineStr">
         <is>
           <t>⚠️ Question</t>
         </is>
       </c>
-      <c r="D26" s="203" t="inlineStr">
+      <c r="D26" s="207" t="inlineStr">
         <is>
           <t>本週執行</t>
         </is>
       </c>
-      <c r="E26" s="196" t="inlineStr">
+      <c r="E26" s="200" t="inlineStr">
         <is>
           <t>CPC</t>
         </is>
       </c>
-      <c r="F26" s="234" t="inlineStr">
+      <c r="F26" s="238" t="inlineStr">
         <is>
           <t>下載 SP Bulk File → 找出 ACOS ≥85% 的關鍵字 → Bid × 0.8（降 20%）</t>
         </is>
       </c>
-      <c r="G26" s="197" t="n">
+      <c r="G26" s="201" t="n">
         <v>1329.7</v>
       </c>
-      <c r="H26" s="204" t="n">
+      <c r="H26" s="208" t="n">
         <v>0.294</v>
       </c>
     </row>
     <row r="27" ht="28" customHeight="1">
-      <c r="A27" s="233" t="inlineStr"/>
-      <c r="B27" s="235" t="n"/>
-      <c r="C27" s="235" t="n"/>
-      <c r="D27" s="235" t="n"/>
-      <c r="E27" s="196" t="inlineStr">
+      <c r="A27" s="237" t="inlineStr"/>
+      <c r="B27" s="239" t="n"/>
+      <c r="C27" s="239" t="n"/>
+      <c r="D27" s="239" t="n"/>
+      <c r="E27" s="200" t="inlineStr">
         <is>
           <t>Pause KW</t>
         </is>
       </c>
-      <c r="F27" s="234" t="inlineStr">
+      <c r="F27" s="238" t="inlineStr">
         <is>
           <t>TACOS ≥85% 且過去 14 天無轉換的關鍵字 → 狀態改為 Paused</t>
         </is>
       </c>
-      <c r="G27" s="235" t="n"/>
-      <c r="H27" s="235" t="n"/>
+      <c r="G27" s="239" t="n"/>
+      <c r="H27" s="239" t="n"/>
     </row>
     <row r="28" ht="28" customHeight="1">
-      <c r="A28" s="233" t="inlineStr"/>
-      <c r="B28" s="235" t="n"/>
-      <c r="C28" s="235" t="n"/>
-      <c r="D28" s="235" t="n"/>
-      <c r="E28" s="196" t="inlineStr">
+      <c r="A28" s="237" t="inlineStr"/>
+      <c r="B28" s="239" t="n"/>
+      <c r="C28" s="239" t="n"/>
+      <c r="D28" s="239" t="n"/>
+      <c r="E28" s="200" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
       </c>
-      <c r="F28" s="234" t="inlineStr">
+      <c r="F28" s="238" t="inlineStr">
         <is>
           <t>SP 活動預算維持不變，待 TACOS 下降再考慮增加</t>
         </is>
       </c>
-      <c r="G28" s="235" t="n"/>
-      <c r="H28" s="235" t="n"/>
+      <c r="G28" s="239" t="n"/>
+      <c r="H28" s="239" t="n"/>
     </row>
     <row r="29" ht="28" customHeight="1">
-      <c r="A29" s="233" t="inlineStr"/>
-      <c r="B29" s="235" t="n"/>
-      <c r="C29" s="235" t="n"/>
-      <c r="D29" s="235" t="n"/>
-      <c r="E29" s="196" t="inlineStr">
+      <c r="A29" s="237" t="inlineStr"/>
+      <c r="B29" s="239" t="n"/>
+      <c r="C29" s="239" t="n"/>
+      <c r="D29" s="239" t="n"/>
+      <c r="E29" s="200" t="inlineStr">
         <is>
           <t>Review</t>
         </is>
       </c>
-      <c r="F29" s="234" t="inlineStr">
+      <c r="F29" s="238" t="inlineStr">
         <is>
           <t>檢查競品 listing 定價，評估是否需要調整售價提高轉換率</t>
         </is>
       </c>
-      <c r="G29" s="235" t="n"/>
-      <c r="H29" s="235" t="n"/>
+      <c r="G29" s="239" t="n"/>
+      <c r="H29" s="239" t="n"/>
     </row>
     <row r="30" ht="4" customHeight="1">
-      <c r="A30" s="232" t="n"/>
-      <c r="B30" s="232" t="n"/>
-      <c r="C30" s="232" t="n"/>
-      <c r="D30" s="232" t="n"/>
-      <c r="E30" s="232" t="n"/>
-      <c r="F30" s="232" t="n"/>
-      <c r="G30" s="232" t="n"/>
-      <c r="H30" s="232" t="n"/>
+      <c r="A30" s="236" t="n"/>
+      <c r="B30" s="236" t="n"/>
+      <c r="C30" s="236" t="n"/>
+      <c r="D30" s="236" t="n"/>
+      <c r="E30" s="236" t="n"/>
+      <c r="F30" s="236" t="n"/>
+      <c r="G30" s="236" t="n"/>
+      <c r="H30" s="236" t="n"/>
     </row>
     <row r="31" ht="28" customHeight="1">
-      <c r="A31" s="233" t="inlineStr"/>
-      <c r="B31" s="195" t="inlineStr">
+      <c r="A31" s="237" t="inlineStr"/>
+      <c r="B31" s="199" t="inlineStr">
         <is>
           <t>Laptop Stand B</t>
         </is>
       </c>
-      <c r="C31" s="194" t="inlineStr">
+      <c r="C31" s="198" t="inlineStr">
         <is>
           <t>⚠️ Question</t>
         </is>
       </c>
-      <c r="D31" s="203" t="inlineStr">
+      <c r="D31" s="207" t="inlineStr">
         <is>
           <t>本週執行</t>
         </is>
       </c>
-      <c r="E31" s="196" t="inlineStr">
+      <c r="E31" s="200" t="inlineStr">
         <is>
           <t>CPC</t>
         </is>
       </c>
-      <c r="F31" s="234" t="inlineStr">
+      <c r="F31" s="238" t="inlineStr">
         <is>
           <t>下載 SP Bulk File → 找出 ACOS ≥85% 的關鍵字 → Bid × 0.8（降 20%）</t>
         </is>
       </c>
-      <c r="G31" s="197" t="n">
+      <c r="G31" s="201" t="n">
         <v>1232.16</v>
       </c>
-      <c r="H31" s="205" t="n"/>
+      <c r="H31" s="209" t="n"/>
     </row>
     <row r="32" ht="28" customHeight="1">
-      <c r="A32" s="233" t="inlineStr"/>
-      <c r="B32" s="235" t="n"/>
-      <c r="C32" s="235" t="n"/>
-      <c r="D32" s="235" t="n"/>
-      <c r="E32" s="196" t="inlineStr">
+      <c r="A32" s="237" t="inlineStr"/>
+      <c r="B32" s="239" t="n"/>
+      <c r="C32" s="239" t="n"/>
+      <c r="D32" s="239" t="n"/>
+      <c r="E32" s="200" t="inlineStr">
         <is>
           <t>Pause KW</t>
         </is>
       </c>
-      <c r="F32" s="234" t="inlineStr">
+      <c r="F32" s="238" t="inlineStr">
         <is>
           <t>TACOS ≥85% 且過去 14 天無轉換的關鍵字 → 狀態改為 Paused</t>
         </is>
       </c>
-      <c r="G32" s="235" t="n"/>
-      <c r="H32" s="235" t="n"/>
+      <c r="G32" s="239" t="n"/>
+      <c r="H32" s="239" t="n"/>
     </row>
     <row r="33" ht="28" customHeight="1">
-      <c r="A33" s="233" t="inlineStr"/>
-      <c r="B33" s="235" t="n"/>
-      <c r="C33" s="235" t="n"/>
-      <c r="D33" s="235" t="n"/>
-      <c r="E33" s="196" t="inlineStr">
+      <c r="A33" s="237" t="inlineStr"/>
+      <c r="B33" s="239" t="n"/>
+      <c r="C33" s="239" t="n"/>
+      <c r="D33" s="239" t="n"/>
+      <c r="E33" s="200" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
       </c>
-      <c r="F33" s="234" t="inlineStr">
+      <c r="F33" s="238" t="inlineStr">
         <is>
           <t>SP 活動預算維持不變，待 TACOS 下降再考慮增加</t>
         </is>
       </c>
-      <c r="G33" s="235" t="n"/>
-      <c r="H33" s="235" t="n"/>
+      <c r="G33" s="239" t="n"/>
+      <c r="H33" s="239" t="n"/>
     </row>
     <row r="34" ht="28" customHeight="1">
-      <c r="A34" s="233" t="inlineStr"/>
-      <c r="B34" s="235" t="n"/>
-      <c r="C34" s="235" t="n"/>
-      <c r="D34" s="235" t="n"/>
-      <c r="E34" s="196" t="inlineStr">
+      <c r="A34" s="237" t="inlineStr"/>
+      <c r="B34" s="239" t="n"/>
+      <c r="C34" s="239" t="n"/>
+      <c r="D34" s="239" t="n"/>
+      <c r="E34" s="200" t="inlineStr">
         <is>
           <t>Review</t>
         </is>
       </c>
-      <c r="F34" s="234" t="inlineStr">
+      <c r="F34" s="238" t="inlineStr">
         <is>
           <t>檢查競品 listing 定價，評估是否需要調整售價提高轉換率</t>
         </is>
       </c>
-      <c r="G34" s="235" t="n"/>
-      <c r="H34" s="235" t="n"/>
+      <c r="G34" s="239" t="n"/>
+      <c r="H34" s="239" t="n"/>
     </row>
     <row r="35" ht="4" customHeight="1">
-      <c r="A35" s="232" t="n"/>
-      <c r="B35" s="232" t="n"/>
-      <c r="C35" s="232" t="n"/>
-      <c r="D35" s="232" t="n"/>
-      <c r="E35" s="232" t="n"/>
-      <c r="F35" s="232" t="n"/>
-      <c r="G35" s="232" t="n"/>
-      <c r="H35" s="232" t="n"/>
+      <c r="A35" s="236" t="n"/>
+      <c r="B35" s="236" t="n"/>
+      <c r="C35" s="236" t="n"/>
+      <c r="D35" s="236" t="n"/>
+      <c r="E35" s="236" t="n"/>
+      <c r="F35" s="236" t="n"/>
+      <c r="G35" s="236" t="n"/>
+      <c r="H35" s="236" t="n"/>
     </row>
     <row r="36" ht="28" customHeight="1">
-      <c r="A36" s="233" t="inlineStr"/>
-      <c r="B36" s="195" t="inlineStr">
+      <c r="A36" s="237" t="inlineStr"/>
+      <c r="B36" s="199" t="inlineStr">
         <is>
           <t>Bathroom Storage</t>
         </is>
       </c>
-      <c r="C36" s="194" t="inlineStr">
+      <c r="C36" s="198" t="inlineStr">
         <is>
           <t>⚠️ Question</t>
         </is>
       </c>
-      <c r="D36" s="203" t="inlineStr">
+      <c r="D36" s="207" t="inlineStr">
         <is>
           <t>本週執行</t>
         </is>
       </c>
-      <c r="E36" s="196" t="inlineStr">
+      <c r="E36" s="200" t="inlineStr">
         <is>
           <t>CPC</t>
         </is>
       </c>
-      <c r="F36" s="234" t="inlineStr">
+      <c r="F36" s="238" t="inlineStr">
         <is>
           <t>下載 SP Bulk File → 找出 ACOS ≥85% 的關鍵字 → Bid × 0.8（降 20%）</t>
         </is>
       </c>
-      <c r="G36" s="197" t="n">
+      <c r="G36" s="201" t="n">
         <v>901.4299999999999</v>
       </c>
-      <c r="H36" s="205" t="n"/>
+      <c r="H36" s="209" t="n"/>
     </row>
     <row r="37" ht="28" customHeight="1">
-      <c r="A37" s="233" t="inlineStr"/>
-      <c r="B37" s="235" t="n"/>
-      <c r="C37" s="235" t="n"/>
-      <c r="D37" s="235" t="n"/>
-      <c r="E37" s="196" t="inlineStr">
+      <c r="A37" s="237" t="inlineStr"/>
+      <c r="B37" s="239" t="n"/>
+      <c r="C37" s="239" t="n"/>
+      <c r="D37" s="239" t="n"/>
+      <c r="E37" s="200" t="inlineStr">
         <is>
           <t>Pause KW</t>
         </is>
       </c>
-      <c r="F37" s="234" t="inlineStr">
+      <c r="F37" s="238" t="inlineStr">
         <is>
           <t>TACOS ≥85% 且過去 14 天無轉換的關鍵字 → 狀態改為 Paused</t>
         </is>
       </c>
-      <c r="G37" s="235" t="n"/>
-      <c r="H37" s="235" t="n"/>
+      <c r="G37" s="239" t="n"/>
+      <c r="H37" s="239" t="n"/>
     </row>
     <row r="38" ht="28" customHeight="1">
-      <c r="A38" s="233" t="inlineStr"/>
-      <c r="B38" s="235" t="n"/>
-      <c r="C38" s="235" t="n"/>
-      <c r="D38" s="235" t="n"/>
-      <c r="E38" s="196" t="inlineStr">
+      <c r="A38" s="237" t="inlineStr"/>
+      <c r="B38" s="239" t="n"/>
+      <c r="C38" s="239" t="n"/>
+      <c r="D38" s="239" t="n"/>
+      <c r="E38" s="200" t="inlineStr">
         <is>
           <t>Budget</t>
         </is>
       </c>
-      <c r="F38" s="234" t="inlineStr">
+      <c r="F38" s="238" t="inlineStr">
         <is>
           <t>SP 活動預算維持不變，待 TACOS 下降再考慮增加</t>
         </is>
       </c>
-      <c r="G38" s="235" t="n"/>
-      <c r="H38" s="235" t="n"/>
+      <c r="G38" s="239" t="n"/>
+      <c r="H38" s="239" t="n"/>
     </row>
     <row r="39" ht="28" customHeight="1">
-      <c r="A39" s="233" t="inlineStr"/>
-      <c r="B39" s="235" t="n"/>
-      <c r="C39" s="235" t="n"/>
-      <c r="D39" s="235" t="n"/>
-      <c r="E39" s="196" t="inlineStr">
+      <c r="A39" s="237" t="inlineStr"/>
+      <c r="B39" s="239" t="n"/>
+      <c r="C39" s="239" t="n"/>
+      <c r="D39" s="239" t="n"/>
+      <c r="E39" s="200" t="inlineStr">
         <is>
           <t>Review</t>
         </is>
       </c>
-      <c r="F39" s="234" t="inlineStr">
+      <c r="F39" s="238" t="inlineStr">
         <is>
           <t>檢查競品 listing 定價，評估是否需要調整售價提高轉換率</t>
         </is>
       </c>
-      <c r="G39" s="235" t="n"/>
-      <c r="H39" s="235" t="n"/>
+      <c r="G39" s="239" t="n"/>
+      <c r="H39" s="239" t="n"/>
     </row>
     <row r="40" ht="4" customHeight="1">
-      <c r="A40" s="232" t="n"/>
-      <c r="B40" s="232" t="n"/>
-      <c r="C40" s="232" t="n"/>
-      <c r="D40" s="232" t="n"/>
-      <c r="E40" s="232" t="n"/>
-      <c r="F40" s="232" t="n"/>
-      <c r="G40" s="232" t="n"/>
-      <c r="H40" s="232" t="n"/>
+      <c r="A40" s="236" t="n"/>
+      <c r="B40" s="236" t="n"/>
+      <c r="C40" s="236" t="n"/>
+      <c r="D40" s="236" t="n"/>
+      <c r="E40" s="236" t="n"/>
+      <c r="F40" s="236" t="n"/>
+      <c r="G40" s="236" t="n"/>
+      <c r="H40" s="236" t="n"/>
     </row>
     <row r="41" ht="15" customHeight="1">
-      <c r="A41" s="206" t="inlineStr">
+      <c r="A41" s="210" t="inlineStr">
         <is>
           <t xml:space="preserve">  🔴 Cut  —  低銷售 · 高 TACOS</t>
         </is>
       </c>
     </row>
     <row r="42" ht="28" customHeight="1">
-      <c r="A42" s="236" t="inlineStr"/>
-      <c r="B42" s="208" t="inlineStr">
+      <c r="A42" s="240" t="inlineStr"/>
+      <c r="B42" s="212" t="inlineStr">
         <is>
           <t>Double Rail Rack</t>
         </is>
       </c>
-      <c r="C42" s="207" t="inlineStr">
+      <c r="C42" s="211" t="inlineStr">
         <is>
           <t>🔴 Cut</t>
         </is>
       </c>
-      <c r="D42" s="216" t="inlineStr">
+      <c r="D42" s="220" t="inlineStr">
         <is>
           <t>本週執行</t>
         </is>
       </c>
-      <c r="E42" s="209" t="inlineStr">
+      <c r="E42" s="213" t="inlineStr">
         <is>
           <t>Price</t>
         </is>
       </c>
-      <c r="F42" s="237" t="inlineStr">
+      <c r="F42" s="241" t="inlineStr">
         <is>
           <t>在 Seller Central 將售價下調 $0.50，觀察轉換率變化</t>
         </is>
       </c>
-      <c r="G42" s="210" t="n">
+      <c r="G42" s="214" t="n">
         <v>887.37</v>
       </c>
-      <c r="H42" s="211" t="n"/>
+      <c r="H42" s="215" t="n"/>
     </row>
     <row r="43" ht="28" customHeight="1">
-      <c r="A43" s="236" t="inlineStr"/>
-      <c r="B43" s="238" t="n"/>
-      <c r="C43" s="238" t="n"/>
-      <c r="D43" s="238" t="n"/>
-      <c r="E43" s="209" t="inlineStr">
+      <c r="A43" s="240" t="inlineStr"/>
+      <c r="B43" s="242" t="n"/>
+      <c r="C43" s="242" t="n"/>
+      <c r="D43" s="242" t="n"/>
+      <c r="E43" s="213" t="inlineStr">
         <is>
           <t>Coupon</t>
         </is>
       </c>
-      <c r="F43" s="237" t="inlineStr">
+      <c r="F43" s="241" t="inlineStr">
         <is>
           <t>建立 Coupon 折扣（建議 5–10%）→ 提升搜尋結果曝光</t>
         </is>
       </c>
-      <c r="G43" s="238" t="n"/>
-      <c r="H43" s="238" t="n"/>
+      <c r="G43" s="242" t="n"/>
+      <c r="H43" s="242" t="n"/>
     </row>
     <row r="44" ht="28" customHeight="1">
-      <c r="A44" s="236" t="inlineStr"/>
-      <c r="B44" s="238" t="n"/>
-      <c r="C44" s="238" t="n"/>
-      <c r="D44" s="238" t="n"/>
-      <c r="E44" s="209" t="inlineStr">
+      <c r="A44" s="240" t="inlineStr"/>
+      <c r="B44" s="242" t="n"/>
+      <c r="C44" s="242" t="n"/>
+      <c r="D44" s="242" t="n"/>
+      <c r="E44" s="213" t="inlineStr">
         <is>
           <t>Deal</t>
         </is>
       </c>
-      <c r="F44" s="237" t="inlineStr">
+      <c r="F44" s="241" t="inlineStr">
         <is>
           <t>申請 Prime Exclusive Discount 或 Lightning Deal（需提前 2 週申請）</t>
         </is>
       </c>
-      <c r="G44" s="238" t="n"/>
-      <c r="H44" s="238" t="n"/>
+      <c r="G44" s="242" t="n"/>
+      <c r="H44" s="242" t="n"/>
     </row>
     <row r="45" ht="28" customHeight="1">
-      <c r="A45" s="236" t="inlineStr"/>
-      <c r="B45" s="238" t="n"/>
-      <c r="C45" s="238" t="n"/>
-      <c r="D45" s="238" t="n"/>
-      <c r="E45" s="209" t="inlineStr">
+      <c r="A45" s="240" t="inlineStr"/>
+      <c r="B45" s="242" t="n"/>
+      <c r="C45" s="242" t="n"/>
+      <c r="D45" s="242" t="n"/>
+      <c r="E45" s="213" t="inlineStr">
         <is>
           <t>SP Bid</t>
         </is>
       </c>
-      <c r="F45" s="237" t="inlineStr">
+      <c r="F45" s="241" t="inlineStr">
         <is>
           <t>下載 SP Bulk File → 全部 Keyword Bid 降至 $2.00 上限</t>
         </is>
       </c>
-      <c r="G45" s="238" t="n"/>
-      <c r="H45" s="238" t="n"/>
+      <c r="G45" s="242" t="n"/>
+      <c r="H45" s="242" t="n"/>
     </row>
     <row r="46" ht="4" customHeight="1">
-      <c r="A46" s="232" t="n"/>
-      <c r="B46" s="232" t="n"/>
-      <c r="C46" s="232" t="n"/>
-      <c r="D46" s="232" t="n"/>
-      <c r="E46" s="232" t="n"/>
-      <c r="F46" s="232" t="n"/>
-      <c r="G46" s="232" t="n"/>
-      <c r="H46" s="232" t="n"/>
+      <c r="A46" s="236" t="n"/>
+      <c r="B46" s="236" t="n"/>
+      <c r="C46" s="236" t="n"/>
+      <c r="D46" s="236" t="n"/>
+      <c r="E46" s="236" t="n"/>
+      <c r="F46" s="236" t="n"/>
+      <c r="G46" s="236" t="n"/>
+      <c r="H46" s="236" t="n"/>
     </row>
     <row r="47" ht="28" customHeight="1">
-      <c r="A47" s="236" t="inlineStr"/>
-      <c r="B47" s="208" t="inlineStr">
+      <c r="A47" s="240" t="inlineStr"/>
+      <c r="B47" s="212" t="inlineStr">
         <is>
           <t>3-Tier Cart</t>
         </is>
       </c>
-      <c r="C47" s="207" t="inlineStr">
+      <c r="C47" s="211" t="inlineStr">
         <is>
           <t>🔴 Cut</t>
         </is>
       </c>
-      <c r="D47" s="216" t="inlineStr">
+      <c r="D47" s="220" t="inlineStr">
         <is>
           <t>本週執行</t>
         </is>
       </c>
-      <c r="E47" s="209" t="inlineStr">
+      <c r="E47" s="213" t="inlineStr">
         <is>
           <t>Price</t>
         </is>
       </c>
-      <c r="F47" s="237" t="inlineStr">
+      <c r="F47" s="241" t="inlineStr">
         <is>
           <t>在 Seller Central 將售價下調 $0.50，觀察轉換率變化</t>
         </is>
       </c>
-      <c r="G47" s="210" t="n">
+      <c r="G47" s="214" t="n">
         <v>804.89</v>
       </c>
-      <c r="H47" s="217" t="n">
+      <c r="H47" s="221" t="n">
         <v>0.3</v>
       </c>
     </row>
     <row r="48" ht="28" customHeight="1">
-      <c r="A48" s="236" t="inlineStr"/>
-      <c r="B48" s="238" t="n"/>
-      <c r="C48" s="238" t="n"/>
-      <c r="D48" s="238" t="n"/>
-      <c r="E48" s="209" t="inlineStr">
+      <c r="A48" s="240" t="inlineStr"/>
+      <c r="B48" s="242" t="n"/>
+      <c r="C48" s="242" t="n"/>
+      <c r="D48" s="242" t="n"/>
+      <c r="E48" s="213" t="inlineStr">
         <is>
           <t>Coupon</t>
         </is>
       </c>
-      <c r="F48" s="237" t="inlineStr">
+      <c r="F48" s="241" t="inlineStr">
         <is>
           <t>建立 Coupon 折扣（建議 5–10%）→ 提升搜尋結果曝光</t>
         </is>
       </c>
-      <c r="G48" s="238" t="n"/>
-      <c r="H48" s="238" t="n"/>
+      <c r="G48" s="242" t="n"/>
+      <c r="H48" s="242" t="n"/>
     </row>
     <row r="49" ht="28" customHeight="1">
-      <c r="A49" s="236" t="inlineStr"/>
-      <c r="B49" s="238" t="n"/>
-      <c r="C49" s="238" t="n"/>
-      <c r="D49" s="238" t="n"/>
-      <c r="E49" s="209" t="inlineStr">
+      <c r="A49" s="240" t="inlineStr"/>
+      <c r="B49" s="242" t="n"/>
+      <c r="C49" s="242" t="n"/>
+      <c r="D49" s="242" t="n"/>
+      <c r="E49" s="213" t="inlineStr">
         <is>
           <t>Deal</t>
         </is>
       </c>
-      <c r="F49" s="237" t="inlineStr">
+      <c r="F49" s="241" t="inlineStr">
         <is>
           <t>申請 Prime Exclusive Discount 或 Lightning Deal（需提前 2 週申請）</t>
         </is>
       </c>
-      <c r="G49" s="238" t="n"/>
-      <c r="H49" s="238" t="n"/>
+      <c r="G49" s="242" t="n"/>
+      <c r="H49" s="242" t="n"/>
     </row>
     <row r="50" ht="28" customHeight="1">
-      <c r="A50" s="236" t="inlineStr"/>
-      <c r="B50" s="238" t="n"/>
-      <c r="C50" s="238" t="n"/>
-      <c r="D50" s="238" t="n"/>
-      <c r="E50" s="209" t="inlineStr">
+      <c r="A50" s="240" t="inlineStr"/>
+      <c r="B50" s="242" t="n"/>
+      <c r="C50" s="242" t="n"/>
+      <c r="D50" s="242" t="n"/>
+      <c r="E50" s="213" t="inlineStr">
         <is>
           <t>SP Bid</t>
         </is>
       </c>
-      <c r="F50" s="237" t="inlineStr">
+      <c r="F50" s="241" t="inlineStr">
         <is>
           <t>下載 SP Bulk File → 全部 Keyword Bid 降至 $2.00 上限</t>
         </is>
       </c>
-      <c r="G50" s="238" t="n"/>
-      <c r="H50" s="238" t="n"/>
+      <c r="G50" s="242" t="n"/>
+      <c r="H50" s="242" t="n"/>
     </row>
     <row r="51" ht="4" customHeight="1">
-      <c r="A51" s="232" t="n"/>
-      <c r="B51" s="232" t="n"/>
-      <c r="C51" s="232" t="n"/>
-      <c r="D51" s="232" t="n"/>
-      <c r="E51" s="232" t="n"/>
-      <c r="F51" s="232" t="n"/>
-      <c r="G51" s="232" t="n"/>
-      <c r="H51" s="232" t="n"/>
+      <c r="A51" s="236" t="n"/>
+      <c r="B51" s="236" t="n"/>
+      <c r="C51" s="236" t="n"/>
+      <c r="D51" s="236" t="n"/>
+      <c r="E51" s="236" t="n"/>
+      <c r="F51" s="236" t="n"/>
+      <c r="G51" s="236" t="n"/>
+      <c r="H51" s="236" t="n"/>
     </row>
     <row r="52" ht="28" customHeight="1">
-      <c r="A52" s="236" t="inlineStr"/>
-      <c r="B52" s="208" t="inlineStr">
+      <c r="A52" s="240" t="inlineStr"/>
+      <c r="B52" s="212" t="inlineStr">
         <is>
           <t>Laptop Stand C</t>
         </is>
       </c>
-      <c r="C52" s="207" t="inlineStr">
+      <c r="C52" s="211" t="inlineStr">
         <is>
           <t>🔴 Cut</t>
         </is>
       </c>
-      <c r="D52" s="216" t="inlineStr">
+      <c r="D52" s="220" t="inlineStr">
         <is>
           <t>本週執行</t>
         </is>
       </c>
-      <c r="E52" s="209" t="inlineStr">
+      <c r="E52" s="213" t="inlineStr">
         <is>
           <t>Price</t>
         </is>
       </c>
-      <c r="F52" s="237" t="inlineStr">
+      <c r="F52" s="241" t="inlineStr">
         <is>
           <t>在 Seller Central 將售價下調 $0.50，觀察轉換率變化</t>
         </is>
       </c>
-      <c r="G52" s="210" t="n">
+      <c r="G52" s="214" t="n">
         <v>670.66</v>
       </c>
-      <c r="H52" s="211" t="n"/>
+      <c r="H52" s="215" t="n"/>
     </row>
     <row r="53" ht="28" customHeight="1">
-      <c r="A53" s="236" t="inlineStr"/>
-      <c r="B53" s="238" t="n"/>
-      <c r="C53" s="238" t="n"/>
-      <c r="D53" s="238" t="n"/>
-      <c r="E53" s="209" t="inlineStr">
+      <c r="A53" s="240" t="inlineStr"/>
+      <c r="B53" s="242" t="n"/>
+      <c r="C53" s="242" t="n"/>
+      <c r="D53" s="242" t="n"/>
+      <c r="E53" s="213" t="inlineStr">
         <is>
           <t>Coupon</t>
         </is>
       </c>
-      <c r="F53" s="237" t="inlineStr">
+      <c r="F53" s="241" t="inlineStr">
         <is>
           <t>建立 Coupon 折扣（建議 5–10%）→ 提升搜尋結果曝光</t>
         </is>
       </c>
-      <c r="G53" s="238" t="n"/>
-      <c r="H53" s="238" t="n"/>
+      <c r="G53" s="242" t="n"/>
+      <c r="H53" s="242" t="n"/>
     </row>
     <row r="54" ht="28" customHeight="1">
-      <c r="A54" s="236" t="inlineStr"/>
-      <c r="B54" s="238" t="n"/>
-      <c r="C54" s="238" t="n"/>
-      <c r="D54" s="238" t="n"/>
-      <c r="E54" s="209" t="inlineStr">
+      <c r="A54" s="240" t="inlineStr"/>
+      <c r="B54" s="242" t="n"/>
+      <c r="C54" s="242" t="n"/>
+      <c r="D54" s="242" t="n"/>
+      <c r="E54" s="213" t="inlineStr">
         <is>
           <t>Deal</t>
         </is>
       </c>
-      <c r="F54" s="237" t="inlineStr">
+      <c r="F54" s="241" t="inlineStr">
         <is>
           <t>申請 Prime Exclusive Discount 或 Lightning Deal（需提前 2 週申請）</t>
         </is>
       </c>
-      <c r="G54" s="238" t="n"/>
-      <c r="H54" s="238" t="n"/>
+      <c r="G54" s="242" t="n"/>
+      <c r="H54" s="242" t="n"/>
     </row>
     <row r="55" ht="28" customHeight="1">
-      <c r="A55" s="236" t="inlineStr"/>
-      <c r="B55" s="238" t="n"/>
-      <c r="C55" s="238" t="n"/>
-      <c r="D55" s="238" t="n"/>
-      <c r="E55" s="209" t="inlineStr">
+      <c r="A55" s="240" t="inlineStr"/>
+      <c r="B55" s="242" t="n"/>
+      <c r="C55" s="242" t="n"/>
+      <c r="D55" s="242" t="n"/>
+      <c r="E55" s="213" t="inlineStr">
         <is>
           <t>SP Bid</t>
         </is>
       </c>
-      <c r="F55" s="237" t="inlineStr">
+      <c r="F55" s="241" t="inlineStr">
         <is>
           <t>下載 SP Bulk File → 全部 Keyword Bid 降至 $2.00 上限</t>
         </is>
       </c>
-      <c r="G55" s="238" t="n"/>
-      <c r="H55" s="238" t="n"/>
+      <c r="G55" s="242" t="n"/>
+      <c r="H55" s="242" t="n"/>
     </row>
     <row r="56" ht="4" customHeight="1">
-      <c r="A56" s="232" t="n"/>
-      <c r="B56" s="232" t="n"/>
-      <c r="C56" s="232" t="n"/>
-      <c r="D56" s="232" t="n"/>
-      <c r="E56" s="232" t="n"/>
-      <c r="F56" s="232" t="n"/>
-      <c r="G56" s="232" t="n"/>
-      <c r="H56" s="232" t="n"/>
+      <c r="A56" s="236" t="n"/>
+      <c r="B56" s="236" t="n"/>
+      <c r="C56" s="236" t="n"/>
+      <c r="D56" s="236" t="n"/>
+      <c r="E56" s="236" t="n"/>
+      <c r="F56" s="236" t="n"/>
+      <c r="G56" s="236" t="n"/>
+      <c r="H56" s="236" t="n"/>
     </row>
     <row r="57" ht="28" customHeight="1">
-      <c r="A57" s="236" t="inlineStr"/>
-      <c r="B57" s="208" t="inlineStr">
+      <c r="A57" s="240" t="inlineStr"/>
+      <c r="B57" s="212" t="inlineStr">
         <is>
           <t>Shoe Rack</t>
         </is>
       </c>
-      <c r="C57" s="207" t="inlineStr">
+      <c r="C57" s="211" t="inlineStr">
         <is>
           <t>🔴 Cut</t>
         </is>
       </c>
-      <c r="D57" s="216" t="inlineStr">
+      <c r="D57" s="220" t="inlineStr">
         <is>
           <t>本週執行</t>
         </is>
       </c>
-      <c r="E57" s="209" t="inlineStr">
+      <c r="E57" s="213" t="inlineStr">
         <is>
           <t>Price</t>
         </is>
       </c>
-      <c r="F57" s="237" t="inlineStr">
+      <c r="F57" s="241" t="inlineStr">
         <is>
           <t>在 Seller Central 將售價下調 $0.50，觀察轉換率變化</t>
         </is>
       </c>
-      <c r="G57" s="210" t="n">
+      <c r="G57" s="214" t="n">
         <v>616.51</v>
       </c>
-      <c r="H57" s="211" t="n"/>
+      <c r="H57" s="215" t="n"/>
     </row>
     <row r="58" ht="28" customHeight="1">
-      <c r="A58" s="236" t="inlineStr"/>
-      <c r="B58" s="238" t="n"/>
-      <c r="C58" s="238" t="n"/>
-      <c r="D58" s="238" t="n"/>
-      <c r="E58" s="209" t="inlineStr">
+      <c r="A58" s="240" t="inlineStr"/>
+      <c r="B58" s="242" t="n"/>
+      <c r="C58" s="242" t="n"/>
+      <c r="D58" s="242" t="n"/>
+      <c r="E58" s="213" t="inlineStr">
         <is>
           <t>Coupon</t>
         </is>
       </c>
-      <c r="F58" s="237" t="inlineStr">
+      <c r="F58" s="241" t="inlineStr">
         <is>
           <t>建立 Coupon 折扣（建議 5–10%）→ 提升搜尋結果曝光</t>
         </is>
       </c>
-      <c r="G58" s="238" t="n"/>
-      <c r="H58" s="238" t="n"/>
+      <c r="G58" s="242" t="n"/>
+      <c r="H58" s="242" t="n"/>
     </row>
     <row r="59" ht="28" customHeight="1">
-      <c r="A59" s="236" t="inlineStr"/>
-      <c r="B59" s="238" t="n"/>
-      <c r="C59" s="238" t="n"/>
-      <c r="D59" s="238" t="n"/>
-      <c r="E59" s="209" t="inlineStr">
+      <c r="A59" s="240" t="inlineStr"/>
+      <c r="B59" s="242" t="n"/>
+      <c r="C59" s="242" t="n"/>
+      <c r="D59" s="242" t="n"/>
+      <c r="E59" s="213" t="inlineStr">
         <is>
           <t>Deal</t>
         </is>
       </c>
-      <c r="F59" s="237" t="inlineStr">
+      <c r="F59" s="241" t="inlineStr">
         <is>
           <t>申請 Prime Exclusive Discount 或 Lightning Deal（需提前 2 週申請）</t>
         </is>
       </c>
-      <c r="G59" s="238" t="n"/>
-      <c r="H59" s="238" t="n"/>
+      <c r="G59" s="242" t="n"/>
+      <c r="H59" s="242" t="n"/>
     </row>
     <row r="60" ht="28" customHeight="1">
-      <c r="A60" s="236" t="inlineStr"/>
-      <c r="B60" s="238" t="n"/>
-      <c r="C60" s="238" t="n"/>
-      <c r="D60" s="238" t="n"/>
-      <c r="E60" s="209" t="inlineStr">
+      <c r="A60" s="240" t="inlineStr"/>
+      <c r="B60" s="242" t="n"/>
+      <c r="C60" s="242" t="n"/>
+      <c r="D60" s="242" t="n"/>
+      <c r="E60" s="213" t="inlineStr">
         <is>
           <t>SP Bid</t>
         </is>
       </c>
-      <c r="F60" s="237" t="inlineStr">
+      <c r="F60" s="241" t="inlineStr">
         <is>
           <t>下載 SP Bulk File → 全部 Keyword Bid 降至 $2.00 上限</t>
         </is>
       </c>
-      <c r="G60" s="238" t="n"/>
-      <c r="H60" s="238" t="n"/>
+      <c r="G60" s="242" t="n"/>
+      <c r="H60" s="242" t="n"/>
     </row>
     <row r="61" ht="4" customHeight="1">
-      <c r="A61" s="232" t="n"/>
-      <c r="B61" s="232" t="n"/>
-      <c r="C61" s="232" t="n"/>
-      <c r="D61" s="232" t="n"/>
-      <c r="E61" s="232" t="n"/>
-      <c r="F61" s="232" t="n"/>
-      <c r="G61" s="232" t="n"/>
-      <c r="H61" s="232" t="n"/>
+      <c r="A61" s="236" t="n"/>
+      <c r="B61" s="236" t="n"/>
+      <c r="C61" s="236" t="n"/>
+      <c r="D61" s="236" t="n"/>
+      <c r="E61" s="236" t="n"/>
+      <c r="F61" s="236" t="n"/>
+      <c r="G61" s="236" t="n"/>
+      <c r="H61" s="236" t="n"/>
     </row>
     <row r="62" ht="28" customHeight="1">
-      <c r="A62" s="236" t="inlineStr"/>
-      <c r="B62" s="208" t="inlineStr">
+      <c r="A62" s="240" t="inlineStr"/>
+      <c r="B62" s="212" t="inlineStr">
         <is>
           <t>Broom Holder</t>
         </is>
       </c>
-      <c r="C62" s="207" t="inlineStr">
+      <c r="C62" s="211" t="inlineStr">
         <is>
           <t>🔴 Cut</t>
         </is>
       </c>
-      <c r="D62" s="216" t="inlineStr">
+      <c r="D62" s="220" t="inlineStr">
         <is>
           <t>本週執行</t>
         </is>
       </c>
-      <c r="E62" s="209" t="inlineStr">
+      <c r="E62" s="213" t="inlineStr">
         <is>
           <t>Price</t>
         </is>
       </c>
-      <c r="F62" s="237" t="inlineStr">
+      <c r="F62" s="241" t="inlineStr">
         <is>
           <t>在 Seller Central 將售價下調 $0.50，觀察轉換率變化</t>
         </is>
       </c>
-      <c r="G62" s="210" t="n">
+      <c r="G62" s="214" t="n">
         <v>276.37</v>
       </c>
-      <c r="H62" s="217" t="n">
+      <c r="H62" s="221" t="n">
         <v>0.185</v>
       </c>
     </row>
     <row r="63" ht="28" customHeight="1">
-      <c r="A63" s="236" t="inlineStr"/>
-      <c r="B63" s="238" t="n"/>
-      <c r="C63" s="238" t="n"/>
-      <c r="D63" s="238" t="n"/>
-      <c r="E63" s="209" t="inlineStr">
+      <c r="A63" s="240" t="inlineStr"/>
+      <c r="B63" s="242" t="n"/>
+      <c r="C63" s="242" t="n"/>
+      <c r="D63" s="242" t="n"/>
+      <c r="E63" s="213" t="inlineStr">
         <is>
           <t>Coupon</t>
         </is>
       </c>
-      <c r="F63" s="237" t="inlineStr">
+      <c r="F63" s="241" t="inlineStr">
         <is>
           <t>建立 Coupon 折扣（建議 5–10%）→ 提升搜尋結果曝光</t>
         </is>
       </c>
-      <c r="G63" s="238" t="n"/>
-      <c r="H63" s="238" t="n"/>
+      <c r="G63" s="242" t="n"/>
+      <c r="H63" s="242" t="n"/>
     </row>
     <row r="64" ht="28" customHeight="1">
-      <c r="A64" s="236" t="inlineStr"/>
-      <c r="B64" s="238" t="n"/>
-      <c r="C64" s="238" t="n"/>
-      <c r="D64" s="238" t="n"/>
-      <c r="E64" s="209" t="inlineStr">
+      <c r="A64" s="240" t="inlineStr"/>
+      <c r="B64" s="242" t="n"/>
+      <c r="C64" s="242" t="n"/>
+      <c r="D64" s="242" t="n"/>
+      <c r="E64" s="213" t="inlineStr">
         <is>
           <t>Deal</t>
         </is>
       </c>
-      <c r="F64" s="237" t="inlineStr">
+      <c r="F64" s="241" t="inlineStr">
         <is>
           <t>申請 Prime Exclusive Discount 或 Lightning Deal（需提前 2 週申請）</t>
         </is>
       </c>
-      <c r="G64" s="238" t="n"/>
-      <c r="H64" s="238" t="n"/>
+      <c r="G64" s="242" t="n"/>
+      <c r="H64" s="242" t="n"/>
     </row>
     <row r="65" ht="28" customHeight="1">
-      <c r="A65" s="236" t="inlineStr"/>
-      <c r="B65" s="238" t="n"/>
-      <c r="C65" s="238" t="n"/>
-      <c r="D65" s="238" t="n"/>
-      <c r="E65" s="209" t="inlineStr">
+      <c r="A65" s="240" t="inlineStr"/>
+      <c r="B65" s="242" t="n"/>
+      <c r="C65" s="242" t="n"/>
+      <c r="D65" s="242" t="n"/>
+      <c r="E65" s="213" t="inlineStr">
         <is>
           <t>SP Bid</t>
         </is>
       </c>
-      <c r="F65" s="237" t="inlineStr">
+      <c r="F65" s="241" t="inlineStr">
         <is>
           <t>下載 SP Bulk File → 全部 Keyword Bid 降至 $2.00 上限</t>
         </is>
       </c>
-      <c r="G65" s="238" t="n"/>
-      <c r="H65" s="238" t="n"/>
+      <c r="G65" s="242" t="n"/>
+      <c r="H65" s="242" t="n"/>
     </row>
     <row r="66" ht="4" customHeight="1">
-      <c r="A66" s="232" t="n"/>
-      <c r="B66" s="232" t="n"/>
-      <c r="C66" s="232" t="n"/>
-      <c r="D66" s="232" t="n"/>
-      <c r="E66" s="232" t="n"/>
-      <c r="F66" s="232" t="n"/>
-      <c r="G66" s="232" t="n"/>
-      <c r="H66" s="232" t="n"/>
+      <c r="A66" s="236" t="n"/>
+      <c r="B66" s="236" t="n"/>
+      <c r="C66" s="236" t="n"/>
+      <c r="D66" s="236" t="n"/>
+      <c r="E66" s="236" t="n"/>
+      <c r="F66" s="236" t="n"/>
+      <c r="G66" s="236" t="n"/>
+      <c r="H66" s="236" t="n"/>
     </row>
     <row r="67" ht="28" customHeight="1">
-      <c r="A67" s="236" t="inlineStr"/>
-      <c r="B67" s="208" t="inlineStr">
+      <c r="A67" s="240" t="inlineStr"/>
+      <c r="B67" s="212" t="inlineStr">
         <is>
           <t>Shower Caddy</t>
         </is>
       </c>
-      <c r="C67" s="207" t="inlineStr">
+      <c r="C67" s="211" t="inlineStr">
         <is>
           <t>🔴 Cut</t>
         </is>
       </c>
-      <c r="D67" s="216" t="inlineStr">
+      <c r="D67" s="220" t="inlineStr">
         <is>
           <t>本週執行</t>
         </is>
       </c>
-      <c r="E67" s="209" t="inlineStr">
+      <c r="E67" s="213" t="inlineStr">
         <is>
           <t>Price</t>
         </is>
       </c>
-      <c r="F67" s="237" t="inlineStr">
+      <c r="F67" s="241" t="inlineStr">
         <is>
           <t>在 Seller Central 將售價下調 $0.50，觀察轉換率變化</t>
         </is>
       </c>
-      <c r="G67" s="210" t="n">
+      <c r="G67" s="214" t="n">
         <v>38.72</v>
       </c>
-      <c r="H67" s="211" t="n"/>
+      <c r="H67" s="215" t="n"/>
     </row>
     <row r="68" ht="28" customHeight="1">
-      <c r="A68" s="236" t="inlineStr"/>
-      <c r="B68" s="238" t="n"/>
-      <c r="C68" s="238" t="n"/>
-      <c r="D68" s="238" t="n"/>
-      <c r="E68" s="209" t="inlineStr">
+      <c r="A68" s="240" t="inlineStr"/>
+      <c r="B68" s="242" t="n"/>
+      <c r="C68" s="242" t="n"/>
+      <c r="D68" s="242" t="n"/>
+      <c r="E68" s="213" t="inlineStr">
         <is>
           <t>Coupon</t>
         </is>
       </c>
-      <c r="F68" s="237" t="inlineStr">
+      <c r="F68" s="241" t="inlineStr">
         <is>
           <t>建立 Coupon 折扣（建議 5–10%）→ 提升搜尋結果曝光</t>
         </is>
       </c>
-      <c r="G68" s="238" t="n"/>
-      <c r="H68" s="238" t="n"/>
+      <c r="G68" s="242" t="n"/>
+      <c r="H68" s="242" t="n"/>
     </row>
     <row r="69" ht="28" customHeight="1">
-      <c r="A69" s="236" t="inlineStr"/>
-      <c r="B69" s="238" t="n"/>
-      <c r="C69" s="238" t="n"/>
-      <c r="D69" s="238" t="n"/>
-      <c r="E69" s="209" t="inlineStr">
+      <c r="A69" s="240" t="inlineStr"/>
+      <c r="B69" s="242" t="n"/>
+      <c r="C69" s="242" t="n"/>
+      <c r="D69" s="242" t="n"/>
+      <c r="E69" s="213" t="inlineStr">
         <is>
           <t>Deal</t>
         </is>
       </c>
-      <c r="F69" s="237" t="inlineStr">
+      <c r="F69" s="241" t="inlineStr">
         <is>
           <t>申請 Prime Exclusive Discount 或 Lightning Deal（需提前 2 週申請）</t>
         </is>
       </c>
-      <c r="G69" s="238" t="n"/>
-      <c r="H69" s="238" t="n"/>
+      <c r="G69" s="242" t="n"/>
+      <c r="H69" s="242" t="n"/>
     </row>
     <row r="70" ht="28" customHeight="1">
-      <c r="A70" s="236" t="inlineStr"/>
-      <c r="B70" s="238" t="n"/>
-      <c r="C70" s="238" t="n"/>
-      <c r="D70" s="238" t="n"/>
-      <c r="E70" s="209" t="inlineStr">
+      <c r="A70" s="240" t="inlineStr"/>
+      <c r="B70" s="242" t="n"/>
+      <c r="C70" s="242" t="n"/>
+      <c r="D70" s="242" t="n"/>
+      <c r="E70" s="213" t="inlineStr">
         <is>
           <t>SP Bid</t>
         </is>
       </c>
-      <c r="F70" s="237" t="inlineStr">
+      <c r="F70" s="241" t="inlineStr">
         <is>
           <t>下載 SP Bulk File → 全部 Keyword Bid 降至 $2.00 上限</t>
         </is>
       </c>
-      <c r="G70" s="238" t="n"/>
-      <c r="H70" s="238" t="n"/>
+      <c r="G70" s="242" t="n"/>
+      <c r="H70" s="242" t="n"/>
     </row>
     <row r="71" ht="4" customHeight="1">
-      <c r="A71" s="232" t="n"/>
-      <c r="B71" s="232" t="n"/>
-      <c r="C71" s="232" t="n"/>
-      <c r="D71" s="232" t="n"/>
-      <c r="E71" s="232" t="n"/>
-      <c r="F71" s="232" t="n"/>
-      <c r="G71" s="232" t="n"/>
-      <c r="H71" s="232" t="n"/>
+      <c r="A71" s="236" t="n"/>
+      <c r="B71" s="236" t="n"/>
+      <c r="C71" s="236" t="n"/>
+      <c r="D71" s="236" t="n"/>
+      <c r="E71" s="236" t="n"/>
+      <c r="F71" s="236" t="n"/>
+      <c r="G71" s="236" t="n"/>
+      <c r="H71" s="236" t="n"/>
     </row>
     <row r="72" ht="15" customHeight="1">
-      <c r="A72" s="218" t="inlineStr">
+      <c r="A72" s="222" t="inlineStr">
         <is>
           <t xml:space="preserve">  💤 Potential  —  低銷售 · 低 TACOS</t>
         </is>
       </c>
     </row>
     <row r="73" ht="28" customHeight="1">
-      <c r="A73" s="239" t="inlineStr"/>
-      <c r="B73" s="220" t="inlineStr">
+      <c r="A73" s="243" t="inlineStr"/>
+      <c r="B73" s="224" t="inlineStr">
         <is>
           <t>Padded Hangers</t>
         </is>
       </c>
-      <c r="C73" s="219" t="inlineStr">
+      <c r="C73" s="223" t="inlineStr">
         <is>
           <t>💤 Potential</t>
         </is>
       </c>
-      <c r="D73" s="228" t="inlineStr">
+      <c r="D73" s="232" t="inlineStr">
         <is>
           <t>下週執行</t>
         </is>
       </c>
-      <c r="E73" s="221" t="inlineStr">
+      <c r="E73" s="225" t="inlineStr">
         <is>
           <t>SP</t>
         </is>
       </c>
-      <c r="F73" s="240" t="inlineStr">
+      <c r="F73" s="244" t="inlineStr">
         <is>
           <t>新建 SP Auto campaign，日預算 $10，CPC 出價 $2.00，30天跑數據</t>
         </is>
       </c>
-      <c r="G73" s="222" t="n">
+      <c r="G73" s="226" t="n">
         <v>734.41</v>
       </c>
-      <c r="H73" s="223" t="n">
+      <c r="H73" s="227" t="n">
         <v>0.09300000000000001</v>
       </c>
     </row>
     <row r="74" ht="28" customHeight="1">
-      <c r="A74" s="239" t="inlineStr"/>
-      <c r="B74" s="241" t="n"/>
-      <c r="C74" s="241" t="n"/>
-      <c r="D74" s="241" t="n"/>
-      <c r="E74" s="221" t="inlineStr">
+      <c r="A74" s="243" t="inlineStr"/>
+      <c r="B74" s="245" t="n"/>
+      <c r="C74" s="245" t="n"/>
+      <c r="D74" s="245" t="n"/>
+      <c r="E74" s="225" t="inlineStr">
         <is>
           <t>SB</t>
         </is>
       </c>
-      <c r="F74" s="240" t="inlineStr">
+      <c r="F74" s="244" t="inlineStr">
         <is>
           <t>新建 SB Banner campaign，指向此產品 Store Page，CPC $2.00</t>
         </is>
       </c>
-      <c r="G74" s="241" t="n"/>
-      <c r="H74" s="241" t="n"/>
+      <c r="G74" s="245" t="n"/>
+      <c r="H74" s="245" t="n"/>
     </row>
     <row r="75" ht="28" customHeight="1">
-      <c r="A75" s="239" t="inlineStr"/>
-      <c r="B75" s="241" t="n"/>
-      <c r="C75" s="241" t="n"/>
-      <c r="D75" s="241" t="n"/>
-      <c r="E75" s="221" t="inlineStr">
+      <c r="A75" s="243" t="inlineStr"/>
+      <c r="B75" s="245" t="n"/>
+      <c r="C75" s="245" t="n"/>
+      <c r="D75" s="245" t="n"/>
+      <c r="E75" s="225" t="inlineStr">
         <is>
           <t>SD</t>
         </is>
       </c>
-      <c r="F75" s="240" t="inlineStr">
+      <c r="F75" s="244" t="inlineStr">
         <is>
           <t>新建 SD Audience campaign，目標 Competitor ASIN 的瀏覽受眾</t>
         </is>
       </c>
-      <c r="G75" s="241" t="n"/>
-      <c r="H75" s="241" t="n"/>
+      <c r="G75" s="245" t="n"/>
+      <c r="H75" s="245" t="n"/>
     </row>
     <row r="76" ht="28" customHeight="1">
-      <c r="A76" s="239" t="inlineStr"/>
-      <c r="B76" s="241" t="n"/>
-      <c r="C76" s="241" t="n"/>
-      <c r="D76" s="241" t="n"/>
-      <c r="E76" s="221" t="inlineStr">
+      <c r="A76" s="243" t="inlineStr"/>
+      <c r="B76" s="245" t="n"/>
+      <c r="C76" s="245" t="n"/>
+      <c r="D76" s="245" t="n"/>
+      <c r="E76" s="225" t="inlineStr">
         <is>
           <t>AMC</t>
         </is>
       </c>
-      <c r="F76" s="240" t="inlineStr">
+      <c r="F76" s="244" t="inlineStr">
         <is>
           <t>建立 AMC Lookalike 受眾 → 相似購買行為 → 套用至 SD campaign</t>
         </is>
       </c>
-      <c r="G76" s="241" t="n"/>
-      <c r="H76" s="241" t="n"/>
+      <c r="G76" s="245" t="n"/>
+      <c r="H76" s="245" t="n"/>
     </row>
     <row r="77" ht="28" customHeight="1">
-      <c r="A77" s="239" t="inlineStr"/>
-      <c r="B77" s="241" t="n"/>
-      <c r="C77" s="241" t="n"/>
-      <c r="D77" s="241" t="n"/>
-      <c r="E77" s="221" t="inlineStr">
+      <c r="A77" s="243" t="inlineStr"/>
+      <c r="B77" s="245" t="n"/>
+      <c r="C77" s="245" t="n"/>
+      <c r="D77" s="245" t="n"/>
+      <c r="E77" s="225" t="inlineStr">
         <is>
           <t>KW</t>
         </is>
       </c>
-      <c r="F77" s="240" t="inlineStr">
+      <c r="F77" s="244" t="inlineStr">
         <is>
           <t>用現有暢銷產品的高轉換 KW 根詞，建立 SP Exact Match campaign</t>
         </is>
       </c>
-      <c r="G77" s="241" t="n"/>
-      <c r="H77" s="241" t="n"/>
+      <c r="G77" s="245" t="n"/>
+      <c r="H77" s="245" t="n"/>
     </row>
     <row r="78" ht="4" customHeight="1">
-      <c r="A78" s="232" t="n"/>
-      <c r="B78" s="232" t="n"/>
-      <c r="C78" s="232" t="n"/>
-      <c r="D78" s="232" t="n"/>
-      <c r="E78" s="232" t="n"/>
-      <c r="F78" s="232" t="n"/>
-      <c r="G78" s="232" t="n"/>
-      <c r="H78" s="232" t="n"/>
+      <c r="A78" s="236" t="n"/>
+      <c r="B78" s="236" t="n"/>
+      <c r="C78" s="236" t="n"/>
+      <c r="D78" s="236" t="n"/>
+      <c r="E78" s="236" t="n"/>
+      <c r="F78" s="236" t="n"/>
+      <c r="G78" s="236" t="n"/>
+      <c r="H78" s="236" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -21348,71 +21656,71 @@
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="242" t="inlineStr">
+      <c r="A1" s="246" t="inlineStr">
         <is>
           <t>DBJ US · Inventory Age Snapshot · VINE $12,153 deducted from Sales</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="243" t="inlineStr">
+      <c r="A2" s="247" t="inlineStr">
         <is>
           <t>ASIN</t>
         </is>
       </c>
-      <c r="B2" s="243" t="inlineStr">
+      <c r="B2" s="247" t="inlineStr">
         <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="C2" s="243" t="inlineStr">
+      <c r="C2" s="247" t="inlineStr">
         <is>
           <t>Available</t>
         </is>
       </c>
-      <c r="D2" s="243" t="inlineStr">
+      <c r="D2" s="247" t="inlineStr">
         <is>
           <t>0–30d</t>
         </is>
       </c>
-      <c r="E2" s="243" t="inlineStr">
+      <c r="E2" s="247" t="inlineStr">
         <is>
           <t>31–60d</t>
         </is>
       </c>
-      <c r="F2" s="243" t="inlineStr">
+      <c r="F2" s="247" t="inlineStr">
         <is>
           <t>61–90d</t>
         </is>
       </c>
-      <c r="G2" s="243" t="inlineStr">
+      <c r="G2" s="247" t="inlineStr">
         <is>
           <t>91–180d</t>
         </is>
       </c>
-      <c r="H2" s="243" t="inlineStr">
+      <c r="H2" s="247" t="inlineStr">
         <is>
           <t>181+d</t>
         </is>
       </c>
-      <c r="I2" s="243" t="inlineStr">
+      <c r="I2" s="247" t="inlineStr">
         <is>
           <t>Shipped 30d</t>
         </is>
       </c>
-      <c r="J2" s="243" t="inlineStr">
+      <c r="J2" s="247" t="inlineStr">
         <is>
           <t>Days of Supply</t>
         </is>
       </c>
-      <c r="K2" s="243" t="inlineStr">
+      <c r="K2" s="247" t="inlineStr">
         <is>
           <t>Inbound</t>
         </is>
       </c>
     </row>
     <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="244" t="inlineStr">
+      <c r="A3" s="248" t="inlineStr">
         <is>
           <t>B0FV8YQTLZ</t>
         </is>
@@ -21422,30 +21730,30 @@
           <t>2-Tier Extendable Shoe Rack</t>
         </is>
       </c>
-      <c r="C3" s="245" t="n">
+      <c r="C3" s="249" t="n">
         <v>48</v>
       </c>
-      <c r="D3" s="246" t="n">
+      <c r="D3" s="250" t="n">
         <v>6</v>
       </c>
-      <c r="E3" s="247" t="n">
+      <c r="E3" s="251" t="n">
         <v>35</v>
       </c>
-      <c r="F3" s="248" t="n">
+      <c r="F3" s="252" t="n">
         <v>7</v>
       </c>
-      <c r="G3" s="245" t="n"/>
-      <c r="H3" s="245" t="n"/>
-      <c r="I3" s="249" t="n">
+      <c r="G3" s="249" t="n"/>
+      <c r="H3" s="249" t="n"/>
+      <c r="I3" s="253" t="n">
         <v>1</v>
       </c>
-      <c r="J3" s="250" t="n">
+      <c r="J3" s="254" t="n">
         <v>351</v>
       </c>
       <c r="K3" s="28" t="n"/>
     </row>
     <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="251" t="inlineStr">
+      <c r="A4" s="255" t="inlineStr">
         <is>
           <t>B09MRGLH3L</t>
         </is>
@@ -21455,28 +21763,28 @@
           <t>Shower Caddy Organizer</t>
         </is>
       </c>
-      <c r="C4" s="252" t="n">
+      <c r="C4" s="256" t="n">
         <v>14</v>
       </c>
-      <c r="D4" s="252" t="n"/>
-      <c r="E4" s="247" t="n">
+      <c r="D4" s="256" t="n"/>
+      <c r="E4" s="251" t="n">
         <v>12</v>
       </c>
-      <c r="F4" s="252" t="n"/>
-      <c r="G4" s="252" t="n"/>
-      <c r="H4" s="253" t="n">
+      <c r="F4" s="256" t="n"/>
+      <c r="G4" s="256" t="n"/>
+      <c r="H4" s="257" t="n">
         <v>2</v>
       </c>
-      <c r="I4" s="254" t="n">
+      <c r="I4" s="258" t="n">
         <v>1</v>
       </c>
-      <c r="J4" s="250" t="n">
+      <c r="J4" s="254" t="n">
         <v>315</v>
       </c>
       <c r="K4" s="12" t="n"/>
     </row>
     <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="244" t="inlineStr">
+      <c r="A5" s="248" t="inlineStr">
         <is>
           <t>B0FV8YD8DP</t>
         </is>
@@ -21486,28 +21794,28 @@
           <t>3-Tier Rolling Cart Metal</t>
         </is>
       </c>
-      <c r="C5" s="245" t="n">
+      <c r="C5" s="249" t="n">
         <v>28</v>
       </c>
-      <c r="D5" s="246" t="n">
+      <c r="D5" s="250" t="n">
         <v>67</v>
       </c>
-      <c r="E5" s="247" t="n">
+      <c r="E5" s="251" t="n">
         <v>11</v>
       </c>
-      <c r="F5" s="245" t="n"/>
-      <c r="G5" s="245" t="n"/>
-      <c r="H5" s="245" t="n"/>
-      <c r="I5" s="249" t="n">
+      <c r="F5" s="249" t="n"/>
+      <c r="G5" s="249" t="n"/>
+      <c r="H5" s="249" t="n"/>
+      <c r="I5" s="253" t="n">
         <v>32</v>
       </c>
-      <c r="J5" s="250" t="n">
+      <c r="J5" s="254" t="n">
         <v>281</v>
       </c>
       <c r="K5" s="28" t="n"/>
     </row>
     <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="251" t="inlineStr">
+      <c r="A6" s="255" t="inlineStr">
         <is>
           <t>B091X2PXZP</t>
         </is>
@@ -21517,30 +21825,30 @@
           <t>5-Tier Wire Shelving Unit</t>
         </is>
       </c>
-      <c r="C6" s="252" t="n">
+      <c r="C6" s="256" t="n">
         <v>51</v>
       </c>
-      <c r="D6" s="252" t="n"/>
-      <c r="E6" s="247" t="n">
+      <c r="D6" s="256" t="n"/>
+      <c r="E6" s="251" t="n">
         <v>1</v>
       </c>
-      <c r="F6" s="248" t="n">
+      <c r="F6" s="252" t="n">
         <v>21</v>
       </c>
-      <c r="G6" s="255" t="n">
+      <c r="G6" s="259" t="n">
         <v>34</v>
       </c>
-      <c r="H6" s="252" t="n"/>
-      <c r="I6" s="254" t="n">
+      <c r="H6" s="256" t="n"/>
+      <c r="I6" s="258" t="n">
         <v>5</v>
       </c>
-      <c r="J6" s="250" t="n">
+      <c r="J6" s="254" t="n">
         <v>214</v>
       </c>
       <c r="K6" s="12" t="n"/>
     </row>
     <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="244" t="inlineStr">
+      <c r="A7" s="248" t="inlineStr">
         <is>
           <t>B097V3JSWH</t>
         </is>
@@ -21550,26 +21858,26 @@
           <t>Clothing Dryer Rack</t>
         </is>
       </c>
-      <c r="C7" s="245" t="n">
+      <c r="C7" s="249" t="n">
         <v>120</v>
       </c>
-      <c r="D7" s="245" t="n"/>
-      <c r="E7" s="247" t="n">
+      <c r="D7" s="249" t="n"/>
+      <c r="E7" s="251" t="n">
         <v>132</v>
       </c>
-      <c r="F7" s="245" t="n"/>
-      <c r="G7" s="245" t="n"/>
-      <c r="H7" s="245" t="n"/>
-      <c r="I7" s="249" t="n">
+      <c r="F7" s="249" t="n"/>
+      <c r="G7" s="249" t="n"/>
+      <c r="H7" s="249" t="n"/>
+      <c r="I7" s="253" t="n">
         <v>22</v>
       </c>
-      <c r="J7" s="256" t="n">
+      <c r="J7" s="260" t="n">
         <v>119</v>
       </c>
       <c r="K7" s="28" t="n"/>
     </row>
     <row r="8" ht="16" customHeight="1">
-      <c r="A8" s="251" t="inlineStr">
+      <c r="A8" s="255" t="inlineStr">
         <is>
           <t>B08M5G2LLT</t>
         </is>
@@ -21579,30 +21887,30 @@
           <t>5-Tier Wire Shelving Heavy Duty</t>
         </is>
       </c>
-      <c r="C8" s="252" t="n">
+      <c r="C8" s="256" t="n">
         <v>31</v>
       </c>
-      <c r="D8" s="246" t="n">
+      <c r="D8" s="250" t="n">
         <v>14</v>
       </c>
-      <c r="E8" s="252" t="n"/>
-      <c r="F8" s="248" t="n">
+      <c r="E8" s="256" t="n"/>
+      <c r="F8" s="252" t="n">
         <v>18</v>
       </c>
-      <c r="G8" s="252" t="n"/>
-      <c r="H8" s="252" t="n"/>
-      <c r="I8" s="254" t="n">
+      <c r="G8" s="256" t="n"/>
+      <c r="H8" s="256" t="n"/>
+      <c r="I8" s="258" t="n">
         <v>10</v>
       </c>
-      <c r="J8" s="256" t="n">
+      <c r="J8" s="260" t="n">
         <v>107</v>
       </c>
-      <c r="K8" s="257" t="n">
+      <c r="K8" s="261" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="244" t="inlineStr">
+      <c r="A9" s="248" t="inlineStr">
         <is>
           <t>B09Z58XKBP</t>
         </is>
@@ -21612,30 +21920,30 @@
           <t>4-Tier Wire Shelving Unit</t>
         </is>
       </c>
-      <c r="C9" s="245" t="n">
+      <c r="C9" s="249" t="n">
         <v>19</v>
       </c>
-      <c r="D9" s="245" t="n"/>
-      <c r="E9" s="245" t="n"/>
-      <c r="F9" s="248" t="n">
+      <c r="D9" s="249" t="n"/>
+      <c r="E9" s="249" t="n"/>
+      <c r="F9" s="252" t="n">
         <v>14</v>
       </c>
-      <c r="G9" s="255" t="n">
+      <c r="G9" s="259" t="n">
         <v>6</v>
       </c>
-      <c r="H9" s="245" t="n"/>
-      <c r="I9" s="249" t="n">
+      <c r="H9" s="249" t="n"/>
+      <c r="I9" s="253" t="n">
         <v>12</v>
       </c>
-      <c r="J9" s="256" t="n">
+      <c r="J9" s="260" t="n">
         <v>90</v>
       </c>
-      <c r="K9" s="258" t="n">
+      <c r="K9" s="262" t="n">
         <v>20</v>
       </c>
     </row>
     <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="251" t="inlineStr">
+      <c r="A10" s="255" t="inlineStr">
         <is>
           <t>B094XBLMGH</t>
         </is>
@@ -21645,30 +21953,30 @@
           <t>3-Tier Wire Shelving B</t>
         </is>
       </c>
-      <c r="C10" s="252" t="n">
+      <c r="C10" s="256" t="n">
         <v>35</v>
       </c>
-      <c r="D10" s="246" t="n">
+      <c r="D10" s="250" t="n">
         <v>11</v>
       </c>
-      <c r="E10" s="247" t="n">
+      <c r="E10" s="251" t="n">
         <v>24</v>
       </c>
-      <c r="F10" s="252" t="n"/>
-      <c r="G10" s="252" t="n"/>
-      <c r="H10" s="252" t="n"/>
-      <c r="I10" s="254" t="n">
+      <c r="F10" s="256" t="n"/>
+      <c r="G10" s="256" t="n"/>
+      <c r="H10" s="256" t="n"/>
+      <c r="I10" s="258" t="n">
         <v>29</v>
       </c>
-      <c r="J10" s="256" t="n">
+      <c r="J10" s="260" t="n">
         <v>89</v>
       </c>
-      <c r="K10" s="257" t="n">
+      <c r="K10" s="261" t="n">
         <v>24</v>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
-      <c r="A11" s="244" t="inlineStr">
+      <c r="A11" s="248" t="inlineStr">
         <is>
           <t>B08ZXJR1DP</t>
         </is>
@@ -21678,28 +21986,28 @@
           <t>4-Tier Wire Shelving Heavy Duty</t>
         </is>
       </c>
-      <c r="C11" s="245" t="n">
+      <c r="C11" s="249" t="n">
         <v>48</v>
       </c>
-      <c r="D11" s="246" t="n">
+      <c r="D11" s="250" t="n">
         <v>46</v>
       </c>
-      <c r="E11" s="247" t="n">
+      <c r="E11" s="251" t="n">
         <v>20</v>
       </c>
-      <c r="F11" s="245" t="n"/>
-      <c r="G11" s="245" t="n"/>
-      <c r="H11" s="245" t="n"/>
-      <c r="I11" s="249" t="n">
+      <c r="F11" s="249" t="n"/>
+      <c r="G11" s="249" t="n"/>
+      <c r="H11" s="249" t="n"/>
+      <c r="I11" s="253" t="n">
         <v>19</v>
       </c>
-      <c r="J11" s="256" t="n">
+      <c r="J11" s="260" t="n">
         <v>85</v>
       </c>
       <c r="K11" s="28" t="n"/>
     </row>
     <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="251" t="inlineStr">
+      <c r="A12" s="255" t="inlineStr">
         <is>
           <t>B0CTK9VRFR</t>
         </is>
@@ -21709,28 +22017,28 @@
           <t>Sweater Hangers Padded Black</t>
         </is>
       </c>
-      <c r="C12" s="252" t="n">
+      <c r="C12" s="256" t="n">
         <v>91</v>
       </c>
-      <c r="D12" s="246" t="n">
+      <c r="D12" s="250" t="n">
         <v>11</v>
       </c>
-      <c r="E12" s="247" t="n">
+      <c r="E12" s="251" t="n">
         <v>82</v>
       </c>
-      <c r="F12" s="252" t="n"/>
-      <c r="G12" s="252" t="n"/>
-      <c r="H12" s="252" t="n"/>
-      <c r="I12" s="254" t="n">
+      <c r="F12" s="256" t="n"/>
+      <c r="G12" s="256" t="n"/>
+      <c r="H12" s="256" t="n"/>
+      <c r="I12" s="258" t="n">
         <v>31</v>
       </c>
-      <c r="J12" s="256" t="n">
+      <c r="J12" s="260" t="n">
         <v>81</v>
       </c>
       <c r="K12" s="12" t="n"/>
     </row>
     <row r="13" ht="16" customHeight="1">
-      <c r="A13" s="244" t="inlineStr">
+      <c r="A13" s="248" t="inlineStr">
         <is>
           <t>B09QW5PD83</t>
         </is>
@@ -21740,32 +22048,32 @@
           <t>Sweater Hangers Multi</t>
         </is>
       </c>
-      <c r="C13" s="245" t="n">
+      <c r="C13" s="249" t="n">
         <v>50</v>
       </c>
-      <c r="D13" s="246" t="n">
+      <c r="D13" s="250" t="n">
         <v>25</v>
       </c>
-      <c r="E13" s="247" t="n">
+      <c r="E13" s="251" t="n">
         <v>25</v>
       </c>
-      <c r="F13" s="248" t="n">
+      <c r="F13" s="252" t="n">
         <v>3</v>
       </c>
-      <c r="G13" s="245" t="n"/>
-      <c r="H13" s="245" t="n"/>
-      <c r="I13" s="249" t="n">
+      <c r="G13" s="249" t="n"/>
+      <c r="H13" s="249" t="n"/>
+      <c r="I13" s="253" t="n">
         <v>21</v>
       </c>
-      <c r="J13" s="256" t="n">
+      <c r="J13" s="260" t="n">
         <v>77</v>
       </c>
-      <c r="K13" s="258" t="n">
+      <c r="K13" s="262" t="n">
         <v>24</v>
       </c>
     </row>
     <row r="14" ht="16" customHeight="1">
-      <c r="A14" s="251" t="inlineStr">
+      <c r="A14" s="255" t="inlineStr">
         <is>
           <t>B09JBVTY9T</t>
         </is>
@@ -21775,30 +22083,30 @@
           <t>Broom &amp; Mop Holder</t>
         </is>
       </c>
-      <c r="C14" s="252" t="n">
+      <c r="C14" s="256" t="n">
         <v>6</v>
       </c>
-      <c r="D14" s="252" t="n"/>
-      <c r="E14" s="247" t="n">
+      <c r="D14" s="256" t="n"/>
+      <c r="E14" s="251" t="n">
         <v>2</v>
       </c>
-      <c r="F14" s="248" t="n">
+      <c r="F14" s="252" t="n">
         <v>8</v>
       </c>
-      <c r="G14" s="252" t="n"/>
-      <c r="H14" s="252" t="n"/>
-      <c r="I14" s="254" t="n">
+      <c r="G14" s="256" t="n"/>
+      <c r="H14" s="256" t="n"/>
+      <c r="I14" s="258" t="n">
         <v>17</v>
       </c>
-      <c r="J14" s="256" t="n">
+      <c r="J14" s="260" t="n">
         <v>71</v>
       </c>
-      <c r="K14" s="257" t="n">
+      <c r="K14" s="261" t="n">
         <v>20</v>
       </c>
     </row>
     <row r="15" ht="16" customHeight="1">
-      <c r="A15" s="244" t="inlineStr">
+      <c r="A15" s="248" t="inlineStr">
         <is>
           <t>B094X854R4</t>
         </is>
@@ -21808,30 +22116,30 @@
           <t>3-Tier Wire Shelving 14x24x30</t>
         </is>
       </c>
-      <c r="C15" s="245" t="n">
+      <c r="C15" s="249" t="n">
         <v>48</v>
       </c>
-      <c r="D15" s="246" t="n">
+      <c r="D15" s="250" t="n">
         <v>35</v>
       </c>
-      <c r="E15" s="247" t="n">
+      <c r="E15" s="251" t="n">
         <v>13</v>
       </c>
-      <c r="F15" s="245" t="n"/>
-      <c r="G15" s="245" t="n"/>
-      <c r="H15" s="245" t="n"/>
-      <c r="I15" s="249" t="n">
+      <c r="F15" s="249" t="n"/>
+      <c r="G15" s="249" t="n"/>
+      <c r="H15" s="249" t="n"/>
+      <c r="I15" s="253" t="n">
         <v>36</v>
       </c>
-      <c r="J15" s="256" t="n">
+      <c r="J15" s="260" t="n">
         <v>68</v>
       </c>
-      <c r="K15" s="258" t="n">
+      <c r="K15" s="262" t="n">
         <v>31</v>
       </c>
     </row>
     <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="251" t="inlineStr">
+      <c r="A16" s="255" t="inlineStr">
         <is>
           <t>B0FV8XKYPM</t>
         </is>
@@ -21841,28 +22149,28 @@
           <t>4-Tier Stackable Shoe Rack Set2</t>
         </is>
       </c>
-      <c r="C16" s="252" t="n">
+      <c r="C16" s="256" t="n">
         <v>22</v>
       </c>
-      <c r="D16" s="246" t="n">
+      <c r="D16" s="250" t="n">
         <v>26</v>
       </c>
-      <c r="E16" s="247" t="n">
+      <c r="E16" s="251" t="n">
         <v>15</v>
       </c>
-      <c r="F16" s="252" t="n"/>
-      <c r="G16" s="252" t="n"/>
-      <c r="H16" s="252" t="n"/>
-      <c r="I16" s="254" t="n">
+      <c r="F16" s="256" t="n"/>
+      <c r="G16" s="256" t="n"/>
+      <c r="H16" s="256" t="n"/>
+      <c r="I16" s="258" t="n">
         <v>26</v>
       </c>
-      <c r="J16" s="259" t="n">
+      <c r="J16" s="263" t="n">
         <v>56</v>
       </c>
       <c r="K16" s="12" t="n"/>
     </row>
     <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="244" t="inlineStr">
+      <c r="A17" s="248" t="inlineStr">
         <is>
           <t>B0FVFGJT63</t>
         </is>
@@ -21872,28 +22180,28 @@
           <t>Storage Cart 10D Black</t>
         </is>
       </c>
-      <c r="C17" s="260" t="n">
-        <v>0</v>
-      </c>
-      <c r="D17" s="246" t="n">
+      <c r="C17" s="264" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="250" t="n">
         <v>20</v>
       </c>
-      <c r="E17" s="245" t="n"/>
-      <c r="F17" s="245" t="n"/>
-      <c r="G17" s="245" t="n"/>
-      <c r="H17" s="245" t="n"/>
-      <c r="I17" s="249" t="n">
+      <c r="E17" s="249" t="n"/>
+      <c r="F17" s="249" t="n"/>
+      <c r="G17" s="249" t="n"/>
+      <c r="H17" s="249" t="n"/>
+      <c r="I17" s="253" t="n">
         <v>27</v>
       </c>
-      <c r="J17" s="259" t="n">
+      <c r="J17" s="263" t="n">
         <v>46</v>
       </c>
-      <c r="K17" s="258" t="n">
+      <c r="K17" s="262" t="n">
         <v>36</v>
       </c>
     </row>
     <row r="18" ht="16" customHeight="1">
-      <c r="A18" s="251" t="inlineStr">
+      <c r="A18" s="255" t="inlineStr">
         <is>
           <t>B0FVF8DRZQ</t>
         </is>
@@ -21903,28 +22211,28 @@
           <t>Rolling Laptop Desk Silver</t>
         </is>
       </c>
-      <c r="C18" s="252" t="n">
+      <c r="C18" s="256" t="n">
         <v>21</v>
       </c>
-      <c r="D18" s="246" t="n">
+      <c r="D18" s="250" t="n">
         <v>13</v>
       </c>
-      <c r="E18" s="247" t="n">
+      <c r="E18" s="251" t="n">
         <v>14</v>
       </c>
-      <c r="F18" s="252" t="n"/>
-      <c r="G18" s="252" t="n"/>
-      <c r="H18" s="252" t="n"/>
-      <c r="I18" s="254" t="n">
+      <c r="F18" s="256" t="n"/>
+      <c r="G18" s="256" t="n"/>
+      <c r="H18" s="256" t="n"/>
+      <c r="I18" s="258" t="n">
         <v>18</v>
       </c>
-      <c r="J18" s="259" t="n">
+      <c r="J18" s="263" t="n">
         <v>43</v>
       </c>
       <c r="K18" s="12" t="n"/>
     </row>
     <row r="19" ht="16" customHeight="1">
-      <c r="A19" s="244" t="inlineStr">
+      <c r="A19" s="248" t="inlineStr">
         <is>
           <t>B0FVD69MYD</t>
         </is>
@@ -21934,28 +22242,28 @@
           <t>Rolling Laptop Desk Tilt</t>
         </is>
       </c>
-      <c r="C19" s="245" t="n">
+      <c r="C19" s="249" t="n">
         <v>19</v>
       </c>
-      <c r="D19" s="246" t="n">
+      <c r="D19" s="250" t="n">
         <v>6</v>
       </c>
-      <c r="E19" s="247" t="n">
+      <c r="E19" s="251" t="n">
         <v>13</v>
       </c>
-      <c r="F19" s="245" t="n"/>
-      <c r="G19" s="245" t="n"/>
-      <c r="H19" s="245" t="n"/>
-      <c r="I19" s="249" t="n">
+      <c r="F19" s="249" t="n"/>
+      <c r="G19" s="249" t="n"/>
+      <c r="H19" s="249" t="n"/>
+      <c r="I19" s="253" t="n">
         <v>31</v>
       </c>
-      <c r="J19" s="259" t="n">
+      <c r="J19" s="263" t="n">
         <v>34</v>
       </c>
       <c r="K19" s="28" t="n"/>
     </row>
     <row r="20" ht="16" customHeight="1">
-      <c r="A20" s="251" t="inlineStr">
+      <c r="A20" s="255" t="inlineStr">
         <is>
           <t>B0FVFCJXWB</t>
         </is>
@@ -21965,28 +22273,28 @@
           <t>Bathroom Storage Rack</t>
         </is>
       </c>
-      <c r="C20" s="252" t="n">
+      <c r="C20" s="256" t="n">
         <v>19</v>
       </c>
-      <c r="D20" s="246" t="n">
+      <c r="D20" s="250" t="n">
         <v>6</v>
       </c>
-      <c r="E20" s="247" t="n">
+      <c r="E20" s="251" t="n">
         <v>13</v>
       </c>
-      <c r="F20" s="252" t="n"/>
-      <c r="G20" s="252" t="n"/>
-      <c r="H20" s="252" t="n"/>
-      <c r="I20" s="254" t="n">
+      <c r="F20" s="256" t="n"/>
+      <c r="G20" s="256" t="n"/>
+      <c r="H20" s="256" t="n"/>
+      <c r="I20" s="258" t="n">
         <v>31</v>
       </c>
-      <c r="J20" s="259" t="n">
+      <c r="J20" s="263" t="n">
         <v>31</v>
       </c>
       <c r="K20" s="12" t="n"/>
     </row>
     <row r="21" ht="16" customHeight="1">
-      <c r="A21" s="244" t="inlineStr">
+      <c r="A21" s="248" t="inlineStr">
         <is>
           <t>B0FVD1Z92C</t>
         </is>
@@ -21996,28 +22304,28 @@
           <t>Rolling Laptop Desk Sit-Stand</t>
         </is>
       </c>
-      <c r="C21" s="245" t="n">
+      <c r="C21" s="249" t="n">
         <v>21</v>
       </c>
-      <c r="D21" s="246" t="n">
+      <c r="D21" s="250" t="n">
         <v>7</v>
       </c>
-      <c r="E21" s="247" t="n">
+      <c r="E21" s="251" t="n">
         <v>14</v>
       </c>
-      <c r="F21" s="245" t="n"/>
-      <c r="G21" s="245" t="n"/>
-      <c r="H21" s="245" t="n"/>
-      <c r="I21" s="249" t="n">
+      <c r="F21" s="249" t="n"/>
+      <c r="G21" s="249" t="n"/>
+      <c r="H21" s="249" t="n"/>
+      <c r="I21" s="253" t="n">
         <v>29</v>
       </c>
-      <c r="J21" s="259" t="n">
+      <c r="J21" s="263" t="n">
         <v>29</v>
       </c>
       <c r="K21" s="28" t="n"/>
     </row>
     <row r="22" ht="16" customHeight="1">
-      <c r="A22" s="251" t="inlineStr">
+      <c r="A22" s="255" t="inlineStr">
         <is>
           <t>B0FV8XGQV4</t>
         </is>
@@ -22027,28 +22335,28 @@
           <t>Double Rail Clothes Rack</t>
         </is>
       </c>
-      <c r="C22" s="252" t="n">
+      <c r="C22" s="256" t="n">
         <v>20</v>
       </c>
-      <c r="D22" s="246" t="n">
+      <c r="D22" s="250" t="n">
         <v>6</v>
       </c>
-      <c r="E22" s="247" t="n">
+      <c r="E22" s="251" t="n">
         <v>14</v>
       </c>
-      <c r="F22" s="252" t="n"/>
-      <c r="G22" s="252" t="n"/>
-      <c r="H22" s="252" t="n"/>
-      <c r="I22" s="254" t="n">
+      <c r="F22" s="256" t="n"/>
+      <c r="G22" s="256" t="n"/>
+      <c r="H22" s="256" t="n"/>
+      <c r="I22" s="258" t="n">
         <v>30</v>
       </c>
-      <c r="J22" s="259" t="n">
+      <c r="J22" s="263" t="n">
         <v>28</v>
       </c>
       <c r="K22" s="12" t="n"/>
     </row>
     <row r="23" ht="16" customHeight="1">
-      <c r="A23" s="244" t="inlineStr">
+      <c r="A23" s="248" t="inlineStr">
         <is>
           <t>B0FVF9GS2S</t>
         </is>
@@ -22058,28 +22366,28 @@
           <t>Storage Cart 10D White</t>
         </is>
       </c>
-      <c r="C23" s="260" t="n">
-        <v>0</v>
-      </c>
-      <c r="D23" s="246" t="n">
+      <c r="C23" s="264" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="250" t="n">
         <v>1</v>
       </c>
-      <c r="E23" s="245" t="n"/>
-      <c r="F23" s="245" t="n"/>
-      <c r="G23" s="245" t="n"/>
-      <c r="H23" s="245" t="n"/>
-      <c r="I23" s="249" t="n">
+      <c r="E23" s="249" t="n"/>
+      <c r="F23" s="249" t="n"/>
+      <c r="G23" s="249" t="n"/>
+      <c r="H23" s="249" t="n"/>
+      <c r="I23" s="253" t="n">
         <v>29</v>
       </c>
-      <c r="J23" s="259" t="n">
+      <c r="J23" s="263" t="n">
         <v>27</v>
       </c>
-      <c r="K23" s="258" t="n">
+      <c r="K23" s="262" t="n">
         <v>36</v>
       </c>
     </row>
     <row r="24" ht="16" customHeight="1">
-      <c r="A24" s="251" t="inlineStr">
+      <c r="A24" s="255" t="inlineStr">
         <is>
           <t>B0FVFBZKSQ</t>
         </is>
@@ -22089,30 +22397,30 @@
           <t>Storage Cart 10D Rainbow</t>
         </is>
       </c>
-      <c r="C24" s="261" t="n">
-        <v>0</v>
-      </c>
-      <c r="D24" s="246" t="n">
+      <c r="C24" s="265" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="250" t="n">
         <v>26</v>
       </c>
-      <c r="E24" s="247" t="n">
+      <c r="E24" s="251" t="n">
         <v>8</v>
       </c>
-      <c r="F24" s="252" t="n"/>
-      <c r="G24" s="252" t="n"/>
-      <c r="H24" s="252" t="n"/>
-      <c r="I24" s="254" t="n">
+      <c r="F24" s="256" t="n"/>
+      <c r="G24" s="256" t="n"/>
+      <c r="H24" s="256" t="n"/>
+      <c r="I24" s="258" t="n">
         <v>35</v>
       </c>
-      <c r="J24" s="259" t="n">
+      <c r="J24" s="263" t="n">
         <v>27</v>
       </c>
-      <c r="K24" s="257" t="n">
+      <c r="K24" s="261" t="n">
         <v>40</v>
       </c>
     </row>
     <row r="25" ht="16" customHeight="1">
-      <c r="A25" s="244" t="inlineStr">
+      <c r="A25" s="248" t="inlineStr">
         <is>
           <t>B09QVW7J24</t>
         </is>
@@ -22122,57 +22430,57 @@
           <t>Sweater Hangers (Blue)</t>
         </is>
       </c>
-      <c r="C25" s="260" t="n">
-        <v>0</v>
-      </c>
-      <c r="D25" s="246" t="n">
+      <c r="C25" s="264" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" s="250" t="n">
         <v>1</v>
       </c>
-      <c r="E25" s="245" t="n"/>
-      <c r="F25" s="245" t="n"/>
-      <c r="G25" s="245" t="n"/>
-      <c r="H25" s="245" t="n"/>
-      <c r="I25" s="249" t="n">
+      <c r="E25" s="249" t="n"/>
+      <c r="F25" s="249" t="n"/>
+      <c r="G25" s="249" t="n"/>
+      <c r="H25" s="249" t="n"/>
+      <c r="I25" s="253" t="n">
         <v>28</v>
       </c>
-      <c r="J25" s="262" t="n"/>
+      <c r="J25" s="266" t="n"/>
       <c r="K25" s="28" t="n"/>
     </row>
     <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="263" t="inlineStr">
+      <c r="A26" s="267" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C26" s="264">
+      <c r="C26" s="268">
         <f>SUM(C3:C25)</f>
         <v/>
       </c>
-      <c r="D26" s="264">
+      <c r="D26" s="268">
         <f>SUM(D3:D25)</f>
         <v/>
       </c>
-      <c r="E26" s="264">
+      <c r="E26" s="268">
         <f>SUM(E3:E25)</f>
         <v/>
       </c>
-      <c r="F26" s="264">
+      <c r="F26" s="268">
         <f>SUM(F3:F25)</f>
         <v/>
       </c>
-      <c r="G26" s="264">
+      <c r="G26" s="268">
         <f>SUM(G3:G25)</f>
         <v/>
       </c>
-      <c r="H26" s="264">
+      <c r="H26" s="268">
         <f>SUM(H3:H25)</f>
         <v/>
       </c>
-      <c r="I26" s="264">
+      <c r="I26" s="268">
         <f>SUM(I3:I25)</f>
         <v/>
       </c>
-      <c r="K26" s="264">
+      <c r="K26" s="268">
         <f>SUM(K3:K25)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
DBJ W6 (Mar 8-14): add weekly report data to dashboard
- W6 total: $4,350 sales, $154 spend, 3.5% TACOS
- Top performers: Wire Shelving ($1,557), Storage Cart ($1,400), Dryer Rack ($708)
- All weeks computed from CSV (no frozen weeks)

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dbj/DBJ_US_Feb-Mar_2026.xlsx
+++ b/dbj/DBJ_US_Feb-Mar_2026.xlsx
@@ -1786,7 +1786,7 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="11" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="B5" s="12" t="inlineStr">
@@ -1882,7 +1882,7 @@
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="27" t="inlineStr">
         <is>
-          <t>Storage Cart 10D</t>
+          <t>十層收納車</t>
         </is>
       </c>
       <c r="B6" s="28" t="inlineStr">
@@ -1978,7 +1978,7 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="11" t="inlineStr">
         <is>
-          <t>Laptop Stand A</t>
+          <t>筆電桌A款</t>
         </is>
       </c>
       <c r="B7" s="12" t="inlineStr">
@@ -2064,7 +2064,7 @@
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="27" t="inlineStr">
         <is>
-          <t>Dryer Rack</t>
+          <t>折疊曬衣架</t>
         </is>
       </c>
       <c r="B8" s="28" t="inlineStr">
@@ -2160,7 +2160,7 @@
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="11" t="inlineStr">
         <is>
-          <t>Laptop Stand B</t>
+          <t>筆電桌B款</t>
         </is>
       </c>
       <c r="B9" s="12" t="inlineStr">
@@ -2246,7 +2246,7 @@
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="27" t="inlineStr">
         <is>
-          <t>Sweater Hangers</t>
+          <t>毛衣防痕架</t>
         </is>
       </c>
       <c r="B10" s="28" t="inlineStr">
@@ -2342,7 +2342,7 @@
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="11" t="inlineStr">
         <is>
-          <t>Bathroom Storage</t>
+          <t>馬桶置物架</t>
         </is>
       </c>
       <c r="B11" s="12" t="inlineStr">
@@ -2430,7 +2430,7 @@
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="27" t="inlineStr">
         <is>
-          <t>Double Rail Rack</t>
+          <t>雙桿掛衣架</t>
         </is>
       </c>
       <c r="B12" s="28" t="inlineStr">
@@ -2518,7 +2518,7 @@
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="11" t="inlineStr">
         <is>
-          <t>3-Tier Cart</t>
+          <t>三層推車網</t>
         </is>
       </c>
       <c r="B13" s="12" t="inlineStr">
@@ -2610,7 +2610,7 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="27" t="inlineStr">
         <is>
-          <t>Padded Hangers</t>
+          <t>軟墊防滑架</t>
         </is>
       </c>
       <c r="B14" s="28" t="inlineStr">
@@ -2706,7 +2706,7 @@
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="11" t="inlineStr">
         <is>
-          <t>Laptop Stand C</t>
+          <t>筆電桌C款</t>
         </is>
       </c>
       <c r="B15" s="12" t="inlineStr">
@@ -2790,7 +2790,7 @@
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="27" t="inlineStr">
         <is>
-          <t>Shoe Rack</t>
+          <t>可伸縮鞋架</t>
         </is>
       </c>
       <c r="B16" s="28" t="inlineStr">
@@ -2874,7 +2874,7 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="11" t="inlineStr">
         <is>
-          <t>Broom Holder</t>
+          <t>壁掛拖把架</t>
         </is>
       </c>
       <c r="B17" s="12" t="inlineStr">
@@ -2970,7 +2970,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="27" t="inlineStr">
         <is>
-          <t>Shower Caddy</t>
+          <t>浴室收納架</t>
         </is>
       </c>
       <c r="B18" s="28" t="inlineStr">
@@ -3279,7 +3279,7 @@
     <row r="4" ht="16" customHeight="1">
       <c r="A4" s="47" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="B4" s="48" t="inlineStr">
@@ -3337,7 +3337,7 @@
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="54" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="B5" s="55" t="inlineStr">
@@ -3395,7 +3395,7 @@
     <row r="6" ht="16" customHeight="1">
       <c r="A6" s="61" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="B6" s="62" t="inlineStr">
@@ -3453,7 +3453,7 @@
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="68" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="B7" s="69" t="inlineStr">
@@ -3511,7 +3511,7 @@
     <row r="8" ht="16" customHeight="1">
       <c r="A8" s="75" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="B8" s="76" t="inlineStr">
@@ -3569,7 +3569,7 @@
     <row r="9" ht="16" customHeight="1">
       <c r="A9" s="82" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="B9" s="83" t="inlineStr">
@@ -3627,7 +3627,7 @@
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="89" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ↳ Wire Shelving Total</t>
+          <t xml:space="preserve">  ↳ 鐵線置物架 Total</t>
         </is>
       </c>
       <c r="B10" s="90" t="inlineStr">
@@ -3688,7 +3688,7 @@
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="47" t="inlineStr">
         <is>
-          <t>Storage Cart 10D</t>
+          <t>十層收納車</t>
         </is>
       </c>
       <c r="B11" s="48" t="inlineStr">
@@ -3746,7 +3746,7 @@
     <row r="12" ht="16" customHeight="1">
       <c r="A12" s="54" t="inlineStr">
         <is>
-          <t>Storage Cart 10D</t>
+          <t>十層收納車</t>
         </is>
       </c>
       <c r="B12" s="55" t="inlineStr">
@@ -3804,7 +3804,7 @@
     <row r="13" ht="16" customHeight="1">
       <c r="A13" s="61" t="inlineStr">
         <is>
-          <t>Storage Cart 10D</t>
+          <t>十層收納車</t>
         </is>
       </c>
       <c r="B13" s="62" t="inlineStr">
@@ -3862,7 +3862,7 @@
     <row r="14" ht="16" customHeight="1">
       <c r="A14" s="68" t="inlineStr">
         <is>
-          <t>Storage Cart 10D</t>
+          <t>十層收納車</t>
         </is>
       </c>
       <c r="B14" s="69" t="inlineStr">
@@ -3920,7 +3920,7 @@
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="75" t="inlineStr">
         <is>
-          <t>Storage Cart 10D</t>
+          <t>十層收納車</t>
         </is>
       </c>
       <c r="B15" s="76" t="inlineStr">
@@ -3978,7 +3978,7 @@
     <row r="16" ht="16" customHeight="1">
       <c r="A16" s="82" t="inlineStr">
         <is>
-          <t>Storage Cart 10D</t>
+          <t>十層收納車</t>
         </is>
       </c>
       <c r="B16" s="83" t="inlineStr">
@@ -4036,7 +4036,7 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="89" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ↳ Storage Cart 10D Total</t>
+          <t xml:space="preserve">  ↳ 十層收納車 Total</t>
         </is>
       </c>
       <c r="B17" s="90" t="inlineStr">
@@ -4097,7 +4097,7 @@
     <row r="18" ht="16" customHeight="1">
       <c r="A18" s="47" t="inlineStr">
         <is>
-          <t>Laptop Stand A</t>
+          <t>筆電桌A款</t>
         </is>
       </c>
       <c r="B18" s="48" t="inlineStr">
@@ -4149,7 +4149,7 @@
     <row r="19" ht="16" customHeight="1">
       <c r="A19" s="54" t="inlineStr">
         <is>
-          <t>Laptop Stand A</t>
+          <t>筆電桌A款</t>
         </is>
       </c>
       <c r="B19" s="55" t="inlineStr">
@@ -4203,7 +4203,7 @@
     <row r="20" ht="16" customHeight="1">
       <c r="A20" s="61" t="inlineStr">
         <is>
-          <t>Laptop Stand A</t>
+          <t>筆電桌A款</t>
         </is>
       </c>
       <c r="B20" s="62" t="inlineStr">
@@ -4255,7 +4255,7 @@
     <row r="21" ht="16" customHeight="1">
       <c r="A21" s="68" t="inlineStr">
         <is>
-          <t>Laptop Stand A</t>
+          <t>筆電桌A款</t>
         </is>
       </c>
       <c r="B21" s="69" t="inlineStr">
@@ -4309,7 +4309,7 @@
     <row r="22" ht="16" customHeight="1">
       <c r="A22" s="75" t="inlineStr">
         <is>
-          <t>Laptop Stand A</t>
+          <t>筆電桌A款</t>
         </is>
       </c>
       <c r="B22" s="76" t="inlineStr">
@@ -4361,7 +4361,7 @@
     <row r="23" ht="16" customHeight="1">
       <c r="A23" s="82" t="inlineStr">
         <is>
-          <t>Laptop Stand A</t>
+          <t>筆電桌A款</t>
         </is>
       </c>
       <c r="B23" s="83" t="inlineStr">
@@ -4413,7 +4413,7 @@
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="89" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ↳ Laptop Stand A Total</t>
+          <t xml:space="preserve">  ↳ 筆電桌A款 Total</t>
         </is>
       </c>
       <c r="B24" s="90" t="inlineStr">
@@ -4474,7 +4474,7 @@
     <row r="25" ht="16" customHeight="1">
       <c r="A25" s="47" t="inlineStr">
         <is>
-          <t>Dryer Rack</t>
+          <t>折疊曬衣架</t>
         </is>
       </c>
       <c r="B25" s="48" t="inlineStr">
@@ -4532,7 +4532,7 @@
     <row r="26" ht="16" customHeight="1">
       <c r="A26" s="54" t="inlineStr">
         <is>
-          <t>Dryer Rack</t>
+          <t>折疊曬衣架</t>
         </is>
       </c>
       <c r="B26" s="55" t="inlineStr">
@@ -4590,7 +4590,7 @@
     <row r="27" ht="16" customHeight="1">
       <c r="A27" s="61" t="inlineStr">
         <is>
-          <t>Dryer Rack</t>
+          <t>折疊曬衣架</t>
         </is>
       </c>
       <c r="B27" s="62" t="inlineStr">
@@ -4648,7 +4648,7 @@
     <row r="28" ht="16" customHeight="1">
       <c r="A28" s="68" t="inlineStr">
         <is>
-          <t>Dryer Rack</t>
+          <t>折疊曬衣架</t>
         </is>
       </c>
       <c r="B28" s="69" t="inlineStr">
@@ -4706,7 +4706,7 @@
     <row r="29" ht="16" customHeight="1">
       <c r="A29" s="75" t="inlineStr">
         <is>
-          <t>Dryer Rack</t>
+          <t>折疊曬衣架</t>
         </is>
       </c>
       <c r="B29" s="76" t="inlineStr">
@@ -4764,7 +4764,7 @@
     <row r="30" ht="16" customHeight="1">
       <c r="A30" s="82" t="inlineStr">
         <is>
-          <t>Dryer Rack</t>
+          <t>折疊曬衣架</t>
         </is>
       </c>
       <c r="B30" s="83" t="inlineStr">
@@ -4822,7 +4822,7 @@
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="89" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ↳ Dryer Rack Total</t>
+          <t xml:space="preserve">  ↳ 折疊曬衣架 Total</t>
         </is>
       </c>
       <c r="B31" s="90" t="inlineStr">
@@ -4883,7 +4883,7 @@
     <row r="32" ht="16" customHeight="1">
       <c r="A32" s="47" t="inlineStr">
         <is>
-          <t>Laptop Stand B</t>
+          <t>筆電桌B款</t>
         </is>
       </c>
       <c r="B32" s="48" t="inlineStr">
@@ -4935,7 +4935,7 @@
     <row r="33" ht="16" customHeight="1">
       <c r="A33" s="54" t="inlineStr">
         <is>
-          <t>Laptop Stand B</t>
+          <t>筆電桌B款</t>
         </is>
       </c>
       <c r="B33" s="55" t="inlineStr">
@@ -4989,7 +4989,7 @@
     <row r="34" ht="16" customHeight="1">
       <c r="A34" s="61" t="inlineStr">
         <is>
-          <t>Laptop Stand B</t>
+          <t>筆電桌B款</t>
         </is>
       </c>
       <c r="B34" s="62" t="inlineStr">
@@ -5043,7 +5043,7 @@
     <row r="35" ht="16" customHeight="1">
       <c r="A35" s="68" t="inlineStr">
         <is>
-          <t>Laptop Stand B</t>
+          <t>筆電桌B款</t>
         </is>
       </c>
       <c r="B35" s="69" t="inlineStr">
@@ -5095,7 +5095,7 @@
     <row r="36" ht="16" customHeight="1">
       <c r="A36" s="75" t="inlineStr">
         <is>
-          <t>Laptop Stand B</t>
+          <t>筆電桌B款</t>
         </is>
       </c>
       <c r="B36" s="76" t="inlineStr">
@@ -5147,7 +5147,7 @@
     <row r="37" ht="16" customHeight="1">
       <c r="A37" s="82" t="inlineStr">
         <is>
-          <t>Laptop Stand B</t>
+          <t>筆電桌B款</t>
         </is>
       </c>
       <c r="B37" s="83" t="inlineStr">
@@ -5199,7 +5199,7 @@
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="89" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ↳ Laptop Stand B Total</t>
+          <t xml:space="preserve">  ↳ 筆電桌B款 Total</t>
         </is>
       </c>
       <c r="B38" s="90" t="inlineStr">
@@ -5260,7 +5260,7 @@
     <row r="39" ht="16" customHeight="1">
       <c r="A39" s="47" t="inlineStr">
         <is>
-          <t>Sweater Hangers</t>
+          <t>毛衣防痕架</t>
         </is>
       </c>
       <c r="B39" s="48" t="inlineStr">
@@ -5318,7 +5318,7 @@
     <row r="40" ht="16" customHeight="1">
       <c r="A40" s="54" t="inlineStr">
         <is>
-          <t>Sweater Hangers</t>
+          <t>毛衣防痕架</t>
         </is>
       </c>
       <c r="B40" s="55" t="inlineStr">
@@ -5376,7 +5376,7 @@
     <row r="41" ht="16" customHeight="1">
       <c r="A41" s="61" t="inlineStr">
         <is>
-          <t>Sweater Hangers</t>
+          <t>毛衣防痕架</t>
         </is>
       </c>
       <c r="B41" s="62" t="inlineStr">
@@ -5434,7 +5434,7 @@
     <row r="42" ht="16" customHeight="1">
       <c r="A42" s="68" t="inlineStr">
         <is>
-          <t>Sweater Hangers</t>
+          <t>毛衣防痕架</t>
         </is>
       </c>
       <c r="B42" s="69" t="inlineStr">
@@ -5492,7 +5492,7 @@
     <row r="43" ht="16" customHeight="1">
       <c r="A43" s="75" t="inlineStr">
         <is>
-          <t>Sweater Hangers</t>
+          <t>毛衣防痕架</t>
         </is>
       </c>
       <c r="B43" s="76" t="inlineStr">
@@ -5550,7 +5550,7 @@
     <row r="44" ht="16" customHeight="1">
       <c r="A44" s="82" t="inlineStr">
         <is>
-          <t>Sweater Hangers</t>
+          <t>毛衣防痕架</t>
         </is>
       </c>
       <c r="B44" s="83" t="inlineStr">
@@ -5608,7 +5608,7 @@
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="89" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ↳ Sweater Hangers Total</t>
+          <t xml:space="preserve">  ↳ 毛衣防痕架 Total</t>
         </is>
       </c>
       <c r="B45" s="90" t="inlineStr">
@@ -5669,7 +5669,7 @@
     <row r="46" ht="16" customHeight="1">
       <c r="A46" s="47" t="inlineStr">
         <is>
-          <t>Bathroom Storage</t>
+          <t>馬桶置物架</t>
         </is>
       </c>
       <c r="B46" s="48" t="inlineStr">
@@ -5721,7 +5721,7 @@
     <row r="47" ht="16" customHeight="1">
       <c r="A47" s="54" t="inlineStr">
         <is>
-          <t>Bathroom Storage</t>
+          <t>馬桶置物架</t>
         </is>
       </c>
       <c r="B47" s="55" t="inlineStr">
@@ -5775,7 +5775,7 @@
     <row r="48" ht="16" customHeight="1">
       <c r="A48" s="61" t="inlineStr">
         <is>
-          <t>Bathroom Storage</t>
+          <t>馬桶置物架</t>
         </is>
       </c>
       <c r="B48" s="62" t="inlineStr">
@@ -5829,7 +5829,7 @@
     <row r="49" ht="16" customHeight="1">
       <c r="A49" s="68" t="inlineStr">
         <is>
-          <t>Bathroom Storage</t>
+          <t>馬桶置物架</t>
         </is>
       </c>
       <c r="B49" s="69" t="inlineStr">
@@ -5883,7 +5883,7 @@
     <row r="50" ht="16" customHeight="1">
       <c r="A50" s="75" t="inlineStr">
         <is>
-          <t>Bathroom Storage</t>
+          <t>馬桶置物架</t>
         </is>
       </c>
       <c r="B50" s="76" t="inlineStr">
@@ -5935,7 +5935,7 @@
     <row r="51" ht="16" customHeight="1">
       <c r="A51" s="82" t="inlineStr">
         <is>
-          <t>Bathroom Storage</t>
+          <t>馬桶置物架</t>
         </is>
       </c>
       <c r="B51" s="83" t="inlineStr">
@@ -5987,7 +5987,7 @@
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="89" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ↳ Bathroom Storage Total</t>
+          <t xml:space="preserve">  ↳ 馬桶置物架 Total</t>
         </is>
       </c>
       <c r="B52" s="90" t="inlineStr">
@@ -6048,7 +6048,7 @@
     <row r="53" ht="16" customHeight="1">
       <c r="A53" s="47" t="inlineStr">
         <is>
-          <t>Double Rail Rack</t>
+          <t>雙桿掛衣架</t>
         </is>
       </c>
       <c r="B53" s="48" t="inlineStr">
@@ -6102,7 +6102,7 @@
     <row r="54" ht="16" customHeight="1">
       <c r="A54" s="54" t="inlineStr">
         <is>
-          <t>Double Rail Rack</t>
+          <t>雙桿掛衣架</t>
         </is>
       </c>
       <c r="B54" s="55" t="inlineStr">
@@ -6156,7 +6156,7 @@
     <row r="55" ht="16" customHeight="1">
       <c r="A55" s="61" t="inlineStr">
         <is>
-          <t>Double Rail Rack</t>
+          <t>雙桿掛衣架</t>
         </is>
       </c>
       <c r="B55" s="62" t="inlineStr">
@@ -6208,7 +6208,7 @@
     <row r="56" ht="16" customHeight="1">
       <c r="A56" s="68" t="inlineStr">
         <is>
-          <t>Double Rail Rack</t>
+          <t>雙桿掛衣架</t>
         </is>
       </c>
       <c r="B56" s="69" t="inlineStr">
@@ -6262,7 +6262,7 @@
     <row r="57" ht="16" customHeight="1">
       <c r="A57" s="75" t="inlineStr">
         <is>
-          <t>Double Rail Rack</t>
+          <t>雙桿掛衣架</t>
         </is>
       </c>
       <c r="B57" s="76" t="inlineStr">
@@ -6314,7 +6314,7 @@
     <row r="58" ht="16" customHeight="1">
       <c r="A58" s="82" t="inlineStr">
         <is>
-          <t>Double Rail Rack</t>
+          <t>雙桿掛衣架</t>
         </is>
       </c>
       <c r="B58" s="83" t="inlineStr">
@@ -6366,7 +6366,7 @@
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="89" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ↳ Double Rail Rack Total</t>
+          <t xml:space="preserve">  ↳ 雙桿掛衣架 Total</t>
         </is>
       </c>
       <c r="B59" s="90" t="inlineStr">
@@ -6427,7 +6427,7 @@
     <row r="60" ht="16" customHeight="1">
       <c r="A60" s="47" t="inlineStr">
         <is>
-          <t>3-Tier Cart</t>
+          <t>三層推車網</t>
         </is>
       </c>
       <c r="B60" s="48" t="inlineStr">
@@ -6481,7 +6481,7 @@
     <row r="61" ht="16" customHeight="1">
       <c r="A61" s="54" t="inlineStr">
         <is>
-          <t>3-Tier Cart</t>
+          <t>三層推車網</t>
         </is>
       </c>
       <c r="B61" s="55" t="inlineStr">
@@ -6533,7 +6533,7 @@
     <row r="62" ht="16" customHeight="1">
       <c r="A62" s="61" t="inlineStr">
         <is>
-          <t>3-Tier Cart</t>
+          <t>三層推車網</t>
         </is>
       </c>
       <c r="B62" s="62" t="inlineStr">
@@ -6585,7 +6585,7 @@
     <row r="63" ht="16" customHeight="1">
       <c r="A63" s="68" t="inlineStr">
         <is>
-          <t>3-Tier Cart</t>
+          <t>三層推車網</t>
         </is>
       </c>
       <c r="B63" s="69" t="inlineStr">
@@ -6643,7 +6643,7 @@
     <row r="64" ht="16" customHeight="1">
       <c r="A64" s="75" t="inlineStr">
         <is>
-          <t>3-Tier Cart</t>
+          <t>三層推車網</t>
         </is>
       </c>
       <c r="B64" s="76" t="inlineStr">
@@ -6701,7 +6701,7 @@
     <row r="65" ht="16" customHeight="1">
       <c r="A65" s="82" t="inlineStr">
         <is>
-          <t>3-Tier Cart</t>
+          <t>三層推車網</t>
         </is>
       </c>
       <c r="B65" s="83" t="inlineStr">
@@ -6759,7 +6759,7 @@
     <row r="66" ht="18" customHeight="1">
       <c r="A66" s="89" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ↳ 3-Tier Cart Total</t>
+          <t xml:space="preserve">  ↳ 三層推車網 Total</t>
         </is>
       </c>
       <c r="B66" s="90" t="inlineStr">
@@ -6820,7 +6820,7 @@
     <row r="67" ht="16" customHeight="1">
       <c r="A67" s="47" t="inlineStr">
         <is>
-          <t>Padded Hangers</t>
+          <t>軟墊防滑架</t>
         </is>
       </c>
       <c r="B67" s="48" t="inlineStr">
@@ -6878,7 +6878,7 @@
     <row r="68" ht="16" customHeight="1">
       <c r="A68" s="54" t="inlineStr">
         <is>
-          <t>Padded Hangers</t>
+          <t>軟墊防滑架</t>
         </is>
       </c>
       <c r="B68" s="55" t="inlineStr">
@@ -6936,7 +6936,7 @@
     <row r="69" ht="16" customHeight="1">
       <c r="A69" s="61" t="inlineStr">
         <is>
-          <t>Padded Hangers</t>
+          <t>軟墊防滑架</t>
         </is>
       </c>
       <c r="B69" s="62" t="inlineStr">
@@ -6994,7 +6994,7 @@
     <row r="70" ht="16" customHeight="1">
       <c r="A70" s="68" t="inlineStr">
         <is>
-          <t>Padded Hangers</t>
+          <t>軟墊防滑架</t>
         </is>
       </c>
       <c r="B70" s="69" t="inlineStr">
@@ -7052,7 +7052,7 @@
     <row r="71" ht="16" customHeight="1">
       <c r="A71" s="75" t="inlineStr">
         <is>
-          <t>Padded Hangers</t>
+          <t>軟墊防滑架</t>
         </is>
       </c>
       <c r="B71" s="76" t="inlineStr">
@@ -7110,7 +7110,7 @@
     <row r="72" ht="16" customHeight="1">
       <c r="A72" s="82" t="inlineStr">
         <is>
-          <t>Padded Hangers</t>
+          <t>軟墊防滑架</t>
         </is>
       </c>
       <c r="B72" s="83" t="inlineStr">
@@ -7168,7 +7168,7 @@
     <row r="73" ht="18" customHeight="1">
       <c r="A73" s="89" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ↳ Padded Hangers Total</t>
+          <t xml:space="preserve">  ↳ 軟墊防滑架 Total</t>
         </is>
       </c>
       <c r="B73" s="90" t="inlineStr">
@@ -7229,7 +7229,7 @@
     <row r="74" ht="16" customHeight="1">
       <c r="A74" s="47" t="inlineStr">
         <is>
-          <t>Laptop Stand C</t>
+          <t>筆電桌C款</t>
         </is>
       </c>
       <c r="B74" s="48" t="inlineStr">
@@ -7281,7 +7281,7 @@
     <row r="75" ht="16" customHeight="1">
       <c r="A75" s="54" t="inlineStr">
         <is>
-          <t>Laptop Stand C</t>
+          <t>筆電桌C款</t>
         </is>
       </c>
       <c r="B75" s="55" t="inlineStr">
@@ -7335,7 +7335,7 @@
     <row r="76" ht="16" customHeight="1">
       <c r="A76" s="61" t="inlineStr">
         <is>
-          <t>Laptop Stand C</t>
+          <t>筆電桌C款</t>
         </is>
       </c>
       <c r="B76" s="62" t="inlineStr">
@@ -7387,7 +7387,7 @@
     <row r="77" ht="16" customHeight="1">
       <c r="A77" s="68" t="inlineStr">
         <is>
-          <t>Laptop Stand C</t>
+          <t>筆電桌C款</t>
         </is>
       </c>
       <c r="B77" s="69" t="inlineStr">
@@ -7439,7 +7439,7 @@
     <row r="78" ht="16" customHeight="1">
       <c r="A78" s="75" t="inlineStr">
         <is>
-          <t>Laptop Stand C</t>
+          <t>筆電桌C款</t>
         </is>
       </c>
       <c r="B78" s="76" t="inlineStr">
@@ -7491,7 +7491,7 @@
     <row r="79" ht="16" customHeight="1">
       <c r="A79" s="82" t="inlineStr">
         <is>
-          <t>Laptop Stand C</t>
+          <t>筆電桌C款</t>
         </is>
       </c>
       <c r="B79" s="83" t="inlineStr">
@@ -7543,7 +7543,7 @@
     <row r="80" ht="18" customHeight="1">
       <c r="A80" s="89" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ↳ Laptop Stand C Total</t>
+          <t xml:space="preserve">  ↳ 筆電桌C款 Total</t>
         </is>
       </c>
       <c r="B80" s="90" t="inlineStr">
@@ -7604,7 +7604,7 @@
     <row r="81" ht="16" customHeight="1">
       <c r="A81" s="47" t="inlineStr">
         <is>
-          <t>Shoe Rack</t>
+          <t>可伸縮鞋架</t>
         </is>
       </c>
       <c r="B81" s="48" t="inlineStr">
@@ -7656,7 +7656,7 @@
     <row r="82" ht="16" customHeight="1">
       <c r="A82" s="54" t="inlineStr">
         <is>
-          <t>Shoe Rack</t>
+          <t>可伸縮鞋架</t>
         </is>
       </c>
       <c r="B82" s="55" t="inlineStr">
@@ -7710,7 +7710,7 @@
     <row r="83" ht="16" customHeight="1">
       <c r="A83" s="61" t="inlineStr">
         <is>
-          <t>Shoe Rack</t>
+          <t>可伸縮鞋架</t>
         </is>
       </c>
       <c r="B83" s="62" t="inlineStr">
@@ -7762,7 +7762,7 @@
     <row r="84" ht="16" customHeight="1">
       <c r="A84" s="68" t="inlineStr">
         <is>
-          <t>Shoe Rack</t>
+          <t>可伸縮鞋架</t>
         </is>
       </c>
       <c r="B84" s="69" t="inlineStr">
@@ -7814,7 +7814,7 @@
     <row r="85" ht="16" customHeight="1">
       <c r="A85" s="75" t="inlineStr">
         <is>
-          <t>Shoe Rack</t>
+          <t>可伸縮鞋架</t>
         </is>
       </c>
       <c r="B85" s="76" t="inlineStr">
@@ -7866,7 +7866,7 @@
     <row r="86" ht="16" customHeight="1">
       <c r="A86" s="82" t="inlineStr">
         <is>
-          <t>Shoe Rack</t>
+          <t>可伸縮鞋架</t>
         </is>
       </c>
       <c r="B86" s="83" t="inlineStr">
@@ -7918,7 +7918,7 @@
     <row r="87" ht="18" customHeight="1">
       <c r="A87" s="89" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ↳ Shoe Rack Total</t>
+          <t xml:space="preserve">  ↳ 可伸縮鞋架 Total</t>
         </is>
       </c>
       <c r="B87" s="90" t="inlineStr">
@@ -7979,7 +7979,7 @@
     <row r="88" ht="16" customHeight="1">
       <c r="A88" s="47" t="inlineStr">
         <is>
-          <t>Broom Holder</t>
+          <t>壁掛拖把架</t>
         </is>
       </c>
       <c r="B88" s="48" t="inlineStr">
@@ -8037,7 +8037,7 @@
     <row r="89" ht="16" customHeight="1">
       <c r="A89" s="54" t="inlineStr">
         <is>
-          <t>Broom Holder</t>
+          <t>壁掛拖把架</t>
         </is>
       </c>
       <c r="B89" s="55" t="inlineStr">
@@ -8095,7 +8095,7 @@
     <row r="90" ht="16" customHeight="1">
       <c r="A90" s="61" t="inlineStr">
         <is>
-          <t>Broom Holder</t>
+          <t>壁掛拖把架</t>
         </is>
       </c>
       <c r="B90" s="62" t="inlineStr">
@@ -8153,7 +8153,7 @@
     <row r="91" ht="16" customHeight="1">
       <c r="A91" s="68" t="inlineStr">
         <is>
-          <t>Broom Holder</t>
+          <t>壁掛拖把架</t>
         </is>
       </c>
       <c r="B91" s="69" t="inlineStr">
@@ -8211,7 +8211,7 @@
     <row r="92" ht="16" customHeight="1">
       <c r="A92" s="75" t="inlineStr">
         <is>
-          <t>Broom Holder</t>
+          <t>壁掛拖把架</t>
         </is>
       </c>
       <c r="B92" s="76" t="inlineStr">
@@ -8269,7 +8269,7 @@
     <row r="93" ht="16" customHeight="1">
       <c r="A93" s="82" t="inlineStr">
         <is>
-          <t>Broom Holder</t>
+          <t>壁掛拖把架</t>
         </is>
       </c>
       <c r="B93" s="83" t="inlineStr">
@@ -8327,7 +8327,7 @@
     <row r="94" ht="18" customHeight="1">
       <c r="A94" s="89" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ↳ Broom Holder Total</t>
+          <t xml:space="preserve">  ↳ 壁掛拖把架 Total</t>
         </is>
       </c>
       <c r="B94" s="90" t="inlineStr">
@@ -8388,7 +8388,7 @@
     <row r="95" ht="16" customHeight="1">
       <c r="A95" s="47" t="inlineStr">
         <is>
-          <t>Shower Caddy</t>
+          <t>浴室收納架</t>
         </is>
       </c>
       <c r="B95" s="48" t="inlineStr">
@@ -8440,7 +8440,7 @@
     <row r="96" ht="16" customHeight="1">
       <c r="A96" s="54" t="inlineStr">
         <is>
-          <t>Shower Caddy</t>
+          <t>浴室收納架</t>
         </is>
       </c>
       <c r="B96" s="55" t="inlineStr">
@@ -8492,7 +8492,7 @@
     <row r="97" ht="16" customHeight="1">
       <c r="A97" s="61" t="inlineStr">
         <is>
-          <t>Shower Caddy</t>
+          <t>浴室收納架</t>
         </is>
       </c>
       <c r="B97" s="62" t="inlineStr">
@@ -8544,7 +8544,7 @@
     <row r="98" ht="16" customHeight="1">
       <c r="A98" s="68" t="inlineStr">
         <is>
-          <t>Shower Caddy</t>
+          <t>浴室收納架</t>
         </is>
       </c>
       <c r="B98" s="69" t="inlineStr">
@@ -8596,7 +8596,7 @@
     <row r="99" ht="16" customHeight="1">
       <c r="A99" s="75" t="inlineStr">
         <is>
-          <t>Shower Caddy</t>
+          <t>浴室收納架</t>
         </is>
       </c>
       <c r="B99" s="76" t="inlineStr">
@@ -8650,7 +8650,7 @@
     <row r="100" ht="16" customHeight="1">
       <c r="A100" s="82" t="inlineStr">
         <is>
-          <t>Shower Caddy</t>
+          <t>浴室收納架</t>
         </is>
       </c>
       <c r="B100" s="83" t="inlineStr">
@@ -8702,7 +8702,7 @@
     <row r="101" ht="18" customHeight="1">
       <c r="A101" s="89" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ↳ Shower Caddy Total</t>
+          <t xml:space="preserve">  ↳ 浴室收納架 Total</t>
         </is>
       </c>
       <c r="B101" s="90" t="inlineStr">
@@ -8871,7 +8871,7 @@
     <row r="4" ht="16" customHeight="1">
       <c r="A4" s="112" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="B4" s="48" t="inlineStr">
@@ -8881,7 +8881,7 @@
       </c>
       <c r="C4" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 Tier Wire Shelving Unit Storage Rack, </t>
+          <t>3層鉻24小</t>
         </is>
       </c>
       <c r="D4" s="49" t="inlineStr">
@@ -8920,7 +8920,7 @@
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="115" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="B5" s="55" t="inlineStr">
@@ -8930,7 +8930,7 @@
       </c>
       <c r="C5" s="54" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 Tier Wire Shelving Unit Storage Rack, </t>
+          <t>3層鉻24小</t>
         </is>
       </c>
       <c r="D5" s="56" t="inlineStr">
@@ -8969,7 +8969,7 @@
     <row r="6" ht="16" customHeight="1">
       <c r="A6" s="118" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="B6" s="62" t="inlineStr">
@@ -8979,7 +8979,7 @@
       </c>
       <c r="C6" s="61" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 Tier Wire Shelving Unit Storage Rack, </t>
+          <t>3層鉻24小</t>
         </is>
       </c>
       <c r="D6" s="63" t="inlineStr">
@@ -9018,7 +9018,7 @@
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="121" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="B7" s="69" t="inlineStr">
@@ -9028,7 +9028,7 @@
       </c>
       <c r="C7" s="68" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 Tier Wire Shelving Unit Storage Rack, </t>
+          <t>3層鉻24小</t>
         </is>
       </c>
       <c r="D7" s="70" t="inlineStr">
@@ -9067,7 +9067,7 @@
     <row r="8" ht="16" customHeight="1">
       <c r="A8" s="124" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="B8" s="76" t="inlineStr">
@@ -9077,7 +9077,7 @@
       </c>
       <c r="C8" s="75" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 Tier Wire Shelving Unit Storage Rack, </t>
+          <t>3層鉻24小</t>
         </is>
       </c>
       <c r="D8" s="77" t="inlineStr">
@@ -9116,7 +9116,7 @@
     <row r="9" ht="16" customHeight="1">
       <c r="A9" s="127" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="B9" s="83" t="inlineStr">
@@ -9126,7 +9126,7 @@
       </c>
       <c r="C9" s="82" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 Tier Wire Shelving Unit Storage Rack, </t>
+          <t>3層鉻24小</t>
         </is>
       </c>
       <c r="D9" s="84" t="inlineStr">
@@ -9165,7 +9165,7 @@
     <row r="10" ht="16" customHeight="1">
       <c r="A10" s="112" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="B10" s="48" t="inlineStr">
@@ -9175,7 +9175,7 @@
       </c>
       <c r="C10" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 Tier Wire Shelving Unit Storage Rack, </t>
+          <t>3層黑24小</t>
         </is>
       </c>
       <c r="D10" s="49" t="inlineStr">
@@ -9214,7 +9214,7 @@
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="115" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="B11" s="55" t="inlineStr">
@@ -9224,7 +9224,7 @@
       </c>
       <c r="C11" s="54" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 Tier Wire Shelving Unit Storage Rack, </t>
+          <t>3層黑24小</t>
         </is>
       </c>
       <c r="D11" s="56" t="inlineStr">
@@ -9263,7 +9263,7 @@
     <row r="12" ht="16" customHeight="1">
       <c r="A12" s="118" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="B12" s="62" t="inlineStr">
@@ -9273,7 +9273,7 @@
       </c>
       <c r="C12" s="61" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 Tier Wire Shelving Unit Storage Rack, </t>
+          <t>3層黑24小</t>
         </is>
       </c>
       <c r="D12" s="63" t="inlineStr">
@@ -9312,7 +9312,7 @@
     <row r="13" ht="16" customHeight="1">
       <c r="A13" s="121" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="B13" s="69" t="inlineStr">
@@ -9322,7 +9322,7 @@
       </c>
       <c r="C13" s="68" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 Tier Wire Shelving Unit Storage Rack, </t>
+          <t>3層黑24小</t>
         </is>
       </c>
       <c r="D13" s="70" t="inlineStr">
@@ -9361,7 +9361,7 @@
     <row r="14" ht="16" customHeight="1">
       <c r="A14" s="124" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="B14" s="76" t="inlineStr">
@@ -9371,7 +9371,7 @@
       </c>
       <c r="C14" s="75" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 Tier Wire Shelving Unit Storage Rack, </t>
+          <t>3層黑24小</t>
         </is>
       </c>
       <c r="D14" s="77" t="inlineStr">
@@ -9410,7 +9410,7 @@
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="127" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="B15" s="83" t="inlineStr">
@@ -9420,7 +9420,7 @@
       </c>
       <c r="C15" s="82" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 Tier Wire Shelving Unit Storage Rack, </t>
+          <t>3層黑24小</t>
         </is>
       </c>
       <c r="D15" s="84" t="inlineStr">
@@ -9459,7 +9459,7 @@
     <row r="16" ht="16" customHeight="1">
       <c r="A16" s="112" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="B16" s="48" t="inlineStr">
@@ -9469,7 +9469,7 @@
       </c>
       <c r="C16" s="47" t="inlineStr">
         <is>
-          <t>Heavy Duty 4 Tier Wire Shelving Unit Sto</t>
+          <t>4層鉻30大</t>
         </is>
       </c>
       <c r="D16" s="49" t="inlineStr">
@@ -9508,7 +9508,7 @@
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="115" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="B17" s="55" t="inlineStr">
@@ -9518,7 +9518,7 @@
       </c>
       <c r="C17" s="54" t="inlineStr">
         <is>
-          <t>Heavy Duty 4 Tier Wire Shelving Unit Sto</t>
+          <t>4層鉻30大</t>
         </is>
       </c>
       <c r="D17" s="56" t="inlineStr">
@@ -9557,7 +9557,7 @@
     <row r="18" ht="16" customHeight="1">
       <c r="A18" s="118" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="B18" s="62" t="inlineStr">
@@ -9567,7 +9567,7 @@
       </c>
       <c r="C18" s="61" t="inlineStr">
         <is>
-          <t>Heavy Duty 4 Tier Wire Shelving Unit Sto</t>
+          <t>4層鉻30大</t>
         </is>
       </c>
       <c r="D18" s="63" t="inlineStr">
@@ -9606,7 +9606,7 @@
     <row r="19" ht="16" customHeight="1">
       <c r="A19" s="121" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="B19" s="69" t="inlineStr">
@@ -9616,7 +9616,7 @@
       </c>
       <c r="C19" s="68" t="inlineStr">
         <is>
-          <t>Heavy Duty 4 Tier Wire Shelving Unit Sto</t>
+          <t>4層鉻30大</t>
         </is>
       </c>
       <c r="D19" s="70" t="inlineStr">
@@ -9655,7 +9655,7 @@
     <row r="20" ht="16" customHeight="1">
       <c r="A20" s="124" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="B20" s="76" t="inlineStr">
@@ -9665,7 +9665,7 @@
       </c>
       <c r="C20" s="75" t="inlineStr">
         <is>
-          <t>Heavy Duty 4 Tier Wire Shelving Unit Sto</t>
+          <t>4層鉻30大</t>
         </is>
       </c>
       <c r="D20" s="77" t="inlineStr">
@@ -9704,7 +9704,7 @@
     <row r="21" ht="16" customHeight="1">
       <c r="A21" s="127" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="B21" s="83" t="inlineStr">
@@ -9714,7 +9714,7 @@
       </c>
       <c r="C21" s="82" t="inlineStr">
         <is>
-          <t>Heavy Duty 4 Tier Wire Shelving Unit Sto</t>
+          <t>4層鉻30大</t>
         </is>
       </c>
       <c r="D21" s="84" t="inlineStr">
@@ -9749,7 +9749,7 @@
     <row r="22" ht="16" customHeight="1">
       <c r="A22" s="112" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="B22" s="48" t="inlineStr">
@@ -9759,7 +9759,7 @@
       </c>
       <c r="C22" s="47" t="inlineStr">
         <is>
-          <t>Displays By Jack 4 Tier Wire Shelving Un</t>
+          <t>4層黑30中</t>
         </is>
       </c>
       <c r="D22" s="49" t="inlineStr">
@@ -9798,7 +9798,7 @@
     <row r="23" ht="16" customHeight="1">
       <c r="A23" s="115" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="B23" s="55" t="inlineStr">
@@ -9808,7 +9808,7 @@
       </c>
       <c r="C23" s="54" t="inlineStr">
         <is>
-          <t>Displays By Jack 4 Tier Wire Shelving Un</t>
+          <t>4層黑30中</t>
         </is>
       </c>
       <c r="D23" s="56" t="inlineStr">
@@ -9847,7 +9847,7 @@
     <row r="24" ht="16" customHeight="1">
       <c r="A24" s="118" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="B24" s="62" t="inlineStr">
@@ -9857,7 +9857,7 @@
       </c>
       <c r="C24" s="61" t="inlineStr">
         <is>
-          <t>Displays By Jack 4 Tier Wire Shelving Un</t>
+          <t>4層黑30中</t>
         </is>
       </c>
       <c r="D24" s="63" t="inlineStr">
@@ -9896,7 +9896,7 @@
     <row r="25" ht="16" customHeight="1">
       <c r="A25" s="121" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="B25" s="69" t="inlineStr">
@@ -9906,7 +9906,7 @@
       </c>
       <c r="C25" s="68" t="inlineStr">
         <is>
-          <t>Displays By Jack 4 Tier Wire Shelving Un</t>
+          <t>4層黑30中</t>
         </is>
       </c>
       <c r="D25" s="70" t="inlineStr">
@@ -9945,7 +9945,7 @@
     <row r="26" ht="16" customHeight="1">
       <c r="A26" s="124" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="B26" s="76" t="inlineStr">
@@ -9955,7 +9955,7 @@
       </c>
       <c r="C26" s="75" t="inlineStr">
         <is>
-          <t>Displays By Jack 4 Tier Wire Shelving Un</t>
+          <t>4層黑30中</t>
         </is>
       </c>
       <c r="D26" s="77" t="inlineStr">
@@ -9994,7 +9994,7 @@
     <row r="27" ht="16" customHeight="1">
       <c r="A27" s="127" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="B27" s="83" t="inlineStr">
@@ -10004,7 +10004,7 @@
       </c>
       <c r="C27" s="82" t="inlineStr">
         <is>
-          <t>Displays By Jack 4 Tier Wire Shelving Un</t>
+          <t>4層黑30中</t>
         </is>
       </c>
       <c r="D27" s="84" t="inlineStr">
@@ -10041,7 +10041,7 @@
     <row r="28" ht="16" customHeight="1">
       <c r="A28" s="112" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="B28" s="48" t="inlineStr">
@@ -10051,7 +10051,7 @@
       </c>
       <c r="C28" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">5 Tier Wire Shelving Unit Storage Rack, </t>
+          <t>5層黑30高</t>
         </is>
       </c>
       <c r="D28" s="49" t="inlineStr">
@@ -10090,7 +10090,7 @@
     <row r="29" ht="16" customHeight="1">
       <c r="A29" s="115" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="B29" s="55" t="inlineStr">
@@ -10100,7 +10100,7 @@
       </c>
       <c r="C29" s="54" t="inlineStr">
         <is>
-          <t xml:space="preserve">5 Tier Wire Shelving Unit Storage Rack, </t>
+          <t>5層黑30高</t>
         </is>
       </c>
       <c r="D29" s="56" t="inlineStr">
@@ -10139,7 +10139,7 @@
     <row r="30" ht="16" customHeight="1">
       <c r="A30" s="118" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="B30" s="62" t="inlineStr">
@@ -10149,7 +10149,7 @@
       </c>
       <c r="C30" s="61" t="inlineStr">
         <is>
-          <t xml:space="preserve">5 Tier Wire Shelving Unit Storage Rack, </t>
+          <t>5層黑30高</t>
         </is>
       </c>
       <c r="D30" s="63" t="inlineStr">
@@ -10188,7 +10188,7 @@
     <row r="31" ht="16" customHeight="1">
       <c r="A31" s="121" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="B31" s="69" t="inlineStr">
@@ -10198,7 +10198,7 @@
       </c>
       <c r="C31" s="68" t="inlineStr">
         <is>
-          <t xml:space="preserve">5 Tier Wire Shelving Unit Storage Rack, </t>
+          <t>5層黑30高</t>
         </is>
       </c>
       <c r="D31" s="70" t="inlineStr">
@@ -10237,7 +10237,7 @@
     <row r="32" ht="16" customHeight="1">
       <c r="A32" s="124" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="B32" s="76" t="inlineStr">
@@ -10247,7 +10247,7 @@
       </c>
       <c r="C32" s="75" t="inlineStr">
         <is>
-          <t xml:space="preserve">5 Tier Wire Shelving Unit Storage Rack, </t>
+          <t>5層黑30高</t>
         </is>
       </c>
       <c r="D32" s="77" t="inlineStr">
@@ -10286,7 +10286,7 @@
     <row r="33" ht="16" customHeight="1">
       <c r="A33" s="127" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="B33" s="83" t="inlineStr">
@@ -10296,7 +10296,7 @@
       </c>
       <c r="C33" s="82" t="inlineStr">
         <is>
-          <t xml:space="preserve">5 Tier Wire Shelving Unit Storage Rack, </t>
+          <t>5層黑30高</t>
         </is>
       </c>
       <c r="D33" s="84" t="inlineStr">
@@ -10331,7 +10331,7 @@
     <row r="34" ht="16" customHeight="1">
       <c r="A34" s="112" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="B34" s="48" t="inlineStr">
@@ -10341,7 +10341,7 @@
       </c>
       <c r="C34" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Displays By Jack 5 Tier Heavy Duty Wire </t>
+          <t>5層鉻30高</t>
         </is>
       </c>
       <c r="D34" s="49" t="inlineStr">
@@ -10380,7 +10380,7 @@
     <row r="35" ht="16" customHeight="1">
       <c r="A35" s="115" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="B35" s="55" t="inlineStr">
@@ -10390,7 +10390,7 @@
       </c>
       <c r="C35" s="54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Displays By Jack 5 Tier Heavy Duty Wire </t>
+          <t>5層鉻30高</t>
         </is>
       </c>
       <c r="D35" s="56" t="inlineStr">
@@ -10429,7 +10429,7 @@
     <row r="36" ht="16" customHeight="1">
       <c r="A36" s="118" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="B36" s="62" t="inlineStr">
@@ -10439,7 +10439,7 @@
       </c>
       <c r="C36" s="61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Displays By Jack 5 Tier Heavy Duty Wire </t>
+          <t>5層鉻30高</t>
         </is>
       </c>
       <c r="D36" s="63" t="inlineStr">
@@ -10478,7 +10478,7 @@
     <row r="37" ht="16" customHeight="1">
       <c r="A37" s="121" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="B37" s="69" t="inlineStr">
@@ -10488,7 +10488,7 @@
       </c>
       <c r="C37" s="68" t="inlineStr">
         <is>
-          <t xml:space="preserve">Displays By Jack 5 Tier Heavy Duty Wire </t>
+          <t>5層鉻30高</t>
         </is>
       </c>
       <c r="D37" s="70" t="inlineStr">
@@ -10523,7 +10523,7 @@
     <row r="38" ht="16" customHeight="1">
       <c r="A38" s="124" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="B38" s="76" t="inlineStr">
@@ -10533,7 +10533,7 @@
       </c>
       <c r="C38" s="75" t="inlineStr">
         <is>
-          <t xml:space="preserve">Displays By Jack 5 Tier Heavy Duty Wire </t>
+          <t>5層鉻30高</t>
         </is>
       </c>
       <c r="D38" s="77" t="inlineStr">
@@ -10572,7 +10572,7 @@
     <row r="39" ht="16" customHeight="1">
       <c r="A39" s="127" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="B39" s="83" t="inlineStr">
@@ -10582,7 +10582,7 @@
       </c>
       <c r="C39" s="82" t="inlineStr">
         <is>
-          <t xml:space="preserve">Displays By Jack 5 Tier Heavy Duty Wire </t>
+          <t>5層鉻30高</t>
         </is>
       </c>
       <c r="D39" s="84" t="inlineStr">
@@ -10621,7 +10621,7 @@
     <row r="40" ht="16" customHeight="1">
       <c r="A40" s="112" t="inlineStr">
         <is>
-          <t>Storage Cart 10D</t>
+          <t>十層收納車</t>
         </is>
       </c>
       <c r="B40" s="48" t="inlineStr">
@@ -10631,7 +10631,7 @@
       </c>
       <c r="C40" s="47" t="inlineStr">
         <is>
-          <t>Display By Jack 10-Drawer Rainbow Storag</t>
+          <t>彩虹抽屜車</t>
         </is>
       </c>
       <c r="D40" s="49" t="inlineStr">
@@ -10670,7 +10670,7 @@
     <row r="41" ht="16" customHeight="1">
       <c r="A41" s="115" t="inlineStr">
         <is>
-          <t>Storage Cart 10D</t>
+          <t>十層收納車</t>
         </is>
       </c>
       <c r="B41" s="55" t="inlineStr">
@@ -10680,7 +10680,7 @@
       </c>
       <c r="C41" s="54" t="inlineStr">
         <is>
-          <t>Display By Jack 10-Drawer Rainbow Storag</t>
+          <t>彩虹抽屜車</t>
         </is>
       </c>
       <c r="D41" s="56" t="inlineStr">
@@ -10719,7 +10719,7 @@
     <row r="42" ht="16" customHeight="1">
       <c r="A42" s="118" t="inlineStr">
         <is>
-          <t>Storage Cart 10D</t>
+          <t>十層收納車</t>
         </is>
       </c>
       <c r="B42" s="62" t="inlineStr">
@@ -10729,7 +10729,7 @@
       </c>
       <c r="C42" s="61" t="inlineStr">
         <is>
-          <t>Display By Jack 10-Drawer Rainbow Storag</t>
+          <t>彩虹抽屜車</t>
         </is>
       </c>
       <c r="D42" s="63" t="inlineStr">
@@ -10768,7 +10768,7 @@
     <row r="43" ht="16" customHeight="1">
       <c r="A43" s="121" t="inlineStr">
         <is>
-          <t>Storage Cart 10D</t>
+          <t>十層收納車</t>
         </is>
       </c>
       <c r="B43" s="69" t="inlineStr">
@@ -10778,7 +10778,7 @@
       </c>
       <c r="C43" s="68" t="inlineStr">
         <is>
-          <t>Display By Jack 10-Drawer Rainbow Storag</t>
+          <t>彩虹抽屜車</t>
         </is>
       </c>
       <c r="D43" s="70" t="inlineStr">
@@ -10817,7 +10817,7 @@
     <row r="44" ht="16" customHeight="1">
       <c r="A44" s="124" t="inlineStr">
         <is>
-          <t>Storage Cart 10D</t>
+          <t>十層收納車</t>
         </is>
       </c>
       <c r="B44" s="76" t="inlineStr">
@@ -10827,7 +10827,7 @@
       </c>
       <c r="C44" s="75" t="inlineStr">
         <is>
-          <t>Display By Jack 10-Drawer Rainbow Storag</t>
+          <t>彩虹抽屜車</t>
         </is>
       </c>
       <c r="D44" s="77" t="inlineStr">
@@ -10866,7 +10866,7 @@
     <row r="45" ht="16" customHeight="1">
       <c r="A45" s="127" t="inlineStr">
         <is>
-          <t>Storage Cart 10D</t>
+          <t>十層收納車</t>
         </is>
       </c>
       <c r="B45" s="83" t="inlineStr">
@@ -10876,7 +10876,7 @@
       </c>
       <c r="C45" s="82" t="inlineStr">
         <is>
-          <t>Display By Jack 10-Drawer Rainbow Storag</t>
+          <t>彩虹抽屜車</t>
         </is>
       </c>
       <c r="D45" s="84" t="inlineStr">
@@ -10915,7 +10915,7 @@
     <row r="46" ht="16" customHeight="1">
       <c r="A46" s="112" t="inlineStr">
         <is>
-          <t>Storage Cart 10D</t>
+          <t>十層收納車</t>
         </is>
       </c>
       <c r="B46" s="48" t="inlineStr">
@@ -10925,7 +10925,7 @@
       </c>
       <c r="C46" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Display By Jack Rolling Storage Cart 10 </t>
+          <t>黑色抽屜車</t>
         </is>
       </c>
       <c r="D46" s="49" t="inlineStr">
@@ -10964,7 +10964,7 @@
     <row r="47" ht="16" customHeight="1">
       <c r="A47" s="115" t="inlineStr">
         <is>
-          <t>Storage Cart 10D</t>
+          <t>十層收納車</t>
         </is>
       </c>
       <c r="B47" s="55" t="inlineStr">
@@ -10974,7 +10974,7 @@
       </c>
       <c r="C47" s="54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Display By Jack Rolling Storage Cart 10 </t>
+          <t>黑色抽屜車</t>
         </is>
       </c>
       <c r="D47" s="56" t="inlineStr">
@@ -11013,7 +11013,7 @@
     <row r="48" ht="16" customHeight="1">
       <c r="A48" s="118" t="inlineStr">
         <is>
-          <t>Storage Cart 10D</t>
+          <t>十層收納車</t>
         </is>
       </c>
       <c r="B48" s="62" t="inlineStr">
@@ -11023,7 +11023,7 @@
       </c>
       <c r="C48" s="61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Display By Jack Rolling Storage Cart 10 </t>
+          <t>黑色抽屜車</t>
         </is>
       </c>
       <c r="D48" s="63" t="inlineStr">
@@ -11062,7 +11062,7 @@
     <row r="49" ht="16" customHeight="1">
       <c r="A49" s="121" t="inlineStr">
         <is>
-          <t>Storage Cart 10D</t>
+          <t>十層收納車</t>
         </is>
       </c>
       <c r="B49" s="69" t="inlineStr">
@@ -11072,7 +11072,7 @@
       </c>
       <c r="C49" s="68" t="inlineStr">
         <is>
-          <t xml:space="preserve">Display By Jack Rolling Storage Cart 10 </t>
+          <t>黑色抽屜車</t>
         </is>
       </c>
       <c r="D49" s="70" t="inlineStr">
@@ -11111,7 +11111,7 @@
     <row r="50" ht="16" customHeight="1">
       <c r="A50" s="124" t="inlineStr">
         <is>
-          <t>Storage Cart 10D</t>
+          <t>十層收納車</t>
         </is>
       </c>
       <c r="B50" s="76" t="inlineStr">
@@ -11121,7 +11121,7 @@
       </c>
       <c r="C50" s="75" t="inlineStr">
         <is>
-          <t xml:space="preserve">Display By Jack Rolling Storage Cart 10 </t>
+          <t>黑色抽屜車</t>
         </is>
       </c>
       <c r="D50" s="77" t="inlineStr">
@@ -11160,7 +11160,7 @@
     <row r="51" ht="16" customHeight="1">
       <c r="A51" s="127" t="inlineStr">
         <is>
-          <t>Storage Cart 10D</t>
+          <t>十層收納車</t>
         </is>
       </c>
       <c r="B51" s="83" t="inlineStr">
@@ -11170,7 +11170,7 @@
       </c>
       <c r="C51" s="82" t="inlineStr">
         <is>
-          <t xml:space="preserve">Display By Jack Rolling Storage Cart 10 </t>
+          <t>黑色抽屜車</t>
         </is>
       </c>
       <c r="D51" s="84" t="inlineStr">
@@ -11207,7 +11207,7 @@
     <row r="52" ht="16" customHeight="1">
       <c r="A52" s="112" t="inlineStr">
         <is>
-          <t>Storage Cart 10D</t>
+          <t>十層收納車</t>
         </is>
       </c>
       <c r="B52" s="48" t="inlineStr">
@@ -11217,7 +11217,7 @@
       </c>
       <c r="C52" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Display By Jack Rolling Storage Cart 10 </t>
+          <t>白色抽屜車</t>
         </is>
       </c>
       <c r="D52" s="49" t="inlineStr">
@@ -11256,7 +11256,7 @@
     <row r="53" ht="16" customHeight="1">
       <c r="A53" s="115" t="inlineStr">
         <is>
-          <t>Storage Cart 10D</t>
+          <t>十層收納車</t>
         </is>
       </c>
       <c r="B53" s="55" t="inlineStr">
@@ -11266,7 +11266,7 @@
       </c>
       <c r="C53" s="54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Display By Jack Rolling Storage Cart 10 </t>
+          <t>白色抽屜車</t>
         </is>
       </c>
       <c r="D53" s="56" t="inlineStr">
@@ -11305,7 +11305,7 @@
     <row r="54" ht="16" customHeight="1">
       <c r="A54" s="118" t="inlineStr">
         <is>
-          <t>Storage Cart 10D</t>
+          <t>十層收納車</t>
         </is>
       </c>
       <c r="B54" s="62" t="inlineStr">
@@ -11315,7 +11315,7 @@
       </c>
       <c r="C54" s="61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Display By Jack Rolling Storage Cart 10 </t>
+          <t>白色抽屜車</t>
         </is>
       </c>
       <c r="D54" s="63" t="inlineStr">
@@ -11354,7 +11354,7 @@
     <row r="55" ht="16" customHeight="1">
       <c r="A55" s="121" t="inlineStr">
         <is>
-          <t>Storage Cart 10D</t>
+          <t>十層收納車</t>
         </is>
       </c>
       <c r="B55" s="69" t="inlineStr">
@@ -11364,7 +11364,7 @@
       </c>
       <c r="C55" s="68" t="inlineStr">
         <is>
-          <t xml:space="preserve">Display By Jack Rolling Storage Cart 10 </t>
+          <t>白色抽屜車</t>
         </is>
       </c>
       <c r="D55" s="70" t="inlineStr">
@@ -11403,7 +11403,7 @@
     <row r="56" ht="16" customHeight="1">
       <c r="A56" s="124" t="inlineStr">
         <is>
-          <t>Storage Cart 10D</t>
+          <t>十層收納車</t>
         </is>
       </c>
       <c r="B56" s="76" t="inlineStr">
@@ -11413,7 +11413,7 @@
       </c>
       <c r="C56" s="75" t="inlineStr">
         <is>
-          <t xml:space="preserve">Display By Jack Rolling Storage Cart 10 </t>
+          <t>白色抽屜車</t>
         </is>
       </c>
       <c r="D56" s="77" t="inlineStr">
@@ -11452,7 +11452,7 @@
     <row r="57" ht="16" customHeight="1">
       <c r="A57" s="127" t="inlineStr">
         <is>
-          <t>Storage Cart 10D</t>
+          <t>十層收納車</t>
         </is>
       </c>
       <c r="B57" s="83" t="inlineStr">
@@ -11462,7 +11462,7 @@
       </c>
       <c r="C57" s="82" t="inlineStr">
         <is>
-          <t xml:space="preserve">Display By Jack Rolling Storage Cart 10 </t>
+          <t>白色抽屜車</t>
         </is>
       </c>
       <c r="D57" s="84" t="inlineStr">
@@ -11501,7 +11501,7 @@
     <row r="58" ht="16" customHeight="1">
       <c r="A58" s="112" t="inlineStr">
         <is>
-          <t>Laptop Stand A</t>
+          <t>筆電桌A款</t>
         </is>
       </c>
       <c r="B58" s="48" t="inlineStr">
@@ -11511,7 +11511,7 @@
       </c>
       <c r="C58" s="47" t="inlineStr">
         <is>
-          <t>Displays By Jack Adjustable Height Rolli</t>
+          <t>傾斜桌附層</t>
         </is>
       </c>
       <c r="D58" s="49" t="inlineStr">
@@ -11546,7 +11546,7 @@
     <row r="59" ht="16" customHeight="1">
       <c r="A59" s="115" t="inlineStr">
         <is>
-          <t>Laptop Stand A</t>
+          <t>筆電桌A款</t>
         </is>
       </c>
       <c r="B59" s="55" t="inlineStr">
@@ -11556,7 +11556,7 @@
       </c>
       <c r="C59" s="54" t="inlineStr">
         <is>
-          <t>Displays By Jack Adjustable Height Rolli</t>
+          <t>傾斜桌附層</t>
         </is>
       </c>
       <c r="D59" s="56" t="inlineStr">
@@ -11593,7 +11593,7 @@
     <row r="60" ht="16" customHeight="1">
       <c r="A60" s="118" t="inlineStr">
         <is>
-          <t>Laptop Stand A</t>
+          <t>筆電桌A款</t>
         </is>
       </c>
       <c r="B60" s="62" t="inlineStr">
@@ -11603,7 +11603,7 @@
       </c>
       <c r="C60" s="61" t="inlineStr">
         <is>
-          <t>Displays By Jack Adjustable Height Rolli</t>
+          <t>傾斜桌附層</t>
         </is>
       </c>
       <c r="D60" s="63" t="inlineStr">
@@ -11638,7 +11638,7 @@
     <row r="61" ht="16" customHeight="1">
       <c r="A61" s="121" t="inlineStr">
         <is>
-          <t>Laptop Stand A</t>
+          <t>筆電桌A款</t>
         </is>
       </c>
       <c r="B61" s="69" t="inlineStr">
@@ -11648,7 +11648,7 @@
       </c>
       <c r="C61" s="68" t="inlineStr">
         <is>
-          <t>Displays By Jack Adjustable Height Rolli</t>
+          <t>傾斜桌附層</t>
         </is>
       </c>
       <c r="D61" s="70" t="inlineStr">
@@ -11685,7 +11685,7 @@
     <row r="62" ht="16" customHeight="1">
       <c r="A62" s="124" t="inlineStr">
         <is>
-          <t>Laptop Stand A</t>
+          <t>筆電桌A款</t>
         </is>
       </c>
       <c r="B62" s="76" t="inlineStr">
@@ -11695,7 +11695,7 @@
       </c>
       <c r="C62" s="75" t="inlineStr">
         <is>
-          <t>Displays By Jack Adjustable Height Rolli</t>
+          <t>傾斜桌附層</t>
         </is>
       </c>
       <c r="D62" s="77" t="inlineStr">
@@ -11730,7 +11730,7 @@
     <row r="63" ht="16" customHeight="1">
       <c r="A63" s="127" t="inlineStr">
         <is>
-          <t>Laptop Stand A</t>
+          <t>筆電桌A款</t>
         </is>
       </c>
       <c r="B63" s="83" t="inlineStr">
@@ -11740,7 +11740,7 @@
       </c>
       <c r="C63" s="82" t="inlineStr">
         <is>
-          <t>Displays By Jack Adjustable Height Rolli</t>
+          <t>傾斜桌附層</t>
         </is>
       </c>
       <c r="D63" s="84" t="inlineStr">
@@ -11775,7 +11775,7 @@
     <row r="64" ht="16" customHeight="1">
       <c r="A64" s="112" t="inlineStr">
         <is>
-          <t>Dryer Rack</t>
+          <t>折疊曬衣架</t>
         </is>
       </c>
       <c r="B64" s="48" t="inlineStr">
@@ -11785,7 +11785,7 @@
       </c>
       <c r="C64" s="47" t="inlineStr">
         <is>
-          <t>Displays By Jack Portable Collapsible Cl</t>
+          <t>折疊鉻曬衣</t>
         </is>
       </c>
       <c r="D64" s="49" t="inlineStr">
@@ -11824,7 +11824,7 @@
     <row r="65" ht="16" customHeight="1">
       <c r="A65" s="115" t="inlineStr">
         <is>
-          <t>Dryer Rack</t>
+          <t>折疊曬衣架</t>
         </is>
       </c>
       <c r="B65" s="55" t="inlineStr">
@@ -11834,7 +11834,7 @@
       </c>
       <c r="C65" s="54" t="inlineStr">
         <is>
-          <t>Displays By Jack Portable Collapsible Cl</t>
+          <t>折疊鉻曬衣</t>
         </is>
       </c>
       <c r="D65" s="56" t="inlineStr">
@@ -11873,7 +11873,7 @@
     <row r="66" ht="16" customHeight="1">
       <c r="A66" s="118" t="inlineStr">
         <is>
-          <t>Dryer Rack</t>
+          <t>折疊曬衣架</t>
         </is>
       </c>
       <c r="B66" s="62" t="inlineStr">
@@ -11883,7 +11883,7 @@
       </c>
       <c r="C66" s="61" t="inlineStr">
         <is>
-          <t>Displays By Jack Portable Collapsible Cl</t>
+          <t>折疊鉻曬衣</t>
         </is>
       </c>
       <c r="D66" s="63" t="inlineStr">
@@ -11922,7 +11922,7 @@
     <row r="67" ht="16" customHeight="1">
       <c r="A67" s="121" t="inlineStr">
         <is>
-          <t>Dryer Rack</t>
+          <t>折疊曬衣架</t>
         </is>
       </c>
       <c r="B67" s="69" t="inlineStr">
@@ -11932,7 +11932,7 @@
       </c>
       <c r="C67" s="68" t="inlineStr">
         <is>
-          <t>Displays By Jack Portable Collapsible Cl</t>
+          <t>折疊鉻曬衣</t>
         </is>
       </c>
       <c r="D67" s="70" t="inlineStr">
@@ -11971,7 +11971,7 @@
     <row r="68" ht="16" customHeight="1">
       <c r="A68" s="124" t="inlineStr">
         <is>
-          <t>Dryer Rack</t>
+          <t>折疊曬衣架</t>
         </is>
       </c>
       <c r="B68" s="76" t="inlineStr">
@@ -11981,7 +11981,7 @@
       </c>
       <c r="C68" s="75" t="inlineStr">
         <is>
-          <t>Displays By Jack Portable Collapsible Cl</t>
+          <t>折疊鉻曬衣</t>
         </is>
       </c>
       <c r="D68" s="77" t="inlineStr">
@@ -12020,7 +12020,7 @@
     <row r="69" ht="16" customHeight="1">
       <c r="A69" s="127" t="inlineStr">
         <is>
-          <t>Dryer Rack</t>
+          <t>折疊曬衣架</t>
         </is>
       </c>
       <c r="B69" s="83" t="inlineStr">
@@ -12030,7 +12030,7 @@
       </c>
       <c r="C69" s="82" t="inlineStr">
         <is>
-          <t>Displays By Jack Portable Collapsible Cl</t>
+          <t>折疊鉻曬衣</t>
         </is>
       </c>
       <c r="D69" s="84" t="inlineStr">
@@ -12069,7 +12069,7 @@
     <row r="70" ht="16" customHeight="1">
       <c r="A70" s="112" t="inlineStr">
         <is>
-          <t>Laptop Stand B</t>
+          <t>筆電桌B款</t>
         </is>
       </c>
       <c r="B70" s="48" t="inlineStr">
@@ -12079,7 +12079,7 @@
       </c>
       <c r="C70" s="47" t="inlineStr">
         <is>
-          <t>Displays By Jack Adjustable Height Rolli</t>
+          <t>平桌16寬</t>
         </is>
       </c>
       <c r="D70" s="49" t="inlineStr">
@@ -12114,7 +12114,7 @@
     <row r="71" ht="16" customHeight="1">
       <c r="A71" s="115" t="inlineStr">
         <is>
-          <t>Laptop Stand B</t>
+          <t>筆電桌B款</t>
         </is>
       </c>
       <c r="B71" s="55" t="inlineStr">
@@ -12124,7 +12124,7 @@
       </c>
       <c r="C71" s="54" t="inlineStr">
         <is>
-          <t>Displays By Jack Adjustable Height Rolli</t>
+          <t>平桌16寬</t>
         </is>
       </c>
       <c r="D71" s="56" t="inlineStr">
@@ -12161,7 +12161,7 @@
     <row r="72" ht="16" customHeight="1">
       <c r="A72" s="118" t="inlineStr">
         <is>
-          <t>Laptop Stand B</t>
+          <t>筆電桌B款</t>
         </is>
       </c>
       <c r="B72" s="62" t="inlineStr">
@@ -12171,7 +12171,7 @@
       </c>
       <c r="C72" s="61" t="inlineStr">
         <is>
-          <t>Displays By Jack Adjustable Height Rolli</t>
+          <t>平桌16寬</t>
         </is>
       </c>
       <c r="D72" s="63" t="inlineStr">
@@ -12208,7 +12208,7 @@
     <row r="73" ht="16" customHeight="1">
       <c r="A73" s="121" t="inlineStr">
         <is>
-          <t>Laptop Stand B</t>
+          <t>筆電桌B款</t>
         </is>
       </c>
       <c r="B73" s="69" t="inlineStr">
@@ -12218,7 +12218,7 @@
       </c>
       <c r="C73" s="68" t="inlineStr">
         <is>
-          <t>Displays By Jack Adjustable Height Rolli</t>
+          <t>平桌16寬</t>
         </is>
       </c>
       <c r="D73" s="70" t="inlineStr">
@@ -12253,7 +12253,7 @@
     <row r="74" ht="16" customHeight="1">
       <c r="A74" s="124" t="inlineStr">
         <is>
-          <t>Laptop Stand B</t>
+          <t>筆電桌B款</t>
         </is>
       </c>
       <c r="B74" s="76" t="inlineStr">
@@ -12263,7 +12263,7 @@
       </c>
       <c r="C74" s="75" t="inlineStr">
         <is>
-          <t>Displays By Jack Adjustable Height Rolli</t>
+          <t>平桌16寬</t>
         </is>
       </c>
       <c r="D74" s="77" t="inlineStr">
@@ -12298,7 +12298,7 @@
     <row r="75" ht="16" customHeight="1">
       <c r="A75" s="127" t="inlineStr">
         <is>
-          <t>Laptop Stand B</t>
+          <t>筆電桌B款</t>
         </is>
       </c>
       <c r="B75" s="83" t="inlineStr">
@@ -12308,7 +12308,7 @@
       </c>
       <c r="C75" s="82" t="inlineStr">
         <is>
-          <t>Displays By Jack Adjustable Height Rolli</t>
+          <t>平桌16寬</t>
         </is>
       </c>
       <c r="D75" s="84" t="inlineStr">
@@ -12343,7 +12343,7 @@
     <row r="76" ht="16" customHeight="1">
       <c r="A76" s="112" t="inlineStr">
         <is>
-          <t>Sweater Hangers</t>
+          <t>毛衣防痕架</t>
         </is>
       </c>
       <c r="B76" s="48" t="inlineStr">
@@ -12353,7 +12353,7 @@
       </c>
       <c r="C76" s="47" t="inlineStr">
         <is>
-          <t>Displays By Jack No Shoulder Bumps Sweat</t>
+          <t>黑21寬10入</t>
         </is>
       </c>
       <c r="D76" s="49" t="inlineStr">
@@ -12392,7 +12392,7 @@
     <row r="77" ht="16" customHeight="1">
       <c r="A77" s="115" t="inlineStr">
         <is>
-          <t>Sweater Hangers</t>
+          <t>毛衣防痕架</t>
         </is>
       </c>
       <c r="B77" s="55" t="inlineStr">
@@ -12402,7 +12402,7 @@
       </c>
       <c r="C77" s="54" t="inlineStr">
         <is>
-          <t>Displays By Jack No Shoulder Bumps Sweat</t>
+          <t>黑21寬10入</t>
         </is>
       </c>
       <c r="D77" s="56" t="inlineStr">
@@ -12441,7 +12441,7 @@
     <row r="78" ht="16" customHeight="1">
       <c r="A78" s="118" t="inlineStr">
         <is>
-          <t>Sweater Hangers</t>
+          <t>毛衣防痕架</t>
         </is>
       </c>
       <c r="B78" s="62" t="inlineStr">
@@ -12451,7 +12451,7 @@
       </c>
       <c r="C78" s="61" t="inlineStr">
         <is>
-          <t>Displays By Jack No Shoulder Bumps Sweat</t>
+          <t>黑21寬10入</t>
         </is>
       </c>
       <c r="D78" s="63" t="inlineStr">
@@ -12490,7 +12490,7 @@
     <row r="79" ht="16" customHeight="1">
       <c r="A79" s="121" t="inlineStr">
         <is>
-          <t>Sweater Hangers</t>
+          <t>毛衣防痕架</t>
         </is>
       </c>
       <c r="B79" s="69" t="inlineStr">
@@ -12500,7 +12500,7 @@
       </c>
       <c r="C79" s="68" t="inlineStr">
         <is>
-          <t>Displays By Jack No Shoulder Bumps Sweat</t>
+          <t>黑21寬10入</t>
         </is>
       </c>
       <c r="D79" s="70" t="inlineStr">
@@ -12539,7 +12539,7 @@
     <row r="80" ht="16" customHeight="1">
       <c r="A80" s="124" t="inlineStr">
         <is>
-          <t>Sweater Hangers</t>
+          <t>毛衣防痕架</t>
         </is>
       </c>
       <c r="B80" s="76" t="inlineStr">
@@ -12549,7 +12549,7 @@
       </c>
       <c r="C80" s="75" t="inlineStr">
         <is>
-          <t>Displays By Jack No Shoulder Bumps Sweat</t>
+          <t>黑21寬10入</t>
         </is>
       </c>
       <c r="D80" s="77" t="inlineStr">
@@ -12588,7 +12588,7 @@
     <row r="81" ht="16" customHeight="1">
       <c r="A81" s="127" t="inlineStr">
         <is>
-          <t>Sweater Hangers</t>
+          <t>毛衣防痕架</t>
         </is>
       </c>
       <c r="B81" s="83" t="inlineStr">
@@ -12598,7 +12598,7 @@
       </c>
       <c r="C81" s="82" t="inlineStr">
         <is>
-          <t>Displays By Jack No Shoulder Bumps Sweat</t>
+          <t>黑21寬10入</t>
         </is>
       </c>
       <c r="D81" s="84" t="inlineStr">
@@ -12637,7 +12637,7 @@
     <row r="82" ht="16" customHeight="1">
       <c r="A82" s="112" t="inlineStr">
         <is>
-          <t>Bathroom Storage</t>
+          <t>馬桶置物架</t>
         </is>
       </c>
       <c r="B82" s="48" t="inlineStr">
@@ -12647,7 +12647,7 @@
       </c>
       <c r="C82" s="47" t="inlineStr">
         <is>
-          <t>Display by Jack Over-The-Toilet Bathroom</t>
+          <t>馬桶上三層</t>
         </is>
       </c>
       <c r="D82" s="49" t="inlineStr">
@@ -12682,7 +12682,7 @@
     <row r="83" ht="16" customHeight="1">
       <c r="A83" s="115" t="inlineStr">
         <is>
-          <t>Bathroom Storage</t>
+          <t>馬桶置物架</t>
         </is>
       </c>
       <c r="B83" s="55" t="inlineStr">
@@ -12692,7 +12692,7 @@
       </c>
       <c r="C83" s="54" t="inlineStr">
         <is>
-          <t>Display by Jack Over-The-Toilet Bathroom</t>
+          <t>馬桶上三層</t>
         </is>
       </c>
       <c r="D83" s="56" t="inlineStr">
@@ -12729,7 +12729,7 @@
     <row r="84" ht="16" customHeight="1">
       <c r="A84" s="118" t="inlineStr">
         <is>
-          <t>Bathroom Storage</t>
+          <t>馬桶置物架</t>
         </is>
       </c>
       <c r="B84" s="62" t="inlineStr">
@@ -12739,7 +12739,7 @@
       </c>
       <c r="C84" s="61" t="inlineStr">
         <is>
-          <t>Display by Jack Over-The-Toilet Bathroom</t>
+          <t>馬桶上三層</t>
         </is>
       </c>
       <c r="D84" s="63" t="inlineStr">
@@ -12776,7 +12776,7 @@
     <row r="85" ht="16" customHeight="1">
       <c r="A85" s="121" t="inlineStr">
         <is>
-          <t>Bathroom Storage</t>
+          <t>馬桶置物架</t>
         </is>
       </c>
       <c r="B85" s="69" t="inlineStr">
@@ -12786,7 +12786,7 @@
       </c>
       <c r="C85" s="68" t="inlineStr">
         <is>
-          <t>Display by Jack Over-The-Toilet Bathroom</t>
+          <t>馬桶上三層</t>
         </is>
       </c>
       <c r="D85" s="70" t="inlineStr">
@@ -12823,7 +12823,7 @@
     <row r="86" ht="16" customHeight="1">
       <c r="A86" s="124" t="inlineStr">
         <is>
-          <t>Bathroom Storage</t>
+          <t>馬桶置物架</t>
         </is>
       </c>
       <c r="B86" s="76" t="inlineStr">
@@ -12833,7 +12833,7 @@
       </c>
       <c r="C86" s="75" t="inlineStr">
         <is>
-          <t>Display by Jack Over-The-Toilet Bathroom</t>
+          <t>馬桶上三層</t>
         </is>
       </c>
       <c r="D86" s="77" t="inlineStr">
@@ -12868,7 +12868,7 @@
     <row r="87" ht="16" customHeight="1">
       <c r="A87" s="127" t="inlineStr">
         <is>
-          <t>Bathroom Storage</t>
+          <t>馬桶置物架</t>
         </is>
       </c>
       <c r="B87" s="83" t="inlineStr">
@@ -12878,7 +12878,7 @@
       </c>
       <c r="C87" s="82" t="inlineStr">
         <is>
-          <t>Display by Jack Over-The-Toilet Bathroom</t>
+          <t>馬桶上三層</t>
         </is>
       </c>
       <c r="D87" s="84" t="inlineStr">
@@ -12913,7 +12913,7 @@
     <row r="88" ht="16" customHeight="1">
       <c r="A88" s="112" t="inlineStr">
         <is>
-          <t>Double Rail Rack</t>
+          <t>雙桿掛衣架</t>
         </is>
       </c>
       <c r="B88" s="48" t="inlineStr">
@@ -12923,7 +12923,7 @@
       </c>
       <c r="C88" s="47" t="inlineStr">
         <is>
-          <t>Displays By Jack Double Rail Clothes Rac</t>
+          <t>雙桿輪掛衣</t>
         </is>
       </c>
       <c r="D88" s="49" t="inlineStr">
@@ -12960,7 +12960,7 @@
     <row r="89" ht="16" customHeight="1">
       <c r="A89" s="115" t="inlineStr">
         <is>
-          <t>Double Rail Rack</t>
+          <t>雙桿掛衣架</t>
         </is>
       </c>
       <c r="B89" s="55" t="inlineStr">
@@ -12970,7 +12970,7 @@
       </c>
       <c r="C89" s="54" t="inlineStr">
         <is>
-          <t>Displays By Jack Double Rail Clothes Rac</t>
+          <t>雙桿輪掛衣</t>
         </is>
       </c>
       <c r="D89" s="56" t="inlineStr">
@@ -13007,7 +13007,7 @@
     <row r="90" ht="16" customHeight="1">
       <c r="A90" s="118" t="inlineStr">
         <is>
-          <t>Double Rail Rack</t>
+          <t>雙桿掛衣架</t>
         </is>
       </c>
       <c r="B90" s="62" t="inlineStr">
@@ -13017,7 +13017,7 @@
       </c>
       <c r="C90" s="61" t="inlineStr">
         <is>
-          <t>Displays By Jack Double Rail Clothes Rac</t>
+          <t>雙桿輪掛衣</t>
         </is>
       </c>
       <c r="D90" s="63" t="inlineStr">
@@ -13052,7 +13052,7 @@
     <row r="91" ht="16" customHeight="1">
       <c r="A91" s="121" t="inlineStr">
         <is>
-          <t>Double Rail Rack</t>
+          <t>雙桿掛衣架</t>
         </is>
       </c>
       <c r="B91" s="69" t="inlineStr">
@@ -13062,7 +13062,7 @@
       </c>
       <c r="C91" s="68" t="inlineStr">
         <is>
-          <t>Displays By Jack Double Rail Clothes Rac</t>
+          <t>雙桿輪掛衣</t>
         </is>
       </c>
       <c r="D91" s="70" t="inlineStr">
@@ -13099,7 +13099,7 @@
     <row r="92" ht="16" customHeight="1">
       <c r="A92" s="124" t="inlineStr">
         <is>
-          <t>Double Rail Rack</t>
+          <t>雙桿掛衣架</t>
         </is>
       </c>
       <c r="B92" s="76" t="inlineStr">
@@ -13109,7 +13109,7 @@
       </c>
       <c r="C92" s="75" t="inlineStr">
         <is>
-          <t>Displays By Jack Double Rail Clothes Rac</t>
+          <t>雙桿輪掛衣</t>
         </is>
       </c>
       <c r="D92" s="77" t="inlineStr">
@@ -13144,7 +13144,7 @@
     <row r="93" ht="16" customHeight="1">
       <c r="A93" s="127" t="inlineStr">
         <is>
-          <t>Double Rail Rack</t>
+          <t>雙桿掛衣架</t>
         </is>
       </c>
       <c r="B93" s="83" t="inlineStr">
@@ -13154,7 +13154,7 @@
       </c>
       <c r="C93" s="82" t="inlineStr">
         <is>
-          <t>Displays By Jack Double Rail Clothes Rac</t>
+          <t>雙桿輪掛衣</t>
         </is>
       </c>
       <c r="D93" s="84" t="inlineStr">
@@ -13189,7 +13189,7 @@
     <row r="94" ht="16" customHeight="1">
       <c r="A94" s="112" t="inlineStr">
         <is>
-          <t>3-Tier Cart</t>
+          <t>三層推車網</t>
         </is>
       </c>
       <c r="B94" s="48" t="inlineStr">
@@ -13199,7 +13199,7 @@
       </c>
       <c r="C94" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Displays By Jack 3-Tier Rolling Storage </t>
+          <t>三層網籃車</t>
         </is>
       </c>
       <c r="D94" s="49" t="inlineStr">
@@ -13236,7 +13236,7 @@
     <row r="95" ht="16" customHeight="1">
       <c r="A95" s="115" t="inlineStr">
         <is>
-          <t>3-Tier Cart</t>
+          <t>三層推車網</t>
         </is>
       </c>
       <c r="B95" s="55" t="inlineStr">
@@ -13246,7 +13246,7 @@
       </c>
       <c r="C95" s="54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Displays By Jack 3-Tier Rolling Storage </t>
+          <t>三層網籃車</t>
         </is>
       </c>
       <c r="D95" s="56" t="inlineStr">
@@ -13281,7 +13281,7 @@
     <row r="96" ht="16" customHeight="1">
       <c r="A96" s="118" t="inlineStr">
         <is>
-          <t>3-Tier Cart</t>
+          <t>三層推車網</t>
         </is>
       </c>
       <c r="B96" s="62" t="inlineStr">
@@ -13291,7 +13291,7 @@
       </c>
       <c r="C96" s="61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Displays By Jack 3-Tier Rolling Storage </t>
+          <t>三層網籃車</t>
         </is>
       </c>
       <c r="D96" s="63" t="inlineStr">
@@ -13326,7 +13326,7 @@
     <row r="97" ht="16" customHeight="1">
       <c r="A97" s="121" t="inlineStr">
         <is>
-          <t>3-Tier Cart</t>
+          <t>三層推車網</t>
         </is>
       </c>
       <c r="B97" s="69" t="inlineStr">
@@ -13336,7 +13336,7 @@
       </c>
       <c r="C97" s="68" t="inlineStr">
         <is>
-          <t xml:space="preserve">Displays By Jack 3-Tier Rolling Storage </t>
+          <t>三層網籃車</t>
         </is>
       </c>
       <c r="D97" s="70" t="inlineStr">
@@ -13375,7 +13375,7 @@
     <row r="98" ht="16" customHeight="1">
       <c r="A98" s="124" t="inlineStr">
         <is>
-          <t>3-Tier Cart</t>
+          <t>三層推車網</t>
         </is>
       </c>
       <c r="B98" s="76" t="inlineStr">
@@ -13385,7 +13385,7 @@
       </c>
       <c r="C98" s="75" t="inlineStr">
         <is>
-          <t xml:space="preserve">Displays By Jack 3-Tier Rolling Storage </t>
+          <t>三層網籃車</t>
         </is>
       </c>
       <c r="D98" s="77" t="inlineStr">
@@ -13424,7 +13424,7 @@
     <row r="99" ht="16" customHeight="1">
       <c r="A99" s="127" t="inlineStr">
         <is>
-          <t>3-Tier Cart</t>
+          <t>三層推車網</t>
         </is>
       </c>
       <c r="B99" s="83" t="inlineStr">
@@ -13434,7 +13434,7 @@
       </c>
       <c r="C99" s="82" t="inlineStr">
         <is>
-          <t xml:space="preserve">Displays By Jack 3-Tier Rolling Storage </t>
+          <t>三層網籃車</t>
         </is>
       </c>
       <c r="D99" s="84" t="inlineStr">
@@ -13473,7 +13473,7 @@
     <row r="100" ht="16" customHeight="1">
       <c r="A100" s="112" t="inlineStr">
         <is>
-          <t>Padded Hangers</t>
+          <t>軟墊防滑架</t>
         </is>
       </c>
       <c r="B100" s="48" t="inlineStr">
@@ -13483,7 +13483,7 @@
       </c>
       <c r="C100" s="47" t="inlineStr">
         <is>
-          <t>Displays By Jack No Shoulder Bumps Sweat</t>
+          <t>藍18寬4入</t>
         </is>
       </c>
       <c r="D100" s="49" t="inlineStr">
@@ -13522,7 +13522,7 @@
     <row r="101" ht="16" customHeight="1">
       <c r="A101" s="115" t="inlineStr">
         <is>
-          <t>Padded Hangers</t>
+          <t>軟墊防滑架</t>
         </is>
       </c>
       <c r="B101" s="55" t="inlineStr">
@@ -13532,7 +13532,7 @@
       </c>
       <c r="C101" s="54" t="inlineStr">
         <is>
-          <t>Displays By Jack No Shoulder Bumps Sweat</t>
+          <t>藍18寬4入</t>
         </is>
       </c>
       <c r="D101" s="56" t="inlineStr">
@@ -13571,7 +13571,7 @@
     <row r="102" ht="16" customHeight="1">
       <c r="A102" s="118" t="inlineStr">
         <is>
-          <t>Padded Hangers</t>
+          <t>軟墊防滑架</t>
         </is>
       </c>
       <c r="B102" s="62" t="inlineStr">
@@ -13581,7 +13581,7 @@
       </c>
       <c r="C102" s="61" t="inlineStr">
         <is>
-          <t>Displays By Jack No Shoulder Bumps Sweat</t>
+          <t>藍18寬4入</t>
         </is>
       </c>
       <c r="D102" s="63" t="inlineStr">
@@ -13620,7 +13620,7 @@
     <row r="103" ht="16" customHeight="1">
       <c r="A103" s="121" t="inlineStr">
         <is>
-          <t>Padded Hangers</t>
+          <t>軟墊防滑架</t>
         </is>
       </c>
       <c r="B103" s="69" t="inlineStr">
@@ -13630,7 +13630,7 @@
       </c>
       <c r="C103" s="68" t="inlineStr">
         <is>
-          <t>Displays By Jack No Shoulder Bumps Sweat</t>
+          <t>藍18寬4入</t>
         </is>
       </c>
       <c r="D103" s="70" t="inlineStr">
@@ -13665,7 +13665,7 @@
     <row r="104" ht="16" customHeight="1">
       <c r="A104" s="124" t="inlineStr">
         <is>
-          <t>Padded Hangers</t>
+          <t>軟墊防滑架</t>
         </is>
       </c>
       <c r="B104" s="76" t="inlineStr">
@@ -13675,7 +13675,7 @@
       </c>
       <c r="C104" s="75" t="inlineStr">
         <is>
-          <t>Displays By Jack No Shoulder Bumps Sweat</t>
+          <t>藍18寬4入</t>
         </is>
       </c>
       <c r="D104" s="77" t="inlineStr">
@@ -13710,7 +13710,7 @@
     <row r="105" ht="16" customHeight="1">
       <c r="A105" s="127" t="inlineStr">
         <is>
-          <t>Padded Hangers</t>
+          <t>軟墊防滑架</t>
         </is>
       </c>
       <c r="B105" s="83" t="inlineStr">
@@ -13720,7 +13720,7 @@
       </c>
       <c r="C105" s="82" t="inlineStr">
         <is>
-          <t>Displays By Jack No Shoulder Bumps Sweat</t>
+          <t>藍18寬4入</t>
         </is>
       </c>
       <c r="D105" s="84" t="inlineStr">
@@ -13755,7 +13755,7 @@
     <row r="106" ht="16" customHeight="1">
       <c r="A106" s="112" t="inlineStr">
         <is>
-          <t>Padded Hangers</t>
+          <t>軟墊防滑架</t>
         </is>
       </c>
       <c r="B106" s="48" t="inlineStr">
@@ -13765,7 +13765,7 @@
       </c>
       <c r="C106" s="47" t="inlineStr">
         <is>
-          <t>Displays By Jack No Shoulder Bumps Sweat</t>
+          <t>彩18寬4入</t>
         </is>
       </c>
       <c r="D106" s="49" t="inlineStr">
@@ -13804,7 +13804,7 @@
     <row r="107" ht="16" customHeight="1">
       <c r="A107" s="115" t="inlineStr">
         <is>
-          <t>Padded Hangers</t>
+          <t>軟墊防滑架</t>
         </is>
       </c>
       <c r="B107" s="55" t="inlineStr">
@@ -13814,7 +13814,7 @@
       </c>
       <c r="C107" s="54" t="inlineStr">
         <is>
-          <t>Displays By Jack No Shoulder Bumps Sweat</t>
+          <t>彩18寬4入</t>
         </is>
       </c>
       <c r="D107" s="56" t="inlineStr">
@@ -13851,7 +13851,7 @@
     <row r="108" ht="16" customHeight="1">
       <c r="A108" s="118" t="inlineStr">
         <is>
-          <t>Padded Hangers</t>
+          <t>軟墊防滑架</t>
         </is>
       </c>
       <c r="B108" s="62" t="inlineStr">
@@ -13861,7 +13861,7 @@
       </c>
       <c r="C108" s="61" t="inlineStr">
         <is>
-          <t>Displays By Jack No Shoulder Bumps Sweat</t>
+          <t>彩18寬4入</t>
         </is>
       </c>
       <c r="D108" s="63" t="inlineStr">
@@ -13900,7 +13900,7 @@
     <row r="109" ht="16" customHeight="1">
       <c r="A109" s="121" t="inlineStr">
         <is>
-          <t>Padded Hangers</t>
+          <t>軟墊防滑架</t>
         </is>
       </c>
       <c r="B109" s="69" t="inlineStr">
@@ -13910,7 +13910,7 @@
       </c>
       <c r="C109" s="68" t="inlineStr">
         <is>
-          <t>Displays By Jack No Shoulder Bumps Sweat</t>
+          <t>彩18寬4入</t>
         </is>
       </c>
       <c r="D109" s="70" t="inlineStr">
@@ -13949,7 +13949,7 @@
     <row r="110" ht="16" customHeight="1">
       <c r="A110" s="124" t="inlineStr">
         <is>
-          <t>Padded Hangers</t>
+          <t>軟墊防滑架</t>
         </is>
       </c>
       <c r="B110" s="76" t="inlineStr">
@@ -13959,7 +13959,7 @@
       </c>
       <c r="C110" s="75" t="inlineStr">
         <is>
-          <t>Displays By Jack No Shoulder Bumps Sweat</t>
+          <t>彩18寬4入</t>
         </is>
       </c>
       <c r="D110" s="77" t="inlineStr">
@@ -13998,7 +13998,7 @@
     <row r="111" ht="16" customHeight="1">
       <c r="A111" s="127" t="inlineStr">
         <is>
-          <t>Padded Hangers</t>
+          <t>軟墊防滑架</t>
         </is>
       </c>
       <c r="B111" s="83" t="inlineStr">
@@ -14008,7 +14008,7 @@
       </c>
       <c r="C111" s="82" t="inlineStr">
         <is>
-          <t>Displays By Jack No Shoulder Bumps Sweat</t>
+          <t>彩18寬4入</t>
         </is>
       </c>
       <c r="D111" s="84" t="inlineStr">
@@ -14047,7 +14047,7 @@
     <row r="112" ht="16" customHeight="1">
       <c r="A112" s="112" t="inlineStr">
         <is>
-          <t>Padded Hangers</t>
+          <t>軟墊防滑架</t>
         </is>
       </c>
       <c r="B112" s="48" t="inlineStr">
@@ -14057,7 +14057,7 @@
       </c>
       <c r="C112" s="47" t="inlineStr">
         <is>
-          <t>Displays By Jack No Shoulder Bumps Sweat</t>
+          <t>黑21寬4入</t>
         </is>
       </c>
       <c r="D112" s="49" t="inlineStr">
@@ -14096,7 +14096,7 @@
     <row r="113" ht="16" customHeight="1">
       <c r="A113" s="115" t="inlineStr">
         <is>
-          <t>Padded Hangers</t>
+          <t>軟墊防滑架</t>
         </is>
       </c>
       <c r="B113" s="55" t="inlineStr">
@@ -14106,7 +14106,7 @@
       </c>
       <c r="C113" s="54" t="inlineStr">
         <is>
-          <t>Displays By Jack No Shoulder Bumps Sweat</t>
+          <t>黑21寬4入</t>
         </is>
       </c>
       <c r="D113" s="56" t="inlineStr">
@@ -14141,7 +14141,7 @@
     <row r="114" ht="16" customHeight="1">
       <c r="A114" s="118" t="inlineStr">
         <is>
-          <t>Padded Hangers</t>
+          <t>軟墊防滑架</t>
         </is>
       </c>
       <c r="B114" s="62" t="inlineStr">
@@ -14151,7 +14151,7 @@
       </c>
       <c r="C114" s="61" t="inlineStr">
         <is>
-          <t>Displays By Jack No Shoulder Bumps Sweat</t>
+          <t>黑21寬4入</t>
         </is>
       </c>
       <c r="D114" s="63" t="inlineStr">
@@ -14186,7 +14186,7 @@
     <row r="115" ht="16" customHeight="1">
       <c r="A115" s="121" t="inlineStr">
         <is>
-          <t>Padded Hangers</t>
+          <t>軟墊防滑架</t>
         </is>
       </c>
       <c r="B115" s="69" t="inlineStr">
@@ -14196,7 +14196,7 @@
       </c>
       <c r="C115" s="68" t="inlineStr">
         <is>
-          <t>Displays By Jack No Shoulder Bumps Sweat</t>
+          <t>黑21寬4入</t>
         </is>
       </c>
       <c r="D115" s="70" t="inlineStr">
@@ -14231,7 +14231,7 @@
     <row r="116" ht="16" customHeight="1">
       <c r="A116" s="124" t="inlineStr">
         <is>
-          <t>Padded Hangers</t>
+          <t>軟墊防滑架</t>
         </is>
       </c>
       <c r="B116" s="76" t="inlineStr">
@@ -14241,7 +14241,7 @@
       </c>
       <c r="C116" s="75" t="inlineStr">
         <is>
-          <t>Displays By Jack No Shoulder Bumps Sweat</t>
+          <t>黑21寬4入</t>
         </is>
       </c>
       <c r="D116" s="77" t="inlineStr">
@@ -14276,7 +14276,7 @@
     <row r="117" ht="16" customHeight="1">
       <c r="A117" s="127" t="inlineStr">
         <is>
-          <t>Padded Hangers</t>
+          <t>軟墊防滑架</t>
         </is>
       </c>
       <c r="B117" s="83" t="inlineStr">
@@ -14286,7 +14286,7 @@
       </c>
       <c r="C117" s="82" t="inlineStr">
         <is>
-          <t>Displays By Jack No Shoulder Bumps Sweat</t>
+          <t>黑21寬4入</t>
         </is>
       </c>
       <c r="D117" s="84" t="inlineStr">
@@ -14321,7 +14321,7 @@
     <row r="118" ht="16" customHeight="1">
       <c r="A118" s="112" t="inlineStr">
         <is>
-          <t>Padded Hangers</t>
+          <t>軟墊防滑架</t>
         </is>
       </c>
       <c r="B118" s="48" t="inlineStr">
@@ -14331,7 +14331,7 @@
       </c>
       <c r="C118" s="47" t="inlineStr">
         <is>
-          <t>Displays By Jack No Shoulder Bumps Sweat</t>
+          <t>藍18寬10入</t>
         </is>
       </c>
       <c r="D118" s="49" t="inlineStr">
@@ -14366,7 +14366,7 @@
     <row r="119" ht="16" customHeight="1">
       <c r="A119" s="115" t="inlineStr">
         <is>
-          <t>Padded Hangers</t>
+          <t>軟墊防滑架</t>
         </is>
       </c>
       <c r="B119" s="55" t="inlineStr">
@@ -14376,7 +14376,7 @@
       </c>
       <c r="C119" s="54" t="inlineStr">
         <is>
-          <t>Displays By Jack No Shoulder Bumps Sweat</t>
+          <t>藍18寬10入</t>
         </is>
       </c>
       <c r="D119" s="56" t="inlineStr">
@@ -14411,7 +14411,7 @@
     <row r="120" ht="16" customHeight="1">
       <c r="A120" s="118" t="inlineStr">
         <is>
-          <t>Padded Hangers</t>
+          <t>軟墊防滑架</t>
         </is>
       </c>
       <c r="B120" s="62" t="inlineStr">
@@ -14421,7 +14421,7 @@
       </c>
       <c r="C120" s="61" t="inlineStr">
         <is>
-          <t>Displays By Jack No Shoulder Bumps Sweat</t>
+          <t>藍18寬10入</t>
         </is>
       </c>
       <c r="D120" s="63" t="inlineStr">
@@ -14456,7 +14456,7 @@
     <row r="121" ht="16" customHeight="1">
       <c r="A121" s="121" t="inlineStr">
         <is>
-          <t>Padded Hangers</t>
+          <t>軟墊防滑架</t>
         </is>
       </c>
       <c r="B121" s="69" t="inlineStr">
@@ -14466,7 +14466,7 @@
       </c>
       <c r="C121" s="68" t="inlineStr">
         <is>
-          <t>Displays By Jack No Shoulder Bumps Sweat</t>
+          <t>藍18寬10入</t>
         </is>
       </c>
       <c r="D121" s="70" t="inlineStr">
@@ -14501,7 +14501,7 @@
     <row r="122" ht="16" customHeight="1">
       <c r="A122" s="124" t="inlineStr">
         <is>
-          <t>Padded Hangers</t>
+          <t>軟墊防滑架</t>
         </is>
       </c>
       <c r="B122" s="76" t="inlineStr">
@@ -14511,7 +14511,7 @@
       </c>
       <c r="C122" s="75" t="inlineStr">
         <is>
-          <t>Displays By Jack No Shoulder Bumps Sweat</t>
+          <t>藍18寬10入</t>
         </is>
       </c>
       <c r="D122" s="77" t="inlineStr">
@@ -14546,7 +14546,7 @@
     <row r="123" ht="16" customHeight="1">
       <c r="A123" s="127" t="inlineStr">
         <is>
-          <t>Padded Hangers</t>
+          <t>軟墊防滑架</t>
         </is>
       </c>
       <c r="B123" s="83" t="inlineStr">
@@ -14556,7 +14556,7 @@
       </c>
       <c r="C123" s="82" t="inlineStr">
         <is>
-          <t>Displays By Jack No Shoulder Bumps Sweat</t>
+          <t>藍18寬10入</t>
         </is>
       </c>
       <c r="D123" s="84" t="inlineStr">
@@ -14591,7 +14591,7 @@
     <row r="124" ht="16" customHeight="1">
       <c r="A124" s="112" t="inlineStr">
         <is>
-          <t>Laptop Stand C</t>
+          <t>筆電桌C款</t>
         </is>
       </c>
       <c r="B124" s="48" t="inlineStr">
@@ -14601,7 +14601,7 @@
       </c>
       <c r="C124" s="47" t="inlineStr">
         <is>
-          <t>Displays By Jack Adjustable Height Rolli</t>
+          <t>銀色桌15寬</t>
         </is>
       </c>
       <c r="D124" s="49" t="inlineStr">
@@ -14636,7 +14636,7 @@
     <row r="125" ht="16" customHeight="1">
       <c r="A125" s="115" t="inlineStr">
         <is>
-          <t>Laptop Stand C</t>
+          <t>筆電桌C款</t>
         </is>
       </c>
       <c r="B125" s="55" t="inlineStr">
@@ -14646,7 +14646,7 @@
       </c>
       <c r="C125" s="54" t="inlineStr">
         <is>
-          <t>Displays By Jack Adjustable Height Rolli</t>
+          <t>銀色桌15寬</t>
         </is>
       </c>
       <c r="D125" s="56" t="inlineStr">
@@ -14683,7 +14683,7 @@
     <row r="126" ht="16" customHeight="1">
       <c r="A126" s="118" t="inlineStr">
         <is>
-          <t>Laptop Stand C</t>
+          <t>筆電桌C款</t>
         </is>
       </c>
       <c r="B126" s="62" t="inlineStr">
@@ -14693,7 +14693,7 @@
       </c>
       <c r="C126" s="61" t="inlineStr">
         <is>
-          <t>Displays By Jack Adjustable Height Rolli</t>
+          <t>銀色桌15寬</t>
         </is>
       </c>
       <c r="D126" s="63" t="inlineStr">
@@ -14728,7 +14728,7 @@
     <row r="127" ht="16" customHeight="1">
       <c r="A127" s="121" t="inlineStr">
         <is>
-          <t>Laptop Stand C</t>
+          <t>筆電桌C款</t>
         </is>
       </c>
       <c r="B127" s="69" t="inlineStr">
@@ -14738,7 +14738,7 @@
       </c>
       <c r="C127" s="68" t="inlineStr">
         <is>
-          <t>Displays By Jack Adjustable Height Rolli</t>
+          <t>銀色桌15寬</t>
         </is>
       </c>
       <c r="D127" s="70" t="inlineStr">
@@ -14773,7 +14773,7 @@
     <row r="128" ht="16" customHeight="1">
       <c r="A128" s="124" t="inlineStr">
         <is>
-          <t>Laptop Stand C</t>
+          <t>筆電桌C款</t>
         </is>
       </c>
       <c r="B128" s="76" t="inlineStr">
@@ -14783,7 +14783,7 @@
       </c>
       <c r="C128" s="75" t="inlineStr">
         <is>
-          <t>Displays By Jack Adjustable Height Rolli</t>
+          <t>銀色桌15寬</t>
         </is>
       </c>
       <c r="D128" s="77" t="inlineStr">
@@ -14818,7 +14818,7 @@
     <row r="129" ht="16" customHeight="1">
       <c r="A129" s="127" t="inlineStr">
         <is>
-          <t>Laptop Stand C</t>
+          <t>筆電桌C款</t>
         </is>
       </c>
       <c r="B129" s="83" t="inlineStr">
@@ -14828,7 +14828,7 @@
       </c>
       <c r="C129" s="82" t="inlineStr">
         <is>
-          <t>Displays By Jack Adjustable Height Rolli</t>
+          <t>銀色桌15寬</t>
         </is>
       </c>
       <c r="D129" s="84" t="inlineStr">
@@ -14863,7 +14863,7 @@
     <row r="130" ht="16" customHeight="1">
       <c r="A130" s="112" t="inlineStr">
         <is>
-          <t>Shoe Rack</t>
+          <t>可伸縮鞋架</t>
         </is>
       </c>
       <c r="B130" s="48" t="inlineStr">
@@ -14873,7 +14873,7 @@
       </c>
       <c r="C130" s="47" t="inlineStr">
         <is>
-          <t>Displays By Jack 4-Tier Stackable Shoe R</t>
+          <t>四層組合鞋</t>
         </is>
       </c>
       <c r="D130" s="49" t="inlineStr">
@@ -14908,7 +14908,7 @@
     <row r="131" ht="16" customHeight="1">
       <c r="A131" s="115" t="inlineStr">
         <is>
-          <t>Shoe Rack</t>
+          <t>可伸縮鞋架</t>
         </is>
       </c>
       <c r="B131" s="55" t="inlineStr">
@@ -14918,7 +14918,7 @@
       </c>
       <c r="C131" s="54" t="inlineStr">
         <is>
-          <t>Displays By Jack 4-Tier Stackable Shoe R</t>
+          <t>四層組合鞋</t>
         </is>
       </c>
       <c r="D131" s="56" t="inlineStr">
@@ -14955,7 +14955,7 @@
     <row r="132" ht="16" customHeight="1">
       <c r="A132" s="118" t="inlineStr">
         <is>
-          <t>Shoe Rack</t>
+          <t>可伸縮鞋架</t>
         </is>
       </c>
       <c r="B132" s="62" t="inlineStr">
@@ -14965,7 +14965,7 @@
       </c>
       <c r="C132" s="61" t="inlineStr">
         <is>
-          <t>Displays By Jack 4-Tier Stackable Shoe R</t>
+          <t>四層組合鞋</t>
         </is>
       </c>
       <c r="D132" s="63" t="inlineStr">
@@ -15000,7 +15000,7 @@
     <row r="133" ht="16" customHeight="1">
       <c r="A133" s="121" t="inlineStr">
         <is>
-          <t>Shoe Rack</t>
+          <t>可伸縮鞋架</t>
         </is>
       </c>
       <c r="B133" s="69" t="inlineStr">
@@ -15010,7 +15010,7 @@
       </c>
       <c r="C133" s="68" t="inlineStr">
         <is>
-          <t>Displays By Jack 4-Tier Stackable Shoe R</t>
+          <t>四層組合鞋</t>
         </is>
       </c>
       <c r="D133" s="70" t="inlineStr">
@@ -15045,7 +15045,7 @@
     <row r="134" ht="16" customHeight="1">
       <c r="A134" s="124" t="inlineStr">
         <is>
-          <t>Shoe Rack</t>
+          <t>可伸縮鞋架</t>
         </is>
       </c>
       <c r="B134" s="76" t="inlineStr">
@@ -15055,7 +15055,7 @@
       </c>
       <c r="C134" s="75" t="inlineStr">
         <is>
-          <t>Displays By Jack 4-Tier Stackable Shoe R</t>
+          <t>四層組合鞋</t>
         </is>
       </c>
       <c r="D134" s="77" t="inlineStr">
@@ -15090,7 +15090,7 @@
     <row r="135" ht="16" customHeight="1">
       <c r="A135" s="127" t="inlineStr">
         <is>
-          <t>Shoe Rack</t>
+          <t>可伸縮鞋架</t>
         </is>
       </c>
       <c r="B135" s="83" t="inlineStr">
@@ -15100,7 +15100,7 @@
       </c>
       <c r="C135" s="82" t="inlineStr">
         <is>
-          <t>Displays By Jack 4-Tier Stackable Shoe R</t>
+          <t>四層組合鞋</t>
         </is>
       </c>
       <c r="D135" s="84" t="inlineStr">
@@ -15135,7 +15135,7 @@
     <row r="136" ht="16" customHeight="1">
       <c r="A136" s="112" t="inlineStr">
         <is>
-          <t>Shoe Rack</t>
+          <t>可伸縮鞋架</t>
         </is>
       </c>
       <c r="B136" s="48" t="inlineStr">
@@ -15145,7 +15145,7 @@
       </c>
       <c r="C136" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Displays By Jack Extendable 2-Tier Shoe </t>
+          <t>兩層組合鞋</t>
         </is>
       </c>
       <c r="D136" s="49" t="inlineStr">
@@ -15180,7 +15180,7 @@
     <row r="137" ht="16" customHeight="1">
       <c r="A137" s="115" t="inlineStr">
         <is>
-          <t>Shoe Rack</t>
+          <t>可伸縮鞋架</t>
         </is>
       </c>
       <c r="B137" s="55" t="inlineStr">
@@ -15190,7 +15190,7 @@
       </c>
       <c r="C137" s="54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Displays By Jack Extendable 2-Tier Shoe </t>
+          <t>兩層組合鞋</t>
         </is>
       </c>
       <c r="D137" s="56" t="inlineStr">
@@ -15227,7 +15227,7 @@
     <row r="138" ht="16" customHeight="1">
       <c r="A138" s="118" t="inlineStr">
         <is>
-          <t>Shoe Rack</t>
+          <t>可伸縮鞋架</t>
         </is>
       </c>
       <c r="B138" s="62" t="inlineStr">
@@ -15237,7 +15237,7 @@
       </c>
       <c r="C138" s="61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Displays By Jack Extendable 2-Tier Shoe </t>
+          <t>兩層組合鞋</t>
         </is>
       </c>
       <c r="D138" s="63" t="inlineStr">
@@ -15272,7 +15272,7 @@
     <row r="139" ht="16" customHeight="1">
       <c r="A139" s="121" t="inlineStr">
         <is>
-          <t>Shoe Rack</t>
+          <t>可伸縮鞋架</t>
         </is>
       </c>
       <c r="B139" s="69" t="inlineStr">
@@ -15282,7 +15282,7 @@
       </c>
       <c r="C139" s="68" t="inlineStr">
         <is>
-          <t xml:space="preserve">Displays By Jack Extendable 2-Tier Shoe </t>
+          <t>兩層組合鞋</t>
         </is>
       </c>
       <c r="D139" s="70" t="inlineStr">
@@ -15317,7 +15317,7 @@
     <row r="140" ht="16" customHeight="1">
       <c r="A140" s="124" t="inlineStr">
         <is>
-          <t>Shoe Rack</t>
+          <t>可伸縮鞋架</t>
         </is>
       </c>
       <c r="B140" s="76" t="inlineStr">
@@ -15327,7 +15327,7 @@
       </c>
       <c r="C140" s="75" t="inlineStr">
         <is>
-          <t xml:space="preserve">Displays By Jack Extendable 2-Tier Shoe </t>
+          <t>兩層組合鞋</t>
         </is>
       </c>
       <c r="D140" s="77" t="inlineStr">
@@ -15362,7 +15362,7 @@
     <row r="141" ht="16" customHeight="1">
       <c r="A141" s="127" t="inlineStr">
         <is>
-          <t>Shoe Rack</t>
+          <t>可伸縮鞋架</t>
         </is>
       </c>
       <c r="B141" s="83" t="inlineStr">
@@ -15372,7 +15372,7 @@
       </c>
       <c r="C141" s="82" t="inlineStr">
         <is>
-          <t xml:space="preserve">Displays By Jack Extendable 2-Tier Shoe </t>
+          <t>兩層組合鞋</t>
         </is>
       </c>
       <c r="D141" s="84" t="inlineStr">
@@ -15407,7 +15407,7 @@
     <row r="142" ht="16" customHeight="1">
       <c r="A142" s="112" t="inlineStr">
         <is>
-          <t>Broom Holder</t>
+          <t>壁掛拖把架</t>
         </is>
       </c>
       <c r="B142" s="48" t="inlineStr">
@@ -15417,7 +15417,7 @@
       </c>
       <c r="C142" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Displays By Jack wall mounted Broom and </t>
+          <t>黑色壁掛架</t>
         </is>
       </c>
       <c r="D142" s="49" t="inlineStr">
@@ -15456,7 +15456,7 @@
     <row r="143" ht="16" customHeight="1">
       <c r="A143" s="115" t="inlineStr">
         <is>
-          <t>Broom Holder</t>
+          <t>壁掛拖把架</t>
         </is>
       </c>
       <c r="B143" s="55" t="inlineStr">
@@ -15466,7 +15466,7 @@
       </c>
       <c r="C143" s="54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Displays By Jack wall mounted Broom and </t>
+          <t>黑色壁掛架</t>
         </is>
       </c>
       <c r="D143" s="56" t="inlineStr">
@@ -15505,7 +15505,7 @@
     <row r="144" ht="16" customHeight="1">
       <c r="A144" s="118" t="inlineStr">
         <is>
-          <t>Broom Holder</t>
+          <t>壁掛拖把架</t>
         </is>
       </c>
       <c r="B144" s="62" t="inlineStr">
@@ -15515,7 +15515,7 @@
       </c>
       <c r="C144" s="61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Displays By Jack wall mounted Broom and </t>
+          <t>黑色壁掛架</t>
         </is>
       </c>
       <c r="D144" s="63" t="inlineStr">
@@ -15554,7 +15554,7 @@
     <row r="145" ht="16" customHeight="1">
       <c r="A145" s="121" t="inlineStr">
         <is>
-          <t>Broom Holder</t>
+          <t>壁掛拖把架</t>
         </is>
       </c>
       <c r="B145" s="69" t="inlineStr">
@@ -15564,7 +15564,7 @@
       </c>
       <c r="C145" s="68" t="inlineStr">
         <is>
-          <t xml:space="preserve">Displays By Jack wall mounted Broom and </t>
+          <t>黑色壁掛架</t>
         </is>
       </c>
       <c r="D145" s="70" t="inlineStr">
@@ -15603,7 +15603,7 @@
     <row r="146" ht="16" customHeight="1">
       <c r="A146" s="124" t="inlineStr">
         <is>
-          <t>Broom Holder</t>
+          <t>壁掛拖把架</t>
         </is>
       </c>
       <c r="B146" s="76" t="inlineStr">
@@ -15613,7 +15613,7 @@
       </c>
       <c r="C146" s="75" t="inlineStr">
         <is>
-          <t xml:space="preserve">Displays By Jack wall mounted Broom and </t>
+          <t>黑色壁掛架</t>
         </is>
       </c>
       <c r="D146" s="77" t="inlineStr">
@@ -15652,7 +15652,7 @@
     <row r="147" ht="16" customHeight="1">
       <c r="A147" s="127" t="inlineStr">
         <is>
-          <t>Broom Holder</t>
+          <t>壁掛拖把架</t>
         </is>
       </c>
       <c r="B147" s="83" t="inlineStr">
@@ -15662,7 +15662,7 @@
       </c>
       <c r="C147" s="82" t="inlineStr">
         <is>
-          <t xml:space="preserve">Displays By Jack wall mounted Broom and </t>
+          <t>黑色壁掛架</t>
         </is>
       </c>
       <c r="D147" s="84" t="inlineStr">
@@ -15701,7 +15701,7 @@
     <row r="148" ht="16" customHeight="1">
       <c r="A148" s="112" t="inlineStr">
         <is>
-          <t>Shower Caddy</t>
+          <t>浴室收納架</t>
         </is>
       </c>
       <c r="B148" s="48" t="inlineStr">
@@ -15711,7 +15711,7 @@
       </c>
       <c r="C148" s="47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Displays By Jack Shower Caddy Organizer </t>
+          <t>免鑽浴室架</t>
         </is>
       </c>
       <c r="D148" s="49" t="inlineStr">
@@ -15746,7 +15746,7 @@
     <row r="149" ht="16" customHeight="1">
       <c r="A149" s="115" t="inlineStr">
         <is>
-          <t>Shower Caddy</t>
+          <t>浴室收納架</t>
         </is>
       </c>
       <c r="B149" s="55" t="inlineStr">
@@ -15756,7 +15756,7 @@
       </c>
       <c r="C149" s="54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Displays By Jack Shower Caddy Organizer </t>
+          <t>免鑽浴室架</t>
         </is>
       </c>
       <c r="D149" s="56" t="inlineStr">
@@ -15791,7 +15791,7 @@
     <row r="150" ht="16" customHeight="1">
       <c r="A150" s="118" t="inlineStr">
         <is>
-          <t>Shower Caddy</t>
+          <t>浴室收納架</t>
         </is>
       </c>
       <c r="B150" s="62" t="inlineStr">
@@ -15801,7 +15801,7 @@
       </c>
       <c r="C150" s="61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Displays By Jack Shower Caddy Organizer </t>
+          <t>免鑽浴室架</t>
         </is>
       </c>
       <c r="D150" s="63" t="inlineStr">
@@ -15836,7 +15836,7 @@
     <row r="151" ht="16" customHeight="1">
       <c r="A151" s="121" t="inlineStr">
         <is>
-          <t>Shower Caddy</t>
+          <t>浴室收納架</t>
         </is>
       </c>
       <c r="B151" s="69" t="inlineStr">
@@ -15846,7 +15846,7 @@
       </c>
       <c r="C151" s="68" t="inlineStr">
         <is>
-          <t xml:space="preserve">Displays By Jack Shower Caddy Organizer </t>
+          <t>免鑽浴室架</t>
         </is>
       </c>
       <c r="D151" s="70" t="inlineStr">
@@ -15881,7 +15881,7 @@
     <row r="152" ht="16" customHeight="1">
       <c r="A152" s="124" t="inlineStr">
         <is>
-          <t>Shower Caddy</t>
+          <t>浴室收納架</t>
         </is>
       </c>
       <c r="B152" s="76" t="inlineStr">
@@ -15891,7 +15891,7 @@
       </c>
       <c r="C152" s="75" t="inlineStr">
         <is>
-          <t xml:space="preserve">Displays By Jack Shower Caddy Organizer </t>
+          <t>免鑽浴室架</t>
         </is>
       </c>
       <c r="D152" s="77" t="inlineStr">
@@ -15928,7 +15928,7 @@
     <row r="153" ht="16" customHeight="1">
       <c r="A153" s="127" t="inlineStr">
         <is>
-          <t>Shower Caddy</t>
+          <t>浴室收納架</t>
         </is>
       </c>
       <c r="B153" s="83" t="inlineStr">
@@ -15938,7 +15938,7 @@
       </c>
       <c r="C153" s="82" t="inlineStr">
         <is>
-          <t xml:space="preserve">Displays By Jack Shower Caddy Organizer </t>
+          <t>免鑽浴室架</t>
         </is>
       </c>
       <c r="D153" s="84" t="inlineStr">
@@ -16142,7 +16142,7 @@
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="27" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="B5" s="144" t="inlineStr">
@@ -16358,7 +16358,7 @@
     <row r="9" ht="16" customHeight="1">
       <c r="A9" s="27" t="inlineStr">
         <is>
-          <t>Storage Cart 10D</t>
+          <t>十層收納車</t>
         </is>
       </c>
       <c r="B9" s="144" t="inlineStr">
@@ -16574,7 +16574,7 @@
     <row r="13" ht="16" customHeight="1">
       <c r="A13" s="27" t="inlineStr">
         <is>
-          <t>Laptop Stand A</t>
+          <t>筆電桌A款</t>
         </is>
       </c>
       <c r="B13" s="144" t="inlineStr">
@@ -16758,7 +16758,7 @@
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="27" t="inlineStr">
         <is>
-          <t>Dryer Rack</t>
+          <t>折疊曬衣架</t>
         </is>
       </c>
       <c r="B17" s="144" t="inlineStr">
@@ -16974,7 +16974,7 @@
     <row r="21" ht="16" customHeight="1">
       <c r="A21" s="27" t="inlineStr">
         <is>
-          <t>Laptop Stand B</t>
+          <t>筆電桌B款</t>
         </is>
       </c>
       <c r="B21" s="144" t="inlineStr">
@@ -17158,7 +17158,7 @@
     <row r="25" ht="16" customHeight="1">
       <c r="A25" s="27" t="inlineStr">
         <is>
-          <t>Sweater Hangers</t>
+          <t>毛衣防痕架</t>
         </is>
       </c>
       <c r="B25" s="144" t="inlineStr">
@@ -17374,7 +17374,7 @@
     <row r="29" ht="16" customHeight="1">
       <c r="A29" s="27" t="inlineStr">
         <is>
-          <t>Bathroom Storage</t>
+          <t>馬桶置物架</t>
         </is>
       </c>
       <c r="B29" s="144" t="inlineStr">
@@ -17562,7 +17562,7 @@
     <row r="33" ht="16" customHeight="1">
       <c r="A33" s="27" t="inlineStr">
         <is>
-          <t>Double Rail Rack</t>
+          <t>雙桿掛衣架</t>
         </is>
       </c>
       <c r="B33" s="144" t="inlineStr">
@@ -17750,7 +17750,7 @@
     <row r="37" ht="16" customHeight="1">
       <c r="A37" s="27" t="inlineStr">
         <is>
-          <t>3-Tier Cart</t>
+          <t>三層推車網</t>
         </is>
       </c>
       <c r="B37" s="144" t="inlineStr">
@@ -17946,7 +17946,7 @@
     <row r="41" ht="16" customHeight="1">
       <c r="A41" s="27" t="inlineStr">
         <is>
-          <t>Padded Hangers</t>
+          <t>軟墊防滑架</t>
         </is>
       </c>
       <c r="B41" s="144" t="inlineStr">
@@ -18162,7 +18162,7 @@
     <row r="45" ht="16" customHeight="1">
       <c r="A45" s="27" t="inlineStr">
         <is>
-          <t>Laptop Stand C</t>
+          <t>筆電桌C款</t>
         </is>
       </c>
       <c r="B45" s="144" t="inlineStr">
@@ -18342,7 +18342,7 @@
     <row r="49" ht="16" customHeight="1">
       <c r="A49" s="27" t="inlineStr">
         <is>
-          <t>Shoe Rack</t>
+          <t>可伸縮鞋架</t>
         </is>
       </c>
       <c r="B49" s="144" t="inlineStr">
@@ -18522,7 +18522,7 @@
     <row r="53" ht="16" customHeight="1">
       <c r="A53" s="27" t="inlineStr">
         <is>
-          <t>Broom Holder</t>
+          <t>壁掛拖把架</t>
         </is>
       </c>
       <c r="B53" s="144" t="inlineStr">
@@ -18738,7 +18738,7 @@
     <row r="57" ht="16" customHeight="1">
       <c r="A57" s="27" t="inlineStr">
         <is>
-          <t>Shower Caddy</t>
+          <t>浴室收納架</t>
         </is>
       </c>
       <c r="B57" s="144" t="inlineStr">
@@ -19068,7 +19068,7 @@
       </c>
       <c r="C6" s="180" t="inlineStr">
         <is>
-          <t>Dryer Rack</t>
+          <t>折疊曬衣架</t>
         </is>
       </c>
       <c r="D6" s="83" t="inlineStr">
@@ -19115,7 +19115,7 @@
       </c>
       <c r="C7" s="180" t="inlineStr">
         <is>
-          <t>Storage Cart 10D</t>
+          <t>十層收納車</t>
         </is>
       </c>
       <c r="D7" s="83" t="inlineStr">
@@ -19162,7 +19162,7 @@
       </c>
       <c r="C8" s="180" t="inlineStr">
         <is>
-          <t>Dryer Rack</t>
+          <t>折疊曬衣架</t>
         </is>
       </c>
       <c r="D8" s="83" t="inlineStr">
@@ -19209,7 +19209,7 @@
       </c>
       <c r="C9" s="180" t="inlineStr">
         <is>
-          <t>Storage Cart 10D</t>
+          <t>十層收納車</t>
         </is>
       </c>
       <c r="D9" s="83" t="inlineStr">
@@ -19256,7 +19256,7 @@
       </c>
       <c r="C10" s="180" t="inlineStr">
         <is>
-          <t>Storage Cart 10D</t>
+          <t>十層收納車</t>
         </is>
       </c>
       <c r="D10" s="83" t="inlineStr">
@@ -19303,7 +19303,7 @@
       </c>
       <c r="C11" s="180" t="inlineStr">
         <is>
-          <t>Storage Cart 10D</t>
+          <t>十層收納車</t>
         </is>
       </c>
       <c r="D11" s="83" t="inlineStr">
@@ -19501,7 +19501,7 @@
       </c>
       <c r="B7" s="188" t="inlineStr">
         <is>
-          <t>Sweater Hangers</t>
+          <t>毛衣防痕架</t>
         </is>
       </c>
       <c r="C7" s="189" t="inlineStr">
@@ -19553,7 +19553,7 @@
       </c>
       <c r="B9" s="199" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="C9" s="200" t="inlineStr">
@@ -19598,7 +19598,7 @@
       </c>
       <c r="B10" s="199" t="inlineStr">
         <is>
-          <t>Storage Cart 10D</t>
+          <t>十層收納車</t>
         </is>
       </c>
       <c r="C10" s="200" t="inlineStr">
@@ -19643,7 +19643,7 @@
       </c>
       <c r="B11" s="199" t="inlineStr">
         <is>
-          <t>Laptop Stand A</t>
+          <t>筆電桌A款</t>
         </is>
       </c>
       <c r="C11" s="200" t="inlineStr">
@@ -19686,7 +19686,7 @@
       </c>
       <c r="B12" s="199" t="inlineStr">
         <is>
-          <t>Dryer Rack</t>
+          <t>折疊曬衣架</t>
         </is>
       </c>
       <c r="C12" s="200" t="inlineStr">
@@ -19731,7 +19731,7 @@
       </c>
       <c r="B13" s="199" t="inlineStr">
         <is>
-          <t>Laptop Stand B</t>
+          <t>筆電桌B款</t>
         </is>
       </c>
       <c r="C13" s="200" t="inlineStr">
@@ -19774,7 +19774,7 @@
       </c>
       <c r="B14" s="199" t="inlineStr">
         <is>
-          <t>Bathroom Storage</t>
+          <t>馬桶置物架</t>
         </is>
       </c>
       <c r="C14" s="200" t="inlineStr">
@@ -19824,7 +19824,7 @@
       </c>
       <c r="B16" s="212" t="inlineStr">
         <is>
-          <t>Double Rail Rack</t>
+          <t>雙桿掛衣架</t>
         </is>
       </c>
       <c r="C16" s="213" t="inlineStr">
@@ -19867,7 +19867,7 @@
       </c>
       <c r="B17" s="212" t="inlineStr">
         <is>
-          <t>3-Tier Cart</t>
+          <t>三層推車網</t>
         </is>
       </c>
       <c r="C17" s="213" t="inlineStr">
@@ -19912,7 +19912,7 @@
       </c>
       <c r="B18" s="212" t="inlineStr">
         <is>
-          <t>Laptop Stand C</t>
+          <t>筆電桌C款</t>
         </is>
       </c>
       <c r="C18" s="213" t="inlineStr">
@@ -19955,7 +19955,7 @@
       </c>
       <c r="B19" s="212" t="inlineStr">
         <is>
-          <t>Shoe Rack</t>
+          <t>可伸縮鞋架</t>
         </is>
       </c>
       <c r="C19" s="213" t="inlineStr">
@@ -19998,7 +19998,7 @@
       </c>
       <c r="B20" s="212" t="inlineStr">
         <is>
-          <t>Broom Holder</t>
+          <t>壁掛拖把架</t>
         </is>
       </c>
       <c r="C20" s="213" t="inlineStr">
@@ -20043,7 +20043,7 @@
       </c>
       <c r="B21" s="212" t="inlineStr">
         <is>
-          <t>Shower Caddy</t>
+          <t>浴室收納架</t>
         </is>
       </c>
       <c r="C21" s="213" t="inlineStr">
@@ -20093,7 +20093,7 @@
       </c>
       <c r="B23" s="224" t="inlineStr">
         <is>
-          <t>Padded Hangers</t>
+          <t>軟墊防滑架</t>
         </is>
       </c>
       <c r="C23" s="225" t="inlineStr">
@@ -20227,7 +20227,7 @@
       <c r="A5" s="233" t="inlineStr"/>
       <c r="B5" s="188" t="inlineStr">
         <is>
-          <t>Sweater Hangers</t>
+          <t>毛衣防痕架</t>
         </is>
       </c>
       <c r="C5" s="187" t="inlineStr">
@@ -20332,7 +20332,7 @@
       <c r="A11" s="237" t="inlineStr"/>
       <c r="B11" s="199" t="inlineStr">
         <is>
-          <t>Wire Shelving</t>
+          <t>鐵線置物架</t>
         </is>
       </c>
       <c r="C11" s="198" t="inlineStr">
@@ -20430,7 +20430,7 @@
       <c r="A16" s="237" t="inlineStr"/>
       <c r="B16" s="199" t="inlineStr">
         <is>
-          <t>Storage Cart 10D</t>
+          <t>十層收納車</t>
         </is>
       </c>
       <c r="C16" s="198" t="inlineStr">
@@ -20528,7 +20528,7 @@
       <c r="A21" s="237" t="inlineStr"/>
       <c r="B21" s="199" t="inlineStr">
         <is>
-          <t>Laptop Stand A</t>
+          <t>筆電桌A款</t>
         </is>
       </c>
       <c r="C21" s="198" t="inlineStr">
@@ -20624,7 +20624,7 @@
       <c r="A26" s="237" t="inlineStr"/>
       <c r="B26" s="199" t="inlineStr">
         <is>
-          <t>Dryer Rack</t>
+          <t>折疊曬衣架</t>
         </is>
       </c>
       <c r="C26" s="198" t="inlineStr">
@@ -20722,7 +20722,7 @@
       <c r="A31" s="237" t="inlineStr"/>
       <c r="B31" s="199" t="inlineStr">
         <is>
-          <t>Laptop Stand B</t>
+          <t>筆電桌B款</t>
         </is>
       </c>
       <c r="C31" s="198" t="inlineStr">
@@ -20818,7 +20818,7 @@
       <c r="A36" s="237" t="inlineStr"/>
       <c r="B36" s="199" t="inlineStr">
         <is>
-          <t>Bathroom Storage</t>
+          <t>馬桶置物架</t>
         </is>
       </c>
       <c r="C36" s="198" t="inlineStr">
@@ -20921,7 +20921,7 @@
       <c r="A42" s="240" t="inlineStr"/>
       <c r="B42" s="212" t="inlineStr">
         <is>
-          <t>Double Rail Rack</t>
+          <t>雙桿掛衣架</t>
         </is>
       </c>
       <c r="C42" s="211" t="inlineStr">
@@ -21017,7 +21017,7 @@
       <c r="A47" s="240" t="inlineStr"/>
       <c r="B47" s="212" t="inlineStr">
         <is>
-          <t>3-Tier Cart</t>
+          <t>三層推車網</t>
         </is>
       </c>
       <c r="C47" s="211" t="inlineStr">
@@ -21115,7 +21115,7 @@
       <c r="A52" s="240" t="inlineStr"/>
       <c r="B52" s="212" t="inlineStr">
         <is>
-          <t>Laptop Stand C</t>
+          <t>筆電桌C款</t>
         </is>
       </c>
       <c r="C52" s="211" t="inlineStr">
@@ -21211,7 +21211,7 @@
       <c r="A57" s="240" t="inlineStr"/>
       <c r="B57" s="212" t="inlineStr">
         <is>
-          <t>Shoe Rack</t>
+          <t>可伸縮鞋架</t>
         </is>
       </c>
       <c r="C57" s="211" t="inlineStr">
@@ -21307,7 +21307,7 @@
       <c r="A62" s="240" t="inlineStr"/>
       <c r="B62" s="212" t="inlineStr">
         <is>
-          <t>Broom Holder</t>
+          <t>壁掛拖把架</t>
         </is>
       </c>
       <c r="C62" s="211" t="inlineStr">
@@ -21405,7 +21405,7 @@
       <c r="A67" s="240" t="inlineStr"/>
       <c r="B67" s="212" t="inlineStr">
         <is>
-          <t>Shower Caddy</t>
+          <t>浴室收納架</t>
         </is>
       </c>
       <c r="C67" s="211" t="inlineStr">
@@ -21508,7 +21508,7 @@
       <c r="A73" s="243" t="inlineStr"/>
       <c r="B73" s="224" t="inlineStr">
         <is>
-          <t>Padded Hangers</t>
+          <t>軟墊防滑架</t>
         </is>
       </c>
       <c r="C73" s="223" t="inlineStr">

</xml_diff>